<commit_message>
Added sprites and sounds, some fixes
</commit_message>
<xml_diff>
--- a/docs/spreadsheets/chaos_redux_events_catalog.xlsx
+++ b/docs/spreadsheets/chaos_redux_events_catalog.xlsx
@@ -1,96 +1,33 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\home\klim\projects\chaos_redux\docs\spreadsheets\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5163BE9E-6627-400F-8232-D874770B147A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Events" sheetId="1" r:id="rId1"/>
+    <sheet name="Events" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Events!$A$1:$I$2</definedName>
-  </definedNames>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
-  <si>
-    <t>ID</t>
-  </si>
-  <si>
-    <t>Type</t>
-  </si>
-  <si>
-    <t>Event Name</t>
-  </si>
-  <si>
-    <t>Details</t>
-  </si>
-  <si>
-    <t>Evolutions I</t>
-  </si>
-  <si>
-    <t>Evolutions II</t>
-  </si>
-  <si>
-    <t>Evolutions III</t>
-  </si>
-  <si>
-    <t>Evolutions IV</t>
-  </si>
-  <si>
-    <t>World end</t>
-  </si>
-  <si>
-    <t>Major Event</t>
-  </si>
-  <si>
-    <t>Zombie Outbreak</t>
-  </si>
-  <si>
-    <t>If the outbreak survives into the late chaos game, the Anti-Zombie League still exists, and the main horde grows large enough, the chain can end in a zombie apocalypse world-end. If the main horde is broken repeatedly instead, outbreaks slow down, the system shuts off after three collapses, and wiping out the last zombie territory triggers a final victory event that also lowers chaos.</t>
-  </si>
-  <si>
-    <t>The first major zombie adaptation makes the horde much harder to starve out and much stronger at night. It is the point where early containment starts slipping, and cure work begins getting harder.</t>
-  </si>
-  <si>
-    <t>The horde turns into a faster assault force with better attack pressure and even less reliance on supply. Finding the cure becomes harder again.</t>
-  </si>
-  <si>
-    <t>At this stage weak fronts can collapse fast, and the cure is at its hardest to finish.</t>
-  </si>
-  <si>
-    <t>The outbreak begins in one random populous state. Zombies use only manpower for their divisions, and thus depend a lot on the population of states they capture. If the horde gets momentum, it spreads fast and captured land is cored right away.
-Secondary outbreaks happen most likely in big, crowded, less developed. Chaos makes those outbreaks more common over time, and each zombie evolution makes the horde harder to contain.
-If you want to keep the event under control, the main things that matter are holding the front, cutting outbreak risk with prevention decisions, pushing cure research, and joining the Anti-Zombie League.</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -179,17 +116,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="7">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -199,16 +136,15 @@
   <dxfs count="15">
     <dxf>
       <font>
-        <b/>
-        <i val="0"/>
+        <b val="1"/>
       </font>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
+      <border outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -222,127 +158,127 @@
       </border>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
+      <border outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
+      <border outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
+      <border outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
+      <border outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
+      <border outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
+      <border outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
+      <border outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
+      <border outline="0">
         <left/>
         <right style="thin">
           <color indexed="64"/>
@@ -356,7 +292,7 @@
       </border>
     </dxf>
     <dxf>
-      <border diagonalUp="0" diagonalDown="0">
+      <border>
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -388,7 +324,7 @@
       </border>
     </dxf>
     <dxf>
-      <border diagonalUp="0" diagonalDown="0">
+      <border>
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -405,39 +341,27 @@
     </dxf>
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16">
-    <tableStyle name="Table Style 1" pivot="0" count="3" xr9:uid="{AEF72196-99EB-4E06-A5D6-D000DE4B8566}">
+    <tableStyle name="Table Style 1" pivot="0" count="3">
       <tableStyleElement type="firstColumnStripe" dxfId="0"/>
     </tableStyle>
   </tableStyles>
-  <colors>
-    <mruColors>
-      <color rgb="FF974833"/>
-    </mruColors>
-  </colors>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors/>
 </styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{EBAC382B-E17D-41F3-A1DB-866849839D0B}" name="Table1" displayName="Table1" ref="A1:I2" totalsRowShown="0" headerRowDxfId="11" dataDxfId="1" headerRowBorderDxfId="13" tableBorderDxfId="14" totalsRowBorderDxfId="12">
-  <autoFilter ref="A1:I2" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:I2" headerRowCount="1" totalsRowShown="0" headerRowDxfId="11" dataDxfId="1" headerRowBorderDxfId="13" tableBorderDxfId="14" totalsRowBorderDxfId="12">
+  <autoFilter ref="A1:I2"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{09E2E79E-E67D-4541-A2D5-F8050D248861}" name="ID" dataDxfId="10"/>
-    <tableColumn id="2" xr3:uid="{E2DB3495-3FA1-4BAF-ABC4-3336FF40B1A3}" name="Type" dataDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{E51D2C0B-22E7-4DD5-BA6B-2748F28F33A5}" name="Event Name" dataDxfId="8"/>
-    <tableColumn id="4" xr3:uid="{65105D20-8E3E-4C88-8E75-99C37C2DDC6A}" name="Details" dataDxfId="7"/>
-    <tableColumn id="5" xr3:uid="{327BD53E-1708-423F-94BD-01326356CBB2}" name="Evolutions I" dataDxfId="6"/>
-    <tableColumn id="6" xr3:uid="{E340BC85-586F-472E-894E-0BD6324AE181}" name="Evolutions II" dataDxfId="5"/>
-    <tableColumn id="7" xr3:uid="{E5F8859C-CAB3-4B28-9E8E-6DAF156E9A96}" name="Evolutions III" dataDxfId="4"/>
-    <tableColumn id="8" xr3:uid="{04AB8C5F-0AA6-4E37-A01D-8E7237252C51}" name="Evolutions IV" dataDxfId="3"/>
-    <tableColumn id="9" xr3:uid="{C1AEC05A-475F-4D3C-A4DF-8E27DC0E5D0E}" name="World end" dataDxfId="2"/>
+    <tableColumn id="1" name="ID" dataDxfId="10"/>
+    <tableColumn id="2" name="Type" dataDxfId="9"/>
+    <tableColumn id="3" name="Event Name" dataDxfId="8"/>
+    <tableColumn id="4" name="Details" dataDxfId="7"/>
+    <tableColumn id="5" name="Evolutions I" dataDxfId="6"/>
+    <tableColumn id="6" name="Evolutions II" dataDxfId="5"/>
+    <tableColumn id="7" name="Evolutions III" dataDxfId="4"/>
+    <tableColumn id="8" name="Evolutions IV" dataDxfId="3"/>
+    <tableColumn id="9" name="World end" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium3" showFirstColumn="1" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -727,83 +651,156 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FF188038"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:I3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7" customWidth="1"/>
-    <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="3" width="22" customWidth="1"/>
-    <col min="4" max="4" width="64" customWidth="1"/>
-    <col min="5" max="7" width="33" customWidth="1"/>
-    <col min="8" max="8" width="16.42578125" customWidth="1"/>
-    <col min="9" max="9" width="44" customWidth="1"/>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="64" customWidth="1" min="4" max="4"/>
+    <col width="33" customWidth="1" min="5" max="7"/>
+    <col width="16.42578125" customWidth="1" min="8" max="8"/>
+    <col width="44" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2" t="s">
+    <row r="1" ht="27.95" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Event Name</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Details</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Evolutions I</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Evolutions II</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Evolutions III</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Evolutions IV</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>World end</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>Major Event</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>Communism Spread</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>Communist influence now escalates through implemented support-driven stages inside the existing communism chain. As support rises, strikes become harsher, soft responses stop being enough, military repression becomes riskier, and rebel seizure plus civil-war pressure become much more dangerous.</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>International Coordination: suggested true evolution for chaos tier 2. Once world chaos reaches tier 2, active communism-spread countries above 15% support should get faster strike MTTH, weaker soft-response decisions, and renewed unrest after complete military failures.</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>Insurrectionary Bloc: suggested true evolution for chaos tier 4. Once world chaos reaches tier 4, countries above 30% support should face looser civil-war triggers, rebound rebel outbreaks after suppression, and military complete failures that can directly push the uprising path.</t>
+        </is>
+      </c>
+      <c r="G2" s="4" t="n"/>
+      <c r="H2" s="4" t="n"/>
+      <c r="I2" s="6" t="inlineStr">
+        <is>
+          <t>No world-end branch planned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" ht="210" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="5">
-        <v>2</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="H2" s="4"/>
-      <c r="I2" s="6" t="s">
-        <v>11</v>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Major Event</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Zombie Outbreak</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>The outbreak begins in one random populous state. Zombies use only manpower for their divisions, and thus depend a lot on the population of states they capture. If the horde gets momentum, it spreads fast and captured land is cored right away.
+Secondary outbreaks happen most likely in big, crowded, less developed. Chaos makes those outbreaks more common over time, and each zombie evolution makes the horde harder to contain.
+If you want to keep the event under control, the main things that matter are holding the front, cutting outbreak risk with prevention decisions, pushing cure research, and joining the Anti-Zombie League.</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>The first major zombie adaptation makes the horde much harder to starve out and much stronger at night. It is the point where early containment starts slipping, and cure work begins getting harder.</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>The horde turns into a faster assault force with better attack pressure and even less reliance on supply. Finding the cure becomes harder again.</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>At this stage weak fronts can collapse fast, and the cure is at its hardest to finish.</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="n"/>
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t>If the outbreak survives into the late chaos game, the Anti-Zombie League still exists, and the main horde grows large enough, the chain can end in a zombie apocalypse world-end. If the main horde is broken repeatedly instead, outbreaks slow down, the system shuts off after three collapses, and wiping out the last zombie territory triggers a final victory event that also lowers chaos.</t>
+        </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait"/>
   <tableParts count="1">
-    <tablePart r:id="rId2"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Completed biological and chemical warfare, reworked the zombies event.
</commit_message>
<xml_diff>
--- a/docs/spreadsheets/chaos_redux_events_catalog.xlsx
+++ b/docs/spreadsheets/chaos_redux_events_catalog.xlsx
@@ -1,33 +1,99 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\home\klim\projects\chaos_redux\docs\spreadsheets\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C506BCF-393F-4392-8F3D-339695CBC9F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Events" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Events" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Event Name</t>
+  </si>
+  <si>
+    <t>Details</t>
+  </si>
+  <si>
+    <t>Evolutions I</t>
+  </si>
+  <si>
+    <t>Evolutions II</t>
+  </si>
+  <si>
+    <t>Evolutions III</t>
+  </si>
+  <si>
+    <t>Evolutions IV</t>
+  </si>
+  <si>
+    <t>World end</t>
+  </si>
+  <si>
+    <t>Communism Spread</t>
+  </si>
+  <si>
+    <t>Zombie Outbreak</t>
+  </si>
+  <si>
+    <t>The outbreak begins in one random populous state. Zombies use only manpower for their divisions, and thus depend a lot on the population of states they capture. If the horde gets momentum, it spreads fast and captured land is cored right away.
+Secondary outbreaks happen most likely in big, crowded, less developed. Chaos makes those outbreaks more common over time, and each zombie evolution makes the horde harder to contain.
+If you want to keep the event under control, the main things that matter are holding the front, cutting outbreak risk with prevention decisions, pushing cure research, and joining the Anti-Zombie League.</t>
+  </si>
+  <si>
+    <t>The first major zombie adaptation makes the horde much harder to starve out and much stronger at night. It is the point where early containment starts slipping, and cure work begins getting harder.</t>
+  </si>
+  <si>
+    <t>The horde turns into a faster assault force with better attack pressure and even less reliance on supply. Finding the cure becomes harder again.</t>
+  </si>
+  <si>
+    <t>At this stage weak fronts can collapse fast, and the cure is at its hardest to finish.</t>
+  </si>
+  <si>
+    <t>If the outbreak survives into the late chaos game, the Anti-Zombie League still exists, and the main horde grows large enough, the chain can end in a zombie apocalypse world-end. If the main horde is broken repeatedly instead, outbreaks slow down, the system shuts off after three collapses, and wiping out the last zombie territory triggers a final victory event that also lowers chaos.</t>
+  </si>
+  <si>
+    <t>Major</t>
+  </si>
+  <si>
+    <t>Fire-once</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -116,17 +182,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="7">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -135,14 +201,6 @@
   </cellStyles>
   <dxfs count="15">
     <dxf>
-      <font>
-        <b val="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="top" wrapText="1"/>
-    </dxf>
-    <dxf>
       <alignment horizontal="general" vertical="top" wrapText="1"/>
       <border outline="0">
         <left style="thin">
@@ -286,6 +344,39 @@
         <top style="thin">
           <color indexed="64"/>
         </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <border>
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
@@ -310,58 +401,40 @@
       </border>
     </dxf>
     <dxf>
-      <border>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
+      <font>
+        <b/>
+      </font>
     </dxf>
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16">
-    <tableStyle name="Table Style 1" pivot="0" count="3">
-      <tableStyleElement type="firstColumnStripe" dxfId="0"/>
+    <tableStyle name="Table Style 1" pivot="0" count="1" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
+      <tableStyleElement type="firstColumnStripe" dxfId="14"/>
     </tableStyle>
   </tableStyles>
-  <colors/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:I2" headerRowCount="1" totalsRowShown="0" headerRowDxfId="11" dataDxfId="1" headerRowBorderDxfId="13" tableBorderDxfId="14" totalsRowBorderDxfId="12">
-  <autoFilter ref="A1:I2"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:I2" totalsRowShown="0" headerRowDxfId="13" dataDxfId="11" headerRowBorderDxfId="12" tableBorderDxfId="10" totalsRowBorderDxfId="9">
+  <autoFilter ref="A1:I2" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="9">
-    <tableColumn id="1" name="ID" dataDxfId="10"/>
-    <tableColumn id="2" name="Type" dataDxfId="9"/>
-    <tableColumn id="3" name="Event Name" dataDxfId="8"/>
-    <tableColumn id="4" name="Details" dataDxfId="7"/>
-    <tableColumn id="5" name="Evolutions I" dataDxfId="6"/>
-    <tableColumn id="6" name="Evolutions II" dataDxfId="5"/>
-    <tableColumn id="7" name="Evolutions III" dataDxfId="4"/>
-    <tableColumn id="8" name="Evolutions IV" dataDxfId="3"/>
-    <tableColumn id="9" name="World end" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="ID" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Type" dataDxfId="7"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Event Name" dataDxfId="6"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Details" dataDxfId="5"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Evolutions I" dataDxfId="4"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Evolutions II" dataDxfId="3"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Evolutions III" dataDxfId="2"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Evolutions IV" dataDxfId="1"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="World end" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium3" showFirstColumn="1" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -651,156 +724,100 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <tabColor rgb="FF188038"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="64" customWidth="1" min="4" max="4"/>
-    <col width="33" customWidth="1" min="5" max="7"/>
-    <col width="16.42578125" customWidth="1" min="8" max="8"/>
-    <col width="44" customWidth="1" min="9" max="9"/>
+    <col min="1" max="1" width="7" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="4" max="4" width="64" customWidth="1"/>
+    <col min="5" max="7" width="33" customWidth="1"/>
+    <col min="8" max="8" width="16.42578125" customWidth="1"/>
+    <col min="9" max="9" width="44" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="27.95" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>Event Name</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>Details</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>Evolutions I</t>
-        </is>
-      </c>
-      <c r="F1" s="2" t="inlineStr">
-        <is>
-          <t>Evolutions II</t>
-        </is>
-      </c>
-      <c r="G1" s="2" t="inlineStr">
-        <is>
-          <t>Evolutions III</t>
-        </is>
-      </c>
-      <c r="H1" s="2" t="inlineStr">
-        <is>
-          <t>Evolutions IV</t>
-        </is>
-      </c>
-      <c r="I1" s="3" t="inlineStr">
-        <is>
-          <t>World end</t>
-        </is>
+    <row r="1" spans="1:9" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>8</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="5" t="n">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" s="5">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>Major Event</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>Communism Spread</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>Communist influence now escalates through implemented support-driven stages inside the existing communism chain. As support rises, strikes become harsher, soft responses stop being enough, military repression becomes riskier, and rebel seizure plus civil-war pressure become much more dangerous.</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>International Coordination: suggested true evolution for chaos tier 2. Once world chaos reaches tier 2, active communism-spread countries above 15% support should get faster strike MTTH, weaker soft-response decisions, and renewed unrest after complete military failures.</t>
-        </is>
-      </c>
-      <c r="F2" s="4" t="inlineStr">
-        <is>
-          <t>Insurrectionary Bloc: suggested true evolution for chaos tier 4. Once world chaos reaches tier 4, countries above 30% support should face looser civil-war triggers, rebound rebel outbreaks after suppression, and military complete failures that can directly push the uprising path.</t>
-        </is>
-      </c>
-      <c r="G2" s="4" t="n"/>
-      <c r="H2" s="4" t="n"/>
-      <c r="I2" s="6" t="inlineStr">
-        <is>
-          <t>No world-end branch planned.</t>
-        </is>
-      </c>
+      <c r="B2" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="6"/>
     </row>
-    <row r="3">
-      <c r="A3" s="5" t="n">
+    <row r="3" spans="1:9" ht="195" x14ac:dyDescent="0.25">
+      <c r="A3" s="5">
         <v>2</v>
       </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>Major Event</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>Zombie Outbreak</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>The outbreak begins in one random populous state. Zombies use only manpower for their divisions, and thus depend a lot on the population of states they capture. If the horde gets momentum, it spreads fast and captured land is cored right away.
-Secondary outbreaks happen most likely in big, crowded, less developed. Chaos makes those outbreaks more common over time, and each zombie evolution makes the horde harder to contain.
-If you want to keep the event under control, the main things that matter are holding the front, cutting outbreak risk with prevention decisions, pushing cure research, and joining the Anti-Zombie League.</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>The first major zombie adaptation makes the horde much harder to starve out and much stronger at night. It is the point where early containment starts slipping, and cure work begins getting harder.</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>The horde turns into a faster assault force with better attack pressure and even less reliance on supply. Finding the cure becomes harder again.</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>At this stage weak fronts can collapse fast, and the cure is at its hardest to finish.</t>
-        </is>
-      </c>
-      <c r="H3" s="4" t="n"/>
-      <c r="I3" s="6" t="inlineStr">
-        <is>
-          <t>If the outbreak survives into the late chaos game, the Anti-Zombie League still exists, and the main horde grows large enough, the chain can end in a zombie apocalypse world-end. If the main horde is broken repeatedly instead, outbreaks slow down, the system shuts off after three collapses, and wiping out the last zombie territory triggers a final victory event that also lowers chaos.</t>
-        </is>
+      <c r="B3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="H3" s="4"/>
+      <c r="I3" s="6" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+    <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Event rework: id 1
</commit_message>
<xml_diff>
--- a/docs/spreadsheets/chaos_redux_events_catalog.xlsx
+++ b/docs/spreadsheets/chaos_redux_events_catalog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\home\klim\projects\chaos_redux\docs\spreadsheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C506BCF-393F-4392-8F3D-339695CBC9F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1A064293-9F89-4881-815E-93682BDC20B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,11 +16,12 @@
     <sheet name="Events" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
+  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
   <si>
     <t>ID</t>
   </si>
@@ -49,7 +50,7 @@
     <t>World end</t>
   </si>
   <si>
-    <t>Communism Spread</t>
+    <t>Communist Insurgency</t>
   </si>
   <si>
     <t>Zombie Outbreak</t>
@@ -76,12 +77,51 @@
   </si>
   <si>
     <t>Fire-once</t>
+  </si>
+  <si>
+    <t>Communist organizers build national pressure while contesting control of individual states. The root event immediately seeds one Level 1 controlled state so the player sees the map layer and response decisions right away. The national spirit gives a small daily communist drift, and each communist-controlled state adds +0.01 daily communist support through dynamic pressure. States progress through Agitation Zone, Insurgent Stronghold, and Communist Lockdown levels; Level 3 creates a demilitarized revolutionary lockdown zone. Local military intervention works only on Levels 1-2; Disrupt Communist Organizing reduces national communist support; emergency national intervention affects all controlled states and can trigger a custom rebel country without vanilla stockpile splitting. A country-level defeat popup fires once controlled states are gone, rebels are not active, and communist support falls below the spread threshold. World Revolution stays locked until Whispers of the World Revolution is reached.</t>
+  </si>
+  <si>
+    <t>Unstable Revolutionary Activity: begins once any state is communist-controlled. Enables rare surprise revolts, including very rare one-state breakaway revolts with rebel armies scaled by state and country strength.</t>
+  </si>
+  <si>
+    <t>Dark Worker Rituals: begins once a Level 2 stronghold exists. Enables rare worker ritual incidents that disrupt a controlled state, raise intervention risk, improve later conversion chance, and slightly increase communist support.</t>
+  </si>
+  <si>
+    <t>Whispers of the World Revolution: begins once a Level 3 lockdown exists. Unlocks World Revolution for the major-event pool. Later whisper events add 200 World Revolution weight and mark states as more likely to join uprisings.</t>
+  </si>
+  <si>
+    <t>World Revolution later uses existing communist-controlled states as REV bases. Level 1, 2, and 3 states scale rebel strength differently, with extra units from industry, population, victory points, country strength, manpower, divisions, war status, and ideology pressure. Rebel unit templates include stronger armor, motorized, and cavalry formations, and names vary by major country plus shared regional and language pools where supported.</t>
+  </si>
+  <si>
+    <t>Evolution I Tier</t>
+  </si>
+  <si>
+    <t>Evolution II Tier</t>
+  </si>
+  <si>
+    <t>Evolution III Tier</t>
+  </si>
+  <si>
+    <t>Communist organizers build national pressure while contesting control of individual states. The root event immediately seeds one Level 1 controlled state so the player sees the map layer and response decisions right away. The national spirit gives a small daily communist drift, and each communist-controlled state adds +0.01 daily communist support through dynamic pressure. States progress through Agitation Zone, Insurgent Stronghold, and Communist Lockdown levels; Level 3 creates a demilitarized revolutionary lockdown zone. Local military intervention works only on Levels 1-2; Disrupt Communist Organizing reduces national communist support; emergency national intervention affects all controlled states and can trigger a custom rebel country without vanilla stockpile splitting. A country-level defeat popup can only fire after a 180-day country grace period, once controlled states are gone, rebels are not active, and communist support falls below the spread threshold. World Revolution stays locked until Whispers of the World Revolution is reached.</t>
+  </si>
+  <si>
+    <t>Gathering Storm</t>
+  </si>
+  <si>
+    <t>Rising Chaos</t>
+  </si>
+  <si>
+    <t>Chaos Tier</t>
+  </si>
+  <si>
+    <t>World Revolution later uses existing communist-controlled states as REV bases. Level 1, 2, and 3 states scale rebel strength differently, with extra units from industry, population, state priority, country strength, manpower, divisions, war status, and ideology pressure. Rebel unit templates include stronger armor, motorized, and cavalry formations, and names vary by major country plus shared regional and language pools where supported.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" xmlns:ns4="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:ns5="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac x16r2 xr xr9">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -91,12 +131,48 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFB7E1CD"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF4CCCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFCE4D6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF4CCCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9D2E9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="7">
@@ -181,7 +257,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -195,6 +271,24 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -407,34 +501,37 @@
     </dxf>
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16">
-    <tableStyle name="Table Style 1" pivot="0" count="1" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
+    <tableStyle name="Table Style 1" pivot="0" count="1" ns3:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
       <tableStyleElement type="firstColumnStripe" dxfId="14"/>
     </tableStyle>
   </tableStyles>
   <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <ns4:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    <ext uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <ns5:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:I2" totalsRowShown="0" headerRowDxfId="13" dataDxfId="11" headerRowBorderDxfId="12" tableBorderDxfId="10" totalsRowBorderDxfId="9">
-  <autoFilter ref="A1:I2" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="ID" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Type" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Event Name" dataDxfId="6"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Details" dataDxfId="5"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Evolutions I" dataDxfId="4"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Evolutions II" dataDxfId="3"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Evolutions III" dataDxfId="2"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Evolutions IV" dataDxfId="1"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="World end" dataDxfId="0"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:L3" totalsRowShown="0" headerRowDxfId="13" dataDxfId="11" headerRowBorderDxfId="12" tableBorderDxfId="10" totalsRowBorderDxfId="9">
+  <autoFilter ref="A1:L3" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <tableColumns count="12">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000000000001}" name="ID"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000000000002}" name="Type"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000000000003}" name="Event Name"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000000000004}" name="Details"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000000000005}" name="Evolutions I"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000000000006}" name="Evolution I Tier"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000000000007}" name="Evolutions II"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000000000008}" name="Evolution II Tier"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000000000009}" name="Evolutions III"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-000000000010}" name="Evolution III Tier"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-000000000011}" name="Evolutions IV"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-000000000012}" name="World end"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium3" showFirstColumn="1" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -724,52 +821,66 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <tabColor rgb="FF188038"/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="3" width="22" customWidth="1"/>
-    <col min="4" max="4" width="64" customWidth="1"/>
-    <col min="5" max="7" width="33" customWidth="1"/>
-    <col min="8" max="8" width="16.42578125" customWidth="1"/>
-    <col min="9" max="9" width="44" customWidth="1"/>
+    <col min="3" max="3" width="24" customWidth="1"/>
+    <col min="4" max="4" width="72" customWidth="1"/>
+    <col min="5" max="5" width="34" customWidth="1"/>
+    <col min="6" max="6" width="18" customWidth="1"/>
+    <col min="7" max="7" width="34" customWidth="1"/>
+    <col min="8" max="8" width="18" customWidth="1"/>
+    <col min="9" max="9" width="34" customWidth="1"/>
+    <col min="10" max="10" width="18" customWidth="1"/>
+    <col min="11" max="11" width="16" customWidth="1"/>
+    <col min="12" max="12" width="48" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:12" ht="29" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="G1" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="J1" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="K1" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="L1" s="7" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" ht="135" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5">
         <v>1</v>
       </c>
@@ -779,14 +890,33 @@
       <c r="C2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="6"/>
+      <c r="D2" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="E2" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F2" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="G2" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="H2" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="I2" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="J2" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="K2" s="4"/>
+      <c r="L2" s="12" t="s">
+        <v>30</v>
+      </c>
     </row>
-    <row r="3" spans="1:9" ht="195" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" ht="210" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5">
         <v>2</v>
       </c>
@@ -799,17 +929,26 @@
       <c r="D3" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="G3" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="H3" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="I3" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="H3" s="4"/>
-      <c r="I3" s="6" t="s">
+      <c r="J3" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="K3" s="4"/>
+      <c r="L3" s="12" t="s">
         <v>15</v>
       </c>
     </row>

</xml_diff>

<commit_message>
event clusters and scenarios
</commit_message>
<xml_diff>
--- a/docs/spreadsheets/chaos_redux_events_catalog.xlsx
+++ b/docs/spreadsheets/chaos_redux_events_catalog.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\klimp\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\home\klim\projects\chaos_redux\docs\spreadsheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{208223F6-78FE-4C7B-A1AD-9A8F9EDB59C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{258FF301-4A1A-49CF-B218-A80F6D29A05D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="872" uniqueCount="596">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="891" uniqueCount="611">
   <si>
     <t>ID</t>
   </si>
@@ -163,9 +163,6 @@
     <t>Final Silence is a world-end scenario only if the Holy Realm exists, is sovereign, has reached the final path, has armed the final doctrine through Ministry of Release authorization, has completed the warning chain, the year is 1945 or later, Chaos Meter is above 1000, the Holy Realm has the most factories in the world, strike capability exists, world-end settings allow it, and no other world-end is active. A 1947 thermonuclear variant applies if thermonuclear logic is available.</t>
   </si>
   <si>
-    <t>In progress</t>
-  </si>
-  <si>
     <t>Research (science)</t>
   </si>
   <si>
@@ -175,9 +172,6 @@
     <t>Random War</t>
   </si>
   <si>
-    <t>Random country declares war on another random country.</t>
-  </si>
-  <si>
     <t>Minor Repeatable</t>
   </si>
   <si>
@@ -193,9 +187,6 @@
     <t>Soviet Union Collapse</t>
   </si>
   <si>
-    <t xml:space="preserve">Soviet Union releases BLR and UKR, and some other countries. Those countries will get free divisions. Soviet Union gets decisions to reclaim the broken away states. The broken away states can form a coalition. </t>
-  </si>
-  <si>
     <t>Further collapse if the crisis is not managed.</t>
   </si>
   <si>
@@ -1811,6 +1802,60 @@
   </si>
   <si>
     <t>Happens on a friday,  everything is heavely discounted for one day. A rare event</t>
+  </si>
+  <si>
+    <t>Gathering Storm: Triangular Incident. Three declarations fire in one linked dispute.</t>
+  </si>
+  <si>
+    <t>Rising Chaos: Four Fronts. Four declarations fire in one conflict web, with a small chance for a compatible special country to appear.</t>
+  </si>
+  <si>
+    <t>Chaos Tier: Contagious Ultimatums. Five declarations fire, major countries and faction members become more likely, and special-country involvement becomes more common.</t>
+  </si>
+  <si>
+    <t>Totalen Chaos: The War Week. Six declarations fire in a short chain, with a strong chance of one compatible special country participating.</t>
+  </si>
+  <si>
+    <t>World Collapse: Open Season. Seven to eight declarations fire while normal random events still run. Compatible special countries are strongly favored when available.</t>
+  </si>
+  <si>
+    <t>SCN-001</t>
+  </si>
+  <si>
+    <t>Zombie Apocalypse</t>
+  </si>
+  <si>
+    <t>Triggerable scenario. Manual setup launched from the Chaos Redux scenario window. Type controls outbreak profile/structure; intensity controls outbreak count, starting affected states, divisions, and early pressure.</t>
+  </si>
+  <si>
+    <t>Manual triggerable scenario</t>
+  </si>
+  <si>
+    <t>Manual Scenario</t>
+  </si>
+  <si>
+    <t>Implemented</t>
+  </si>
+  <si>
+    <t>SCN-002</t>
+  </si>
+  <si>
+    <t>Army of Mengele Clones</t>
+  </si>
+  <si>
+    <t>Triggerable scenario. Manual setup launched from the Chaos Redux scenario window. Type switches between the standard clone army and the stronger Aryan variant; intensity controls starting territory, division count, army strength, equipment, and neighboring pressure.</t>
+  </si>
+  <si>
+    <t>A random eligible country declares war on another eligible country. Higher chaos stages create larger linked war webs. Compatible special countries can appear in later stages.</t>
+  </si>
+  <si>
+    <t>Repeatable Wars cluster.</t>
+  </si>
+  <si>
+    <t>4, (later add more)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Soviet Union releases some countries inside its territory, and more countries through like crisis maybe if not contained. Those countries will get free divisions, so that the soviet union wouldn't be able to invade them easily right away. Soviet Union gets decisions to reclaim the broken away states. The broken away states can form a coalition (like a faction to fight the soviet union), their goal is to completely make every possible country inside soviet union a free democratic country. </t>
   </si>
 </sst>
 </file>
@@ -1891,22 +1936,6 @@
   </cellStyles>
   <dxfs count="8">
     <dxf>
-      <border>
-        <left style="thin">
-          <color rgb="FF9B3642"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF9B3642"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF9B3642"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF9B3642"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFF6F8F9"/>
@@ -1970,19 +1999,35 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color rgb="FF9B3642"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF9B3642"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF9B3642"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF9B3642"/>
+        </bottom>
+      </border>
+    </dxf>
   </dxfs>
   <tableStyles count="2">
     <tableStyle name="Main Sheet-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="4"/>
-      <tableStyleElement type="headerRow" dxfId="7"/>
-      <tableStyleElement type="firstRowStripe" dxfId="6"/>
-      <tableStyleElement type="secondRowStripe" dxfId="5"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="7"/>
+      <tableStyleElement type="headerRow" dxfId="6"/>
+      <tableStyleElement type="firstRowStripe" dxfId="5"/>
+      <tableStyleElement type="secondRowStripe" dxfId="4"/>
     </tableStyle>
     <tableStyle name="Main Sheet-style 2" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF01000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="0"/>
-      <tableStyleElement type="headerRow" dxfId="3"/>
-      <tableStyleElement type="firstRowStripe" dxfId="2"/>
-      <tableStyleElement type="secondRowStripe" dxfId="1"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="3"/>
+      <tableStyleElement type="headerRow" dxfId="2"/>
+      <tableStyleElement type="firstRowStripe" dxfId="1"/>
+      <tableStyleElement type="secondRowStripe" dxfId="0"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -2427,10 +2472,10 @@
         <v>22</v>
       </c>
       <c r="L4" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N4" s="7" t="s">
         <v>46</v>
-      </c>
-      <c r="N4" s="7" t="s">
-        <v>47</v>
       </c>
       <c r="O4" s="8"/>
       <c r="P4" s="8"/>
@@ -2443,54 +2488,68 @@
     </row>
     <row r="5" spans="1:18" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B5" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="B5" s="5" t="s">
-        <v>49</v>
-      </c>
       <c r="C5" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="D5" s="6"/>
-      <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
-      <c r="G5" s="6"/>
-      <c r="H5" s="6"/>
+        <v>607</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>593</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>594</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>595</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>596</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>597</v>
+      </c>
       <c r="I5" s="6"/>
       <c r="J5" s="6"/>
       <c r="K5" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="L5" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="N5" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="L5" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="N5" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="O5" s="8"/>
-      <c r="P5" s="8"/>
+      <c r="O5" s="8" t="s">
+        <v>608</v>
+      </c>
+      <c r="P5" s="8" t="s">
+        <v>609</v>
+      </c>
       <c r="Q5" s="8">
         <v>2</v>
       </c>
       <c r="R5" s="8" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6" spans="1:18" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>56</v>
+        <v>610</v>
       </c>
       <c r="D6" s="6"/>
       <c r="E6" s="6"/>
       <c r="F6" s="6"/>
       <c r="G6" s="6" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="H6" s="6"/>
       <c r="I6" s="6"/>
@@ -2499,10 +2558,10 @@
         <v>22</v>
       </c>
       <c r="L6" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="N6" s="7" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="O6" s="8"/>
       <c r="P6" s="8"/>
@@ -2515,13 +2574,13 @@
     </row>
     <row r="7" spans="1:18" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="D7" s="6"/>
       <c r="E7" s="6"/>
@@ -2531,13 +2590,13 @@
       <c r="I7" s="6"/>
       <c r="J7" s="6"/>
       <c r="K7" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L7" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="N7" s="7" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="O7" s="8"/>
       <c r="P7" s="8"/>
@@ -2550,13 +2609,13 @@
     </row>
     <row r="8" spans="1:18" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="D8" s="6"/>
       <c r="E8" s="6"/>
@@ -2566,16 +2625,16 @@
       <c r="I8" s="6"/>
       <c r="J8" s="6"/>
       <c r="K8" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L8" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="N8" s="7" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="O8" s="8" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="P8" s="8"/>
       <c r="Q8" s="8">
@@ -2587,13 +2646,13 @@
     </row>
     <row r="9" spans="1:18" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="D9" s="6"/>
       <c r="E9" s="6"/>
@@ -2603,13 +2662,13 @@
       <c r="I9" s="6"/>
       <c r="J9" s="6"/>
       <c r="K9" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L9" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="N9" s="7" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="O9" s="8"/>
       <c r="P9" s="8"/>
@@ -2622,13 +2681,13 @@
     </row>
     <row r="10" spans="1:18" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="D10" s="6"/>
       <c r="E10" s="6"/>
@@ -2638,13 +2697,13 @@
       <c r="I10" s="6"/>
       <c r="J10" s="6"/>
       <c r="K10" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L10" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="N10" s="7" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="O10" s="8"/>
       <c r="P10" s="8"/>
@@ -2657,13 +2716,13 @@
     </row>
     <row r="11" spans="1:18" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D11" s="6"/>
       <c r="E11" s="6"/>
@@ -2676,13 +2735,13 @@
         <v>22</v>
       </c>
       <c r="L11" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="N11" s="7" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="O11" s="8" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="P11" s="8"/>
       <c r="Q11" s="8">
@@ -2694,13 +2753,13 @@
     </row>
     <row r="12" spans="1:18" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D12" s="6"/>
       <c r="E12" s="6"/>
@@ -2713,13 +2772,13 @@
         <v>22</v>
       </c>
       <c r="L12" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="N12" s="7" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="O12" s="8" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="P12" s="8"/>
       <c r="Q12" s="8">
@@ -2731,13 +2790,13 @@
     </row>
     <row r="13" spans="1:18" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="4" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="D13" s="6"/>
       <c r="E13" s="6"/>
@@ -2750,10 +2809,10 @@
         <v>22</v>
       </c>
       <c r="L13" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="N13" s="7" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="O13" s="8"/>
       <c r="P13" s="8"/>
@@ -2766,31 +2825,31 @@
     </row>
     <row r="14" spans="1:18" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="4" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D14" s="6"/>
       <c r="E14" s="6"/>
       <c r="F14" s="6"/>
       <c r="G14" s="6" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="H14" s="6"/>
       <c r="I14" s="6"/>
       <c r="J14" s="6"/>
       <c r="K14" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L14" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="N14" s="7" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="O14" s="8"/>
       <c r="P14" s="8"/>
@@ -2803,13 +2862,13 @@
     </row>
     <row r="15" spans="1:18" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="4" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D15" s="6"/>
       <c r="E15" s="6"/>
@@ -2819,16 +2878,16 @@
       <c r="I15" s="6"/>
       <c r="J15" s="6"/>
       <c r="K15" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L15" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="N15" s="7" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="O15" s="8" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="P15" s="8"/>
       <c r="Q15" s="8">
@@ -2840,13 +2899,13 @@
     </row>
     <row r="16" spans="1:18" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="4" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="D16" s="6"/>
       <c r="E16" s="6"/>
@@ -2856,21 +2915,21 @@
       <c r="I16" s="6"/>
       <c r="J16" s="6"/>
       <c r="K16" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L16" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="17" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D17" s="6"/>
       <c r="E17" s="6"/>
@@ -2883,18 +2942,18 @@
         <v>22</v>
       </c>
       <c r="L17" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="18" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="4" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="D18" s="6"/>
       <c r="E18" s="6"/>
@@ -2904,21 +2963,21 @@
       <c r="I18" s="6"/>
       <c r="J18" s="6"/>
       <c r="K18" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L18" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="19" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="4" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="D19" s="6"/>
       <c r="E19" s="6"/>
@@ -2928,21 +2987,21 @@
       <c r="I19" s="6"/>
       <c r="J19" s="6"/>
       <c r="K19" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L19" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="20" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="4" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="D20" s="6"/>
       <c r="E20" s="6"/>
@@ -2952,27 +3011,27 @@
       <c r="I20" s="6"/>
       <c r="J20" s="6"/>
       <c r="K20" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L20" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="21" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="4" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="D21" s="6"/>
       <c r="E21" s="6"/>
       <c r="F21" s="6"/>
       <c r="G21" s="6" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="H21" s="6"/>
       <c r="I21" s="6"/>
@@ -2981,18 +3040,18 @@
         <v>22</v>
       </c>
       <c r="L21" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="22" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="4" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="D22" s="6"/>
       <c r="E22" s="6"/>
@@ -3002,24 +3061,24 @@
       <c r="I22" s="6"/>
       <c r="J22" s="6"/>
       <c r="K22" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L22" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="Q22" s="9" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="23" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="4" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="D23" s="6"/>
       <c r="E23" s="6"/>
@@ -3032,18 +3091,18 @@
         <v>22</v>
       </c>
       <c r="L23" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="24" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="4" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="D24" s="6"/>
       <c r="E24" s="6"/>
@@ -3056,18 +3115,18 @@
         <v>22</v>
       </c>
       <c r="L24" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="25" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="4" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="D25" s="6"/>
       <c r="E25" s="6"/>
@@ -3080,18 +3139,18 @@
         <v>22</v>
       </c>
       <c r="L25" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="26" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="4" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="D26" s="6"/>
       <c r="E26" s="6"/>
@@ -3104,18 +3163,18 @@
         <v>34</v>
       </c>
       <c r="L26" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="27" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="4" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="D27" s="6"/>
       <c r="E27" s="6"/>
@@ -3128,18 +3187,18 @@
         <v>22</v>
       </c>
       <c r="L27" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="28" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="4" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="D28" s="6"/>
       <c r="E28" s="6"/>
@@ -3152,18 +3211,18 @@
         <v>22</v>
       </c>
       <c r="L28" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="29" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="4" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="D29" s="6"/>
       <c r="E29" s="6"/>
@@ -3173,21 +3232,21 @@
       <c r="I29" s="6"/>
       <c r="J29" s="6"/>
       <c r="K29" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L29" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="30" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="4" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="D30" s="6"/>
       <c r="E30" s="6"/>
@@ -3197,27 +3256,27 @@
       <c r="I30" s="6"/>
       <c r="J30" s="6"/>
       <c r="K30" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L30" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="31" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="4" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="D31" s="6"/>
       <c r="E31" s="6"/>
       <c r="F31" s="6"/>
       <c r="G31" s="6" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="H31" s="6"/>
       <c r="I31" s="6"/>
@@ -3226,18 +3285,18 @@
         <v>34</v>
       </c>
       <c r="L31" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="32" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="4" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="D32" s="6"/>
       <c r="E32" s="6"/>
@@ -3247,21 +3306,21 @@
       <c r="I32" s="6"/>
       <c r="J32" s="6"/>
       <c r="K32" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L32" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="33" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="4" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="D33" s="6"/>
       <c r="E33" s="6"/>
@@ -3271,21 +3330,21 @@
       <c r="I33" s="6"/>
       <c r="J33" s="6"/>
       <c r="K33" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L33" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="34" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="4" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="D34" s="6"/>
       <c r="E34" s="6"/>
@@ -3295,21 +3354,21 @@
       <c r="I34" s="6"/>
       <c r="J34" s="6"/>
       <c r="K34" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L34" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="35" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="4" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="D35" s="6"/>
       <c r="E35" s="6"/>
@@ -3319,21 +3378,21 @@
       <c r="I35" s="6"/>
       <c r="J35" s="6"/>
       <c r="K35" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L35" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="36" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="4" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="D36" s="6"/>
       <c r="E36" s="6"/>
@@ -3343,21 +3402,21 @@
       <c r="I36" s="6"/>
       <c r="J36" s="6"/>
       <c r="K36" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L36" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="37" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="4" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="D37" s="6"/>
       <c r="E37" s="6"/>
@@ -3367,21 +3426,21 @@
       <c r="I37" s="6"/>
       <c r="J37" s="6"/>
       <c r="K37" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L37" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="38" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="4" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="D38" s="6"/>
       <c r="E38" s="6"/>
@@ -3391,27 +3450,27 @@
       <c r="I38" s="6"/>
       <c r="J38" s="6"/>
       <c r="K38" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L38" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="39" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="4" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="D39" s="6"/>
       <c r="E39" s="6"/>
       <c r="F39" s="6"/>
       <c r="G39" s="6" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="H39" s="6"/>
       <c r="I39" s="6"/>
@@ -3420,18 +3479,18 @@
         <v>22</v>
       </c>
       <c r="L39" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="40" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="4" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="D40" s="6"/>
       <c r="E40" s="6"/>
@@ -3441,21 +3500,21 @@
       <c r="I40" s="6"/>
       <c r="J40" s="6"/>
       <c r="K40" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L40" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="41" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="4" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="D41" s="6"/>
       <c r="E41" s="6"/>
@@ -3465,21 +3524,21 @@
       <c r="I41" s="6"/>
       <c r="J41" s="6"/>
       <c r="K41" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L41" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="42" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="4" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="D42" s="6"/>
       <c r="E42" s="6"/>
@@ -3489,21 +3548,21 @@
       <c r="I42" s="6"/>
       <c r="J42" s="6"/>
       <c r="K42" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L42" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="43" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="4" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="D43" s="6"/>
       <c r="E43" s="6"/>
@@ -3513,21 +3572,21 @@
       <c r="I43" s="6"/>
       <c r="J43" s="6"/>
       <c r="K43" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L43" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="44" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="4" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="D44" s="6"/>
       <c r="E44" s="6"/>
@@ -3537,21 +3596,21 @@
       <c r="I44" s="6"/>
       <c r="J44" s="6"/>
       <c r="K44" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L44" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="45" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="4" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="D45" s="6"/>
       <c r="E45" s="6"/>
@@ -3564,18 +3623,18 @@
         <v>34</v>
       </c>
       <c r="L45" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="46" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="4" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="D46" s="6"/>
       <c r="E46" s="6"/>
@@ -3588,18 +3647,18 @@
         <v>22</v>
       </c>
       <c r="L46" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="47" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="4" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="D47" s="6"/>
       <c r="E47" s="6"/>
@@ -3609,21 +3668,21 @@
       <c r="I47" s="6"/>
       <c r="J47" s="6"/>
       <c r="K47" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L47" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="48" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="4" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="D48" s="6"/>
       <c r="E48" s="6"/>
@@ -3633,21 +3692,21 @@
       <c r="I48" s="6"/>
       <c r="J48" s="6"/>
       <c r="K48" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L48" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="49" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="4" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="D49" s="6"/>
       <c r="E49" s="6"/>
@@ -3660,18 +3719,18 @@
         <v>22</v>
       </c>
       <c r="L49" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="50" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="4" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="D50" s="6"/>
       <c r="E50" s="6"/>
@@ -3684,18 +3743,18 @@
         <v>34</v>
       </c>
       <c r="L50" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="51" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="4" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="C51" s="5" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="D51" s="6"/>
       <c r="E51" s="6"/>
@@ -3705,21 +3764,21 @@
       <c r="I51" s="6"/>
       <c r="J51" s="6"/>
       <c r="K51" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L51" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="52" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="4" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="D52" s="6"/>
       <c r="E52" s="6"/>
@@ -3732,18 +3791,18 @@
         <v>22</v>
       </c>
       <c r="L52" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="53" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="4" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="B53" s="5" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="C53" s="5" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="D53" s="6"/>
       <c r="E53" s="6"/>
@@ -3753,21 +3812,21 @@
       <c r="I53" s="6"/>
       <c r="J53" s="6"/>
       <c r="K53" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L53" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="54" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="4" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="C54" s="5" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="D54" s="6"/>
       <c r="E54" s="6"/>
@@ -3780,18 +3839,18 @@
         <v>22</v>
       </c>
       <c r="L54" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="55" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="4" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="B55" s="5" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="C55" s="5" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="D55" s="6"/>
       <c r="E55" s="6"/>
@@ -3801,21 +3860,21 @@
       <c r="I55" s="6"/>
       <c r="J55" s="6"/>
       <c r="K55" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L55" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="56" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="4" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="B56" s="5" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="C56" s="5" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="D56" s="6"/>
       <c r="E56" s="6"/>
@@ -3825,21 +3884,21 @@
       <c r="I56" s="6"/>
       <c r="J56" s="6"/>
       <c r="K56" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L56" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="57" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="4" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="B57" s="5" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="C57" s="5" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="D57" s="6"/>
       <c r="E57" s="6"/>
@@ -3849,21 +3908,21 @@
       <c r="I57" s="6"/>
       <c r="J57" s="6"/>
       <c r="K57" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L57" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="58" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="4" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="B58" s="5" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="C58" s="5" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="D58" s="6"/>
       <c r="E58" s="6"/>
@@ -3873,21 +3932,21 @@
       <c r="I58" s="6"/>
       <c r="J58" s="6"/>
       <c r="K58" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L58" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="59" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="4" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="C59" s="5" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="D59" s="6"/>
       <c r="E59" s="6"/>
@@ -3897,21 +3956,21 @@
       <c r="I59" s="6"/>
       <c r="J59" s="6"/>
       <c r="K59" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L59" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="60" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="4" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="B60" s="5" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="C60" s="5" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="D60" s="6"/>
       <c r="E60" s="6"/>
@@ -3924,18 +3983,18 @@
         <v>22</v>
       </c>
       <c r="L60" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="61" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="4" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="B61" s="5" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="C61" s="5" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="D61" s="6"/>
       <c r="E61" s="6"/>
@@ -3945,21 +4004,21 @@
       <c r="I61" s="6"/>
       <c r="J61" s="6"/>
       <c r="K61" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L61" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="62" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="4" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="B62" s="5" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="C62" s="5" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="D62" s="6"/>
       <c r="E62" s="6"/>
@@ -3969,21 +4028,21 @@
       <c r="I62" s="6"/>
       <c r="J62" s="6"/>
       <c r="K62" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L62" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="63" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="4" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="B63" s="5" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="C63" s="5" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="D63" s="6"/>
       <c r="E63" s="6"/>
@@ -3993,21 +4052,21 @@
       <c r="I63" s="6"/>
       <c r="J63" s="6"/>
       <c r="K63" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L63" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="64" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="4" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="B64" s="5" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="C64" s="5" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D64" s="6"/>
       <c r="E64" s="6"/>
@@ -4017,21 +4076,21 @@
       <c r="I64" s="6"/>
       <c r="J64" s="6"/>
       <c r="K64" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L64" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="65" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="4" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="B65" s="5" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="C65" s="5" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="D65" s="6"/>
       <c r="E65" s="6"/>
@@ -4041,21 +4100,21 @@
       <c r="I65" s="6"/>
       <c r="J65" s="6"/>
       <c r="K65" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L65" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="66" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="4" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="B66" s="5" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="C66" s="5" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="D66" s="6"/>
       <c r="E66" s="6"/>
@@ -4065,21 +4124,21 @@
       <c r="I66" s="6"/>
       <c r="J66" s="6"/>
       <c r="K66" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L66" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="67" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="4" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="B67" s="5" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="C67" s="5" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="D67" s="6"/>
       <c r="E67" s="6"/>
@@ -4089,21 +4148,21 @@
       <c r="I67" s="6"/>
       <c r="J67" s="6"/>
       <c r="K67" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L67" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="68" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="4" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="B68" s="5" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="C68" s="5" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="D68" s="6"/>
       <c r="E68" s="6"/>
@@ -4116,24 +4175,24 @@
         <v>22</v>
       </c>
       <c r="L68" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="69" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="4" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B69" s="5" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="C69" s="5" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D69" s="6"/>
       <c r="E69" s="6"/>
       <c r="F69" s="6"/>
       <c r="G69" s="6" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="H69" s="6"/>
       <c r="I69" s="6"/>
@@ -4142,18 +4201,18 @@
         <v>22</v>
       </c>
       <c r="L69" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="70" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="4" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="B70" s="5" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="C70" s="5" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="D70" s="6"/>
       <c r="E70" s="6"/>
@@ -4166,18 +4225,18 @@
         <v>22</v>
       </c>
       <c r="L70" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="71" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="4" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="B71" s="5" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="C71" s="5" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="D71" s="6"/>
       <c r="E71" s="6"/>
@@ -4190,18 +4249,18 @@
         <v>34</v>
       </c>
       <c r="L71" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="72" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="4" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="B72" s="5" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="C72" s="5" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="D72" s="6"/>
       <c r="E72" s="6"/>
@@ -4214,18 +4273,18 @@
         <v>22</v>
       </c>
       <c r="L72" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="73" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="4" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="B73" s="5" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="C73" s="5" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="D73" s="6"/>
       <c r="E73" s="6"/>
@@ -4238,18 +4297,18 @@
         <v>22</v>
       </c>
       <c r="L73" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="74" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="4" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="B74" s="5" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="C74" s="5" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="D74" s="6"/>
       <c r="E74" s="6"/>
@@ -4262,18 +4321,18 @@
         <v>22</v>
       </c>
       <c r="L74" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="75" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="4" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="B75" s="5" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="C75" s="5" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="D75" s="6"/>
       <c r="E75" s="6"/>
@@ -4286,18 +4345,18 @@
         <v>22</v>
       </c>
       <c r="L75" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="76" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" s="4" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="B76" s="5" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="C76" s="5" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="D76" s="6"/>
       <c r="E76" s="6"/>
@@ -4310,18 +4369,18 @@
         <v>22</v>
       </c>
       <c r="L76" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="77" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A77" s="4" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="B77" s="5" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="C77" s="5" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="D77" s="6"/>
       <c r="E77" s="6"/>
@@ -4331,21 +4390,21 @@
       <c r="I77" s="6"/>
       <c r="J77" s="6"/>
       <c r="K77" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L77" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="78" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A78" s="4" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="B78" s="5" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="C78" s="5" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="D78" s="6"/>
       <c r="E78" s="6"/>
@@ -4355,21 +4414,21 @@
       <c r="I78" s="6"/>
       <c r="J78" s="6"/>
       <c r="K78" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L78" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="79" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79" s="4" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="B79" s="5" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="C79" s="5" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="D79" s="6"/>
       <c r="E79" s="6"/>
@@ -4379,21 +4438,21 @@
       <c r="I79" s="6"/>
       <c r="J79" s="6"/>
       <c r="K79" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L79" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="80" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A80" s="4" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="B80" s="5" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="C80" s="5" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="D80" s="6"/>
       <c r="E80" s="6"/>
@@ -4403,21 +4462,21 @@
       <c r="I80" s="6"/>
       <c r="J80" s="6"/>
       <c r="K80" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L80" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="81" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" s="4" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="B81" s="5" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="C81" s="5" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="D81" s="6"/>
       <c r="E81" s="6"/>
@@ -4430,18 +4489,18 @@
         <v>34</v>
       </c>
       <c r="L81" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="82" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A82" s="4" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="B82" s="5" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="C82" s="5" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="D82" s="6"/>
       <c r="E82" s="6"/>
@@ -4454,18 +4513,18 @@
         <v>22</v>
       </c>
       <c r="L82" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="83" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" s="4" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="B83" s="5" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="C83" s="5" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="D83" s="6"/>
       <c r="E83" s="6"/>
@@ -4475,21 +4534,21 @@
       <c r="I83" s="6"/>
       <c r="J83" s="6"/>
       <c r="K83" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L83" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="84" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A84" s="4" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="B84" s="5" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="C84" s="5" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="D84" s="6"/>
       <c r="E84" s="6"/>
@@ -4499,21 +4558,21 @@
       <c r="I84" s="6"/>
       <c r="J84" s="6"/>
       <c r="K84" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L84" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="85" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A85" s="4" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="B85" s="5" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="C85" s="5" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="D85" s="6"/>
       <c r="E85" s="6"/>
@@ -4523,21 +4582,21 @@
       <c r="I85" s="6"/>
       <c r="J85" s="6"/>
       <c r="K85" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L85" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="86" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A86" s="4" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="B86" s="5" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="C86" s="5" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="D86" s="6"/>
       <c r="E86" s="6"/>
@@ -4547,21 +4606,21 @@
       <c r="I86" s="6"/>
       <c r="J86" s="6"/>
       <c r="K86" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L86" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="87" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A87" s="4" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
       <c r="B87" s="5" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="C87" s="5" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
       <c r="D87" s="6"/>
       <c r="E87" s="6"/>
@@ -4574,18 +4633,18 @@
         <v>22</v>
       </c>
       <c r="L87" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="88" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A88" s="4" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="B88" s="5" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
       <c r="C88" s="5" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="D88" s="6"/>
       <c r="E88" s="6"/>
@@ -4595,21 +4654,21 @@
       <c r="I88" s="6"/>
       <c r="J88" s="6"/>
       <c r="K88" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L88" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="89" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A89" s="4" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
       <c r="B89" s="5" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
       <c r="C89" s="5" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="D89" s="6"/>
       <c r="E89" s="6"/>
@@ -4622,18 +4681,18 @@
         <v>22</v>
       </c>
       <c r="L89" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="90" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A90" s="4" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="B90" s="5" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
       <c r="C90" s="5" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="D90" s="6"/>
       <c r="E90" s="6"/>
@@ -4646,18 +4705,18 @@
         <v>22</v>
       </c>
       <c r="L90" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="91" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A91" s="4" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="B91" s="5" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="C91" s="5" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="D91" s="6"/>
       <c r="E91" s="6"/>
@@ -4670,24 +4729,24 @@
         <v>22</v>
       </c>
       <c r="L91" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="92" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A92" s="4" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="B92" s="5" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="C92" s="5" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="D92" s="6"/>
       <c r="E92" s="6"/>
       <c r="F92" s="6"/>
       <c r="G92" s="6" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="H92" s="6"/>
       <c r="I92" s="6"/>
@@ -4696,18 +4755,18 @@
         <v>34</v>
       </c>
       <c r="L92" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="93" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A93" s="4" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="B93" s="5" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="C93" s="5" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="D93" s="6"/>
       <c r="E93" s="6"/>
@@ -4720,18 +4779,18 @@
         <v>22</v>
       </c>
       <c r="L93" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="94" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A94" s="4" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="B94" s="5" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="C94" s="5" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="D94" s="6"/>
       <c r="E94" s="6"/>
@@ -4744,18 +4803,18 @@
         <v>22</v>
       </c>
       <c r="L94" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="95" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A95" s="4" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="B95" s="5" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
       <c r="C95" s="5" t="s">
-        <v>344</v>
+        <v>341</v>
       </c>
       <c r="D95" s="6"/>
       <c r="E95" s="6"/>
@@ -4765,21 +4824,21 @@
       <c r="I95" s="6"/>
       <c r="J95" s="6"/>
       <c r="K95" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L95" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="96" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A96" s="4" t="s">
-        <v>345</v>
+        <v>342</v>
       </c>
       <c r="B96" s="5" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="C96" s="5" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
       <c r="D96" s="6"/>
       <c r="E96" s="6"/>
@@ -4789,21 +4848,21 @@
       <c r="I96" s="6"/>
       <c r="J96" s="6"/>
       <c r="K96" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L96" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="97" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A97" s="4" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="B97" s="5" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="C97" s="5" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="D97" s="6"/>
       <c r="E97" s="6"/>
@@ -4813,21 +4872,21 @@
       <c r="I97" s="6"/>
       <c r="J97" s="6"/>
       <c r="K97" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L97" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="98" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A98" s="4" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="B98" s="5" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="C98" s="5" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="D98" s="6"/>
       <c r="E98" s="6"/>
@@ -4837,21 +4896,21 @@
       <c r="I98" s="6"/>
       <c r="J98" s="6"/>
       <c r="K98" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="L98" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="99" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A99" s="4" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
       <c r="B99" s="5" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
       <c r="C99" s="5" t="s">
-        <v>356</v>
+        <v>353</v>
       </c>
       <c r="D99" s="6"/>
       <c r="E99" s="6"/>
@@ -4864,18 +4923,18 @@
         <v>22</v>
       </c>
       <c r="L99" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="100" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A100" s="4" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
       <c r="B100" s="5" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
       <c r="C100" s="5" t="s">
-        <v>359</v>
+        <v>356</v>
       </c>
       <c r="D100" s="6"/>
       <c r="E100" s="6"/>
@@ -4888,18 +4947,18 @@
         <v>22</v>
       </c>
       <c r="L100" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="101" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A101" s="4" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
       <c r="B101" s="5" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="C101" s="5" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="D101" s="6"/>
       <c r="E101" s="6"/>
@@ -4915,13 +4974,13 @@
     </row>
     <row r="102" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A102" s="4" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="B102" s="5" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="C102" s="5" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="D102" s="6"/>
       <c r="E102" s="6"/>
@@ -4937,13 +4996,13 @@
     </row>
     <row r="103" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A103" s="4" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="B103" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="C103" s="5" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="D103" s="6"/>
       <c r="E103" s="6"/>
@@ -4959,13 +5018,13 @@
     </row>
     <row r="104" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A104" s="4" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="B104" s="5" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="C104" s="5" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="D104" s="6"/>
       <c r="E104" s="6"/>
@@ -4981,13 +5040,13 @@
     </row>
     <row r="105" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A105" s="4" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
       <c r="B105" s="5" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="C105" s="5" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="D105" s="6"/>
       <c r="E105" s="6"/>
@@ -5003,13 +5062,13 @@
     </row>
     <row r="106" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A106" s="4" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
       <c r="B106" s="5" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="C106" s="5" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
       <c r="D106" s="6"/>
       <c r="E106" s="6"/>
@@ -5025,13 +5084,13 @@
     </row>
     <row r="107" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A107" s="4" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
       <c r="B107" s="5" t="s">
-        <v>379</v>
+        <v>376</v>
       </c>
       <c r="C107" s="5" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
       <c r="D107" s="6"/>
       <c r="E107" s="6"/>
@@ -5047,13 +5106,13 @@
     </row>
     <row r="108" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A108" s="4" t="s">
-        <v>381</v>
+        <v>378</v>
       </c>
       <c r="B108" s="5" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="C108" s="5" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
       <c r="D108" s="6"/>
       <c r="E108" s="6"/>
@@ -5069,13 +5128,13 @@
     </row>
     <row r="109" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A109" s="4" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
       <c r="B109" s="5" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="C109" s="5" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
       <c r="D109" s="6"/>
       <c r="E109" s="6"/>
@@ -5091,13 +5150,13 @@
     </row>
     <row r="110" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A110" s="4" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
       <c r="B110" s="5" t="s">
-        <v>388</v>
+        <v>385</v>
       </c>
       <c r="C110" s="5" t="s">
-        <v>389</v>
+        <v>386</v>
       </c>
       <c r="D110" s="6"/>
       <c r="E110" s="6"/>
@@ -5113,13 +5172,13 @@
     </row>
     <row r="111" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A111" s="4" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
       <c r="B111" s="5" t="s">
-        <v>391</v>
+        <v>388</v>
       </c>
       <c r="C111" s="5" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
       <c r="D111" s="6"/>
       <c r="E111" s="6"/>
@@ -5135,13 +5194,13 @@
     </row>
     <row r="112" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A112" s="4" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
       <c r="B112" s="5" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
       <c r="C112" s="5" t="s">
-        <v>395</v>
+        <v>392</v>
       </c>
       <c r="D112" s="6"/>
       <c r="E112" s="6"/>
@@ -5157,13 +5216,13 @@
     </row>
     <row r="113" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A113" s="4" t="s">
-        <v>396</v>
+        <v>393</v>
       </c>
       <c r="B113" s="5" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
       <c r="C113" s="5" t="s">
-        <v>398</v>
+        <v>395</v>
       </c>
       <c r="D113" s="6"/>
       <c r="E113" s="6"/>
@@ -5179,13 +5238,13 @@
     </row>
     <row r="114" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A114" s="4" t="s">
-        <v>399</v>
+        <v>396</v>
       </c>
       <c r="B114" s="5" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="C114" s="5" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
       <c r="D114" s="6"/>
       <c r="E114" s="6"/>
@@ -5201,13 +5260,13 @@
     </row>
     <row r="115" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A115" s="4" t="s">
-        <v>402</v>
+        <v>399</v>
       </c>
       <c r="B115" s="5" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
       <c r="C115" s="5" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
       <c r="D115" s="6"/>
       <c r="E115" s="6"/>
@@ -5223,13 +5282,13 @@
     </row>
     <row r="116" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A116" s="4" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
       <c r="B116" s="5" t="s">
-        <v>406</v>
+        <v>403</v>
       </c>
       <c r="C116" s="5" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="D116" s="6"/>
       <c r="E116" s="6"/>
@@ -5245,13 +5304,13 @@
     </row>
     <row r="117" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A117" s="4" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="B117" s="5" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
       <c r="C117" s="5" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
       <c r="D117" s="6"/>
       <c r="E117" s="6"/>
@@ -5267,13 +5326,13 @@
     </row>
     <row r="118" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A118" s="4" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="B118" s="5" t="s">
-        <v>412</v>
+        <v>409</v>
       </c>
       <c r="C118" s="5" t="s">
-        <v>413</v>
+        <v>410</v>
       </c>
       <c r="D118" s="6"/>
       <c r="E118" s="6"/>
@@ -5289,13 +5348,13 @@
     </row>
     <row r="119" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A119" s="4" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
       <c r="B119" s="5" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
       <c r="C119" s="5" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
       <c r="D119" s="6"/>
       <c r="E119" s="6"/>
@@ -5311,13 +5370,13 @@
     </row>
     <row r="120" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A120" s="4" t="s">
-        <v>417</v>
+        <v>414</v>
       </c>
       <c r="B120" s="5" t="s">
-        <v>418</v>
+        <v>415</v>
       </c>
       <c r="C120" s="5" t="s">
-        <v>419</v>
+        <v>416</v>
       </c>
       <c r="D120" s="6"/>
       <c r="E120" s="6"/>
@@ -5333,13 +5392,13 @@
     </row>
     <row r="121" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A121" s="4" t="s">
-        <v>420</v>
+        <v>417</v>
       </c>
       <c r="B121" s="5" t="s">
-        <v>421</v>
+        <v>418</v>
       </c>
       <c r="C121" s="5" t="s">
-        <v>422</v>
+        <v>419</v>
       </c>
       <c r="D121" s="6"/>
       <c r="E121" s="6"/>
@@ -5355,13 +5414,13 @@
     </row>
     <row r="122" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A122" s="4" t="s">
-        <v>423</v>
+        <v>420</v>
       </c>
       <c r="B122" s="5" t="s">
-        <v>424</v>
+        <v>421</v>
       </c>
       <c r="C122" s="5" t="s">
-        <v>425</v>
+        <v>422</v>
       </c>
       <c r="D122" s="6"/>
       <c r="E122" s="6"/>
@@ -5377,13 +5436,13 @@
     </row>
     <row r="123" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A123" s="4" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
       <c r="B123" s="5" t="s">
-        <v>427</v>
+        <v>424</v>
       </c>
       <c r="C123" s="5" t="s">
-        <v>428</v>
+        <v>425</v>
       </c>
       <c r="D123" s="6"/>
       <c r="E123" s="6"/>
@@ -5399,13 +5458,13 @@
     </row>
     <row r="124" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A124" s="4" t="s">
-        <v>429</v>
+        <v>426</v>
       </c>
       <c r="B124" s="5" t="s">
-        <v>430</v>
+        <v>427</v>
       </c>
       <c r="C124" s="5" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="D124" s="6"/>
       <c r="E124" s="6"/>
@@ -5421,13 +5480,13 @@
     </row>
     <row r="125" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A125" s="4" t="s">
-        <v>432</v>
+        <v>429</v>
       </c>
       <c r="B125" s="5" t="s">
-        <v>433</v>
+        <v>430</v>
       </c>
       <c r="C125" s="5" t="s">
-        <v>434</v>
+        <v>431</v>
       </c>
       <c r="D125" s="6"/>
       <c r="E125" s="6"/>
@@ -5443,13 +5502,13 @@
     </row>
     <row r="126" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A126" s="4" t="s">
-        <v>435</v>
+        <v>432</v>
       </c>
       <c r="B126" s="5" t="s">
-        <v>436</v>
+        <v>433</v>
       </c>
       <c r="C126" s="5" t="s">
-        <v>437</v>
+        <v>434</v>
       </c>
       <c r="D126" s="6"/>
       <c r="E126" s="6"/>
@@ -5465,13 +5524,13 @@
     </row>
     <row r="127" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A127" s="4" t="s">
-        <v>438</v>
+        <v>435</v>
       </c>
       <c r="B127" s="5" t="s">
-        <v>439</v>
+        <v>436</v>
       </c>
       <c r="C127" s="5" t="s">
-        <v>440</v>
+        <v>437</v>
       </c>
       <c r="D127" s="6"/>
       <c r="E127" s="6"/>
@@ -5487,13 +5546,13 @@
     </row>
     <row r="128" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A128" s="4" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="B128" s="5" t="s">
-        <v>442</v>
+        <v>439</v>
       </c>
       <c r="C128" s="5" t="s">
-        <v>443</v>
+        <v>440</v>
       </c>
       <c r="D128" s="6"/>
       <c r="E128" s="6"/>
@@ -5509,13 +5568,13 @@
     </row>
     <row r="129" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A129" s="4" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
       <c r="B129" s="5" t="s">
-        <v>445</v>
+        <v>442</v>
       </c>
       <c r="C129" s="5" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
       <c r="D129" s="6"/>
       <c r="E129" s="6"/>
@@ -5531,13 +5590,13 @@
     </row>
     <row r="130" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A130" s="4" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
       <c r="B130" s="5" t="s">
-        <v>448</v>
+        <v>445</v>
       </c>
       <c r="C130" s="5" t="s">
-        <v>449</v>
+        <v>446</v>
       </c>
       <c r="D130" s="6"/>
       <c r="E130" s="6"/>
@@ -5553,13 +5612,13 @@
     </row>
     <row r="131" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A131" s="4" t="s">
-        <v>450</v>
+        <v>447</v>
       </c>
       <c r="B131" s="5" t="s">
-        <v>451</v>
+        <v>448</v>
       </c>
       <c r="C131" s="5" t="s">
-        <v>452</v>
+        <v>449</v>
       </c>
       <c r="D131" s="6"/>
       <c r="E131" s="6"/>
@@ -5575,13 +5634,13 @@
     </row>
     <row r="132" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A132" s="4" t="s">
-        <v>453</v>
+        <v>450</v>
       </c>
       <c r="B132" s="5" t="s">
-        <v>454</v>
+        <v>451</v>
       </c>
       <c r="C132" s="5" t="s">
-        <v>455</v>
+        <v>452</v>
       </c>
       <c r="D132" s="6"/>
       <c r="E132" s="6"/>
@@ -5597,13 +5656,13 @@
     </row>
     <row r="133" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A133" s="4" t="s">
-        <v>456</v>
+        <v>453</v>
       </c>
       <c r="B133" s="5" t="s">
-        <v>457</v>
+        <v>454</v>
       </c>
       <c r="C133" s="5" t="s">
-        <v>458</v>
+        <v>455</v>
       </c>
       <c r="D133" s="6"/>
       <c r="E133" s="6"/>
@@ -5619,13 +5678,13 @@
     </row>
     <row r="134" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A134" s="4" t="s">
-        <v>459</v>
+        <v>456</v>
       </c>
       <c r="B134" s="5" t="s">
-        <v>460</v>
+        <v>457</v>
       </c>
       <c r="C134" s="5" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="D134" s="6"/>
       <c r="E134" s="6"/>
@@ -5641,13 +5700,13 @@
     </row>
     <row r="135" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A135" s="4" t="s">
-        <v>462</v>
+        <v>459</v>
       </c>
       <c r="B135" s="5" t="s">
-        <v>463</v>
+        <v>460</v>
       </c>
       <c r="C135" s="5" t="s">
-        <v>464</v>
+        <v>461</v>
       </c>
       <c r="D135" s="6"/>
       <c r="E135" s="6"/>
@@ -5663,13 +5722,13 @@
     </row>
     <row r="136" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A136" s="4" t="s">
-        <v>465</v>
+        <v>462</v>
       </c>
       <c r="B136" s="5" t="s">
-        <v>466</v>
+        <v>463</v>
       </c>
       <c r="C136" s="5" t="s">
-        <v>467</v>
+        <v>464</v>
       </c>
       <c r="D136" s="6"/>
       <c r="E136" s="6"/>
@@ -5685,13 +5744,13 @@
     </row>
     <row r="137" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A137" s="4" t="s">
-        <v>468</v>
+        <v>465</v>
       </c>
       <c r="B137" s="5" t="s">
-        <v>469</v>
+        <v>466</v>
       </c>
       <c r="C137" s="5" t="s">
-        <v>470</v>
+        <v>467</v>
       </c>
       <c r="D137" s="6"/>
       <c r="E137" s="6"/>
@@ -5707,13 +5766,13 @@
     </row>
     <row r="138" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A138" s="4" t="s">
-        <v>471</v>
+        <v>468</v>
       </c>
       <c r="B138" s="5" t="s">
-        <v>472</v>
+        <v>469</v>
       </c>
       <c r="C138" s="5" t="s">
-        <v>473</v>
+        <v>470</v>
       </c>
       <c r="D138" s="6"/>
       <c r="E138" s="6"/>
@@ -5729,13 +5788,13 @@
     </row>
     <row r="139" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A139" s="4" t="s">
-        <v>474</v>
+        <v>471</v>
       </c>
       <c r="B139" s="5" t="s">
-        <v>475</v>
+        <v>472</v>
       </c>
       <c r="C139" s="5" t="s">
-        <v>476</v>
+        <v>473</v>
       </c>
       <c r="D139" s="6"/>
       <c r="E139" s="6"/>
@@ -5751,13 +5810,13 @@
     </row>
     <row r="140" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A140" s="4" t="s">
-        <v>477</v>
+        <v>474</v>
       </c>
       <c r="B140" s="5" t="s">
-        <v>478</v>
+        <v>475</v>
       </c>
       <c r="C140" s="5" t="s">
-        <v>479</v>
+        <v>476</v>
       </c>
       <c r="D140" s="6"/>
       <c r="E140" s="6"/>
@@ -5773,13 +5832,13 @@
     </row>
     <row r="141" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A141" s="4" t="s">
-        <v>480</v>
+        <v>477</v>
       </c>
       <c r="B141" s="5" t="s">
-        <v>481</v>
+        <v>478</v>
       </c>
       <c r="C141" s="5" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
       <c r="D141" s="6"/>
       <c r="E141" s="6"/>
@@ -5795,13 +5854,13 @@
     </row>
     <row r="142" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A142" s="4" t="s">
-        <v>483</v>
+        <v>480</v>
       </c>
       <c r="B142" s="5" t="s">
-        <v>484</v>
+        <v>481</v>
       </c>
       <c r="C142" s="5" t="s">
-        <v>485</v>
+        <v>482</v>
       </c>
       <c r="D142" s="6"/>
       <c r="E142" s="6"/>
@@ -5817,13 +5876,13 @@
     </row>
     <row r="143" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A143" s="4" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="B143" s="5" t="s">
-        <v>487</v>
+        <v>484</v>
       </c>
       <c r="C143" s="5" t="s">
-        <v>488</v>
+        <v>485</v>
       </c>
       <c r="D143" s="6"/>
       <c r="E143" s="6"/>
@@ -5839,13 +5898,13 @@
     </row>
     <row r="144" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A144" s="4" t="s">
-        <v>489</v>
+        <v>486</v>
       </c>
       <c r="B144" s="5" t="s">
-        <v>490</v>
+        <v>487</v>
       </c>
       <c r="C144" s="5" t="s">
-        <v>491</v>
+        <v>488</v>
       </c>
       <c r="D144" s="6"/>
       <c r="E144" s="6"/>
@@ -5861,13 +5920,13 @@
     </row>
     <row r="145" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A145" s="4" t="s">
-        <v>492</v>
+        <v>489</v>
       </c>
       <c r="B145" s="5" t="s">
-        <v>493</v>
+        <v>490</v>
       </c>
       <c r="C145" s="5" t="s">
-        <v>494</v>
+        <v>491</v>
       </c>
       <c r="D145" s="6"/>
       <c r="E145" s="6"/>
@@ -5883,13 +5942,13 @@
     </row>
     <row r="146" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A146" s="4" t="s">
-        <v>495</v>
+        <v>492</v>
       </c>
       <c r="B146" s="5" t="s">
-        <v>496</v>
+        <v>493</v>
       </c>
       <c r="C146" s="5" t="s">
-        <v>497</v>
+        <v>494</v>
       </c>
       <c r="D146" s="6"/>
       <c r="E146" s="6"/>
@@ -5905,13 +5964,13 @@
     </row>
     <row r="147" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A147" s="4" t="s">
-        <v>498</v>
+        <v>495</v>
       </c>
       <c r="B147" s="5" t="s">
-        <v>499</v>
+        <v>496</v>
       </c>
       <c r="C147" s="5" t="s">
-        <v>500</v>
+        <v>497</v>
       </c>
       <c r="D147" s="6"/>
       <c r="E147" s="6"/>
@@ -5927,13 +5986,13 @@
     </row>
     <row r="148" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A148" s="4" t="s">
-        <v>501</v>
+        <v>498</v>
       </c>
       <c r="B148" s="5" t="s">
-        <v>502</v>
+        <v>499</v>
       </c>
       <c r="C148" s="5" t="s">
-        <v>503</v>
+        <v>500</v>
       </c>
       <c r="D148" s="6"/>
       <c r="E148" s="6"/>
@@ -5949,13 +6008,13 @@
     </row>
     <row r="149" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A149" s="4" t="s">
-        <v>504</v>
+        <v>501</v>
       </c>
       <c r="B149" s="5" t="s">
-        <v>505</v>
+        <v>502</v>
       </c>
       <c r="C149" s="5" t="s">
-        <v>506</v>
+        <v>503</v>
       </c>
       <c r="D149" s="6"/>
       <c r="E149" s="6"/>
@@ -5971,13 +6030,13 @@
     </row>
     <row r="150" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A150" s="4" t="s">
-        <v>507</v>
+        <v>504</v>
       </c>
       <c r="B150" s="5" t="s">
-        <v>508</v>
+        <v>505</v>
       </c>
       <c r="C150" s="5" t="s">
-        <v>509</v>
+        <v>506</v>
       </c>
       <c r="D150" s="6"/>
       <c r="E150" s="6"/>
@@ -5993,13 +6052,13 @@
     </row>
     <row r="151" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A151" s="4" t="s">
-        <v>510</v>
+        <v>507</v>
       </c>
       <c r="B151" s="5" t="s">
-        <v>511</v>
+        <v>508</v>
       </c>
       <c r="C151" s="5" t="s">
-        <v>512</v>
+        <v>509</v>
       </c>
       <c r="D151" s="6"/>
       <c r="E151" s="6"/>
@@ -6015,19 +6074,19 @@
     </row>
     <row r="152" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A152" s="4" t="s">
-        <v>513</v>
+        <v>510</v>
       </c>
       <c r="B152" s="5" t="s">
-        <v>514</v>
+        <v>511</v>
       </c>
       <c r="C152" s="5" t="s">
-        <v>515</v>
+        <v>512</v>
       </c>
       <c r="D152" s="6"/>
       <c r="E152" s="6"/>
       <c r="F152" s="6"/>
       <c r="G152" s="6" t="s">
-        <v>516</v>
+        <v>513</v>
       </c>
       <c r="H152" s="6"/>
       <c r="I152" s="6"/>
@@ -6039,13 +6098,13 @@
     </row>
     <row r="153" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A153" s="4" t="s">
-        <v>517</v>
+        <v>514</v>
       </c>
       <c r="B153" s="5" t="s">
-        <v>518</v>
+        <v>515</v>
       </c>
       <c r="C153" s="5" t="s">
-        <v>519</v>
+        <v>516</v>
       </c>
       <c r="D153" s="6"/>
       <c r="E153" s="6"/>
@@ -6061,13 +6120,13 @@
     </row>
     <row r="154" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A154" s="4" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
       <c r="B154" s="5" t="s">
-        <v>521</v>
+        <v>518</v>
       </c>
       <c r="C154" s="5" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
       <c r="D154" s="6"/>
       <c r="E154" s="6"/>
@@ -6083,13 +6142,13 @@
     </row>
     <row r="155" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A155" s="4" t="s">
-        <v>523</v>
+        <v>520</v>
       </c>
       <c r="B155" s="5" t="s">
-        <v>524</v>
+        <v>521</v>
       </c>
       <c r="C155" s="5" t="s">
-        <v>525</v>
+        <v>522</v>
       </c>
       <c r="D155" s="6"/>
       <c r="E155" s="6"/>
@@ -6105,13 +6164,13 @@
     </row>
     <row r="156" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A156" s="4" t="s">
-        <v>526</v>
+        <v>523</v>
       </c>
       <c r="B156" s="5" t="s">
-        <v>527</v>
+        <v>524</v>
       </c>
       <c r="C156" s="5" t="s">
-        <v>528</v>
+        <v>525</v>
       </c>
       <c r="D156" s="6"/>
       <c r="E156" s="6"/>
@@ -6127,13 +6186,13 @@
     </row>
     <row r="157" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A157" s="4" t="s">
-        <v>529</v>
+        <v>526</v>
       </c>
       <c r="B157" s="5" t="s">
-        <v>530</v>
+        <v>527</v>
       </c>
       <c r="C157" s="5" t="s">
-        <v>531</v>
+        <v>528</v>
       </c>
       <c r="D157" s="6"/>
       <c r="E157" s="6"/>
@@ -6149,13 +6208,13 @@
     </row>
     <row r="158" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A158" s="4" t="s">
-        <v>532</v>
+        <v>529</v>
       </c>
       <c r="B158" s="5" t="s">
-        <v>533</v>
+        <v>530</v>
       </c>
       <c r="C158" s="5" t="s">
-        <v>534</v>
+        <v>531</v>
       </c>
       <c r="D158" s="6"/>
       <c r="E158" s="6"/>
@@ -6171,13 +6230,13 @@
     </row>
     <row r="159" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A159" s="4" t="s">
-        <v>535</v>
+        <v>532</v>
       </c>
       <c r="B159" s="5" t="s">
-        <v>536</v>
+        <v>533</v>
       </c>
       <c r="C159" s="5" t="s">
-        <v>537</v>
+        <v>534</v>
       </c>
       <c r="D159" s="6"/>
       <c r="E159" s="6"/>
@@ -6193,13 +6252,13 @@
     </row>
     <row r="160" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A160" s="4" t="s">
-        <v>538</v>
+        <v>535</v>
       </c>
       <c r="B160" s="5" t="s">
-        <v>539</v>
+        <v>536</v>
       </c>
       <c r="C160" s="5" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
       <c r="D160" s="6"/>
       <c r="E160" s="6"/>
@@ -6215,13 +6274,13 @@
     </row>
     <row r="161" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A161" s="4" t="s">
-        <v>541</v>
+        <v>538</v>
       </c>
       <c r="B161" s="5" t="s">
-        <v>542</v>
+        <v>539</v>
       </c>
       <c r="C161" s="5" t="s">
-        <v>543</v>
+        <v>540</v>
       </c>
       <c r="D161" s="6"/>
       <c r="E161" s="6"/>
@@ -6237,19 +6296,19 @@
     </row>
     <row r="162" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A162" s="4" t="s">
-        <v>544</v>
+        <v>541</v>
       </c>
       <c r="B162" s="5" t="s">
-        <v>545</v>
+        <v>542</v>
       </c>
       <c r="C162" s="5" t="s">
-        <v>546</v>
+        <v>543</v>
       </c>
       <c r="D162" s="6"/>
       <c r="E162" s="6"/>
       <c r="F162" s="6"/>
       <c r="G162" s="6" t="s">
-        <v>547</v>
+        <v>544</v>
       </c>
       <c r="H162" s="6"/>
       <c r="I162" s="6"/>
@@ -6261,13 +6320,13 @@
     </row>
     <row r="163" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A163" s="4" t="s">
-        <v>548</v>
+        <v>545</v>
       </c>
       <c r="B163" s="5" t="s">
-        <v>549</v>
+        <v>546</v>
       </c>
       <c r="C163" s="5" t="s">
-        <v>550</v>
+        <v>547</v>
       </c>
       <c r="D163" s="6"/>
       <c r="E163" s="6"/>
@@ -6283,13 +6342,13 @@
     </row>
     <row r="164" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A164" s="4" t="s">
-        <v>551</v>
+        <v>548</v>
       </c>
       <c r="B164" s="5" t="s">
-        <v>552</v>
+        <v>549</v>
       </c>
       <c r="C164" s="5" t="s">
-        <v>553</v>
+        <v>550</v>
       </c>
       <c r="D164" s="6"/>
       <c r="E164" s="6"/>
@@ -6305,13 +6364,13 @@
     </row>
     <row r="165" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A165" s="4" t="s">
-        <v>554</v>
+        <v>551</v>
       </c>
       <c r="B165" s="5" t="s">
-        <v>555</v>
+        <v>552</v>
       </c>
       <c r="C165" s="5" t="s">
-        <v>556</v>
+        <v>553</v>
       </c>
       <c r="D165" s="6"/>
       <c r="E165" s="6"/>
@@ -6327,13 +6386,13 @@
     </row>
     <row r="166" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A166" s="4" t="s">
-        <v>557</v>
+        <v>554</v>
       </c>
       <c r="B166" s="5" t="s">
-        <v>558</v>
+        <v>555</v>
       </c>
       <c r="C166" s="5" t="s">
-        <v>559</v>
+        <v>556</v>
       </c>
       <c r="D166" s="6"/>
       <c r="E166" s="6"/>
@@ -6349,13 +6408,13 @@
     </row>
     <row r="167" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A167" s="4" t="s">
-        <v>560</v>
+        <v>557</v>
       </c>
       <c r="B167" s="5" t="s">
-        <v>561</v>
+        <v>558</v>
       </c>
       <c r="C167" s="5" t="s">
-        <v>562</v>
+        <v>559</v>
       </c>
       <c r="D167" s="6"/>
       <c r="E167" s="6"/>
@@ -6374,10 +6433,10 @@
     <row r="168" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A168" s="5"/>
       <c r="B168" s="5" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
       <c r="C168" s="5" t="s">
-        <v>564</v>
+        <v>561</v>
       </c>
       <c r="D168" s="6"/>
       <c r="E168" s="6"/>
@@ -6392,10 +6451,10 @@
     <row r="169" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A169" s="5"/>
       <c r="B169" s="5" t="s">
-        <v>565</v>
+        <v>562</v>
       </c>
       <c r="C169" s="5" t="s">
-        <v>566</v>
+        <v>563</v>
       </c>
       <c r="D169" s="6"/>
       <c r="E169" s="6"/>
@@ -6410,10 +6469,10 @@
     <row r="170" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A170" s="5"/>
       <c r="B170" s="5" t="s">
-        <v>567</v>
+        <v>564</v>
       </c>
       <c r="C170" s="5" t="s">
-        <v>568</v>
+        <v>565</v>
       </c>
       <c r="D170" s="6"/>
       <c r="E170" s="6"/>
@@ -6428,10 +6487,10 @@
     <row r="171" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A171" s="5"/>
       <c r="B171" s="5" t="s">
-        <v>569</v>
+        <v>566</v>
       </c>
       <c r="C171" s="5" t="s">
-        <v>570</v>
+        <v>567</v>
       </c>
       <c r="D171" s="6"/>
       <c r="E171" s="6"/>
@@ -6446,10 +6505,10 @@
     <row r="172" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A172" s="5"/>
       <c r="B172" s="5" t="s">
-        <v>571</v>
+        <v>568</v>
       </c>
       <c r="C172" s="5" t="s">
-        <v>572</v>
+        <v>569</v>
       </c>
       <c r="D172" s="6"/>
       <c r="E172" s="6"/>
@@ -6464,16 +6523,16 @@
     <row r="173" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A173" s="5"/>
       <c r="B173" s="5" t="s">
-        <v>573</v>
+        <v>570</v>
       </c>
       <c r="C173" s="5" t="s">
-        <v>574</v>
+        <v>571</v>
       </c>
       <c r="D173" s="6"/>
       <c r="E173" s="6"/>
       <c r="F173" s="6"/>
       <c r="G173" s="6" t="s">
-        <v>575</v>
+        <v>572</v>
       </c>
       <c r="H173" s="6"/>
       <c r="I173" s="6"/>
@@ -6484,10 +6543,10 @@
     <row r="174" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A174" s="5"/>
       <c r="B174" s="5" t="s">
-        <v>576</v>
+        <v>573</v>
       </c>
       <c r="C174" s="5" t="s">
-        <v>577</v>
+        <v>574</v>
       </c>
       <c r="D174" s="6"/>
       <c r="E174" s="6"/>
@@ -6502,10 +6561,10 @@
     <row r="175" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A175" s="5"/>
       <c r="B175" s="5" t="s">
-        <v>578</v>
+        <v>575</v>
       </c>
       <c r="C175" s="5" t="s">
-        <v>579</v>
+        <v>576</v>
       </c>
       <c r="D175" s="6"/>
       <c r="E175" s="6"/>
@@ -6520,10 +6579,10 @@
     <row r="176" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A176" s="5"/>
       <c r="B176" s="5" t="s">
-        <v>580</v>
+        <v>577</v>
       </c>
       <c r="C176" s="5" t="s">
-        <v>581</v>
+        <v>578</v>
       </c>
       <c r="D176" s="6"/>
       <c r="E176" s="6"/>
@@ -6538,10 +6597,10 @@
     <row r="177" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A177" s="5"/>
       <c r="B177" s="5" t="s">
-        <v>582</v>
+        <v>579</v>
       </c>
       <c r="C177" s="5" t="s">
-        <v>583</v>
+        <v>580</v>
       </c>
       <c r="D177" s="6"/>
       <c r="E177" s="6"/>
@@ -6556,10 +6615,10 @@
     <row r="178" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A178" s="5"/>
       <c r="B178" s="5" t="s">
-        <v>584</v>
+        <v>581</v>
       </c>
       <c r="C178" s="5" t="s">
-        <v>585</v>
+        <v>582</v>
       </c>
       <c r="D178" s="6"/>
       <c r="E178" s="6"/>
@@ -6574,10 +6633,10 @@
     <row r="179" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A179" s="5"/>
       <c r="B179" s="5" t="s">
-        <v>586</v>
+        <v>583</v>
       </c>
       <c r="C179" s="5" t="s">
-        <v>587</v>
+        <v>584</v>
       </c>
       <c r="D179" s="6"/>
       <c r="E179" s="6"/>
@@ -6592,10 +6651,10 @@
     <row r="180" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A180" s="5"/>
       <c r="B180" s="5" t="s">
-        <v>588</v>
+        <v>585</v>
       </c>
       <c r="C180" s="5" t="s">
-        <v>589</v>
+        <v>586</v>
       </c>
       <c r="D180" s="6"/>
       <c r="E180" s="6"/>
@@ -6610,10 +6669,10 @@
     <row r="181" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A181" s="5"/>
       <c r="B181" s="5" t="s">
-        <v>590</v>
+        <v>587</v>
       </c>
       <c r="C181" s="5" t="s">
-        <v>591</v>
+        <v>588</v>
       </c>
       <c r="D181" s="6"/>
       <c r="E181" s="6"/>
@@ -6628,10 +6687,10 @@
     <row r="182" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A182" s="5"/>
       <c r="B182" s="5" t="s">
-        <v>592</v>
+        <v>589</v>
       </c>
       <c r="C182" s="5" t="s">
-        <v>593</v>
+        <v>590</v>
       </c>
       <c r="D182" s="6"/>
       <c r="E182" s="6"/>
@@ -6646,10 +6705,10 @@
     <row r="183" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A183" s="5"/>
       <c r="B183" s="5" t="s">
-        <v>594</v>
+        <v>591</v>
       </c>
       <c r="C183" s="5" t="s">
-        <v>595</v>
+        <v>592</v>
       </c>
       <c r="D183" s="6"/>
       <c r="E183" s="6"/>
@@ -18310,20 +18369,14 @@
       <c r="L1015" s="6"/>
     </row>
     <row r="1016" spans="1:12" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1016" s="5" t="inlineStr">
-        <is>
-          <t>SCN-001</t>
-        </is>
-      </c>
-      <c r="B1016" s="5" t="inlineStr">
-        <is>
-          <t>Zombie Apocalypse</t>
-        </is>
-      </c>
-      <c r="C1016" s="5" t="inlineStr">
-        <is>
-          <t>Triggerable scenario. Manual setup launched from the Chaos Redux scenario window. Type controls outbreak profile/structure; intensity controls outbreak count, starting affected states, divisions, and early pressure.</t>
-        </is>
+      <c r="A1016" s="5" t="s">
+        <v>598</v>
+      </c>
+      <c r="B1016" s="5" t="s">
+        <v>599</v>
+      </c>
+      <c r="C1016" s="5" t="s">
+        <v>600</v>
       </c>
       <c r="D1016" s="6"/>
       <c r="E1016" s="6"/>
@@ -18331,37 +18384,25 @@
       <c r="G1016" s="6"/>
       <c r="H1016" s="6"/>
       <c r="I1016" s="6"/>
-      <c r="J1016" s="6" t="inlineStr">
-        <is>
-          <t>Manual triggerable scenario</t>
-        </is>
-      </c>
-      <c r="K1016" s="6" t="inlineStr">
-        <is>
-          <t>Manual Scenario</t>
-        </is>
-      </c>
-      <c r="L1016" s="6" t="inlineStr">
-        <is>
-          <t>Implemented</t>
-        </is>
+      <c r="J1016" s="6" t="s">
+        <v>601</v>
+      </c>
+      <c r="K1016" s="6" t="s">
+        <v>602</v>
+      </c>
+      <c r="L1016" s="6" t="s">
+        <v>603</v>
       </c>
     </row>
     <row r="1017" spans="1:12" ht="72" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1017" s="5" t="inlineStr">
-        <is>
-          <t>SCN-002</t>
-        </is>
-      </c>
-      <c r="B1017" s="5" t="inlineStr">
-        <is>
-          <t>Army of Mengele Clones</t>
-        </is>
-      </c>
-      <c r="C1017" s="5" t="inlineStr">
-        <is>
-          <t>Triggerable scenario. Manual setup launched from the Chaos Redux scenario window. Type switches between the standard clone army and the stronger Aryan variant; intensity controls starting territory, division count, army strength, equipment, and neighboring pressure.</t>
-        </is>
+      <c r="A1017" s="5" t="s">
+        <v>604</v>
+      </c>
+      <c r="B1017" s="5" t="s">
+        <v>605</v>
+      </c>
+      <c r="C1017" s="5" t="s">
+        <v>606</v>
       </c>
       <c r="D1017" s="6"/>
       <c r="E1017" s="6"/>
@@ -18369,20 +18410,14 @@
       <c r="G1017" s="6"/>
       <c r="H1017" s="6"/>
       <c r="I1017" s="6"/>
-      <c r="J1017" s="6" t="inlineStr">
-        <is>
-          <t>Manual triggerable scenario</t>
-        </is>
-      </c>
-      <c r="K1017" s="6" t="inlineStr">
-        <is>
-          <t>Manual Scenario</t>
-        </is>
-      </c>
-      <c r="L1017" s="6" t="inlineStr">
-        <is>
-          <t>Implemented</t>
-        </is>
+      <c r="J1017" s="6" t="s">
+        <v>601</v>
+      </c>
+      <c r="K1017" s="6" t="s">
+        <v>602</v>
+      </c>
+      <c r="L1017" s="6" t="s">
+        <v>603</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
final fixes and added missing assets
</commit_message>
<xml_diff>
--- a/docs/spreadsheets/chaos_redux_events_catalog.xlsx
+++ b/docs/spreadsheets/chaos_redux_events_catalog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\home\klim\projects\chaos_redux\docs\spreadsheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{258FF301-4A1A-49CF-B218-A80F6D29A05D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{654CBF13-214A-458E-AFA9-9C0DD2C2BB93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="891" uniqueCount="611">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="892" uniqueCount="610">
   <si>
     <t>ID</t>
   </si>
@@ -187,9 +187,6 @@
     <t>Soviet Union Collapse</t>
   </si>
   <si>
-    <t>Further collapse if the crisis is not managed.</t>
-  </si>
-  <si>
     <t>Diseases</t>
   </si>
   <si>
@@ -199,9 +196,6 @@
     <t>Independence Wave</t>
   </si>
   <si>
-    <t>Three random countries that do not exist will declare their independence.</t>
-  </si>
-  <si>
     <t>Aliens</t>
   </si>
   <si>
@@ -1855,7 +1849,10 @@
     <t>4, (later add more)</t>
   </si>
   <si>
-    <t xml:space="preserve">Soviet Union releases some countries inside its territory, and more countries through like crisis maybe if not contained. Those countries will get free divisions, so that the soviet union wouldn't be able to invade them easily right away. Soviet Union gets decisions to reclaim the broken away states. The broken away states can form a coalition (like a faction to fight the soviet union), their goal is to completely make every possible country inside soviet union a free democratic country. </t>
+    <t>to be reworked</t>
+  </si>
+  <si>
+    <t>Liberations</t>
   </si>
 </sst>
 </file>
@@ -2062,7 +2059,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Event_Clusters" displayName="Event_Clusters" ref="N1:R15">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Event_Clusters" displayName="Event_Clusters" ref="N1:R16">
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Cluster Name"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Details"/>
@@ -2494,22 +2491,22 @@
         <v>48</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>607</v>
+        <v>605</v>
       </c>
       <c r="D5" s="6" t="s">
+        <v>591</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>592</v>
+      </c>
+      <c r="F5" s="6" t="s">
         <v>593</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="G5" s="6" t="s">
         <v>594</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="H5" s="6" t="s">
         <v>595</v>
-      </c>
-      <c r="G5" s="6" t="s">
-        <v>596</v>
-      </c>
-      <c r="H5" s="6" t="s">
-        <v>597</v>
       </c>
       <c r="I5" s="6"/>
       <c r="J5" s="6"/>
@@ -2523,10 +2520,10 @@
         <v>51</v>
       </c>
       <c r="O5" s="8" t="s">
-        <v>608</v>
+        <v>606</v>
       </c>
       <c r="P5" s="8" t="s">
-        <v>609</v>
+        <v>607</v>
       </c>
       <c r="Q5" s="8">
         <v>2</v>
@@ -2543,14 +2540,12 @@
         <v>53</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>610</v>
+        <v>608</v>
       </c>
       <c r="D6" s="6"/>
       <c r="E6" s="6"/>
       <c r="F6" s="6"/>
-      <c r="G6" s="6" t="s">
-        <v>54</v>
-      </c>
+      <c r="G6" s="6"/>
       <c r="H6" s="6"/>
       <c r="I6" s="6"/>
       <c r="J6" s="6"/>
@@ -2561,7 +2556,7 @@
         <v>50</v>
       </c>
       <c r="N6" s="7" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="O6" s="8"/>
       <c r="P6" s="8"/>
@@ -2574,13 +2569,13 @@
     </row>
     <row r="7" spans="1:18" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="B7" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="B7" s="5" t="s">
-        <v>57</v>
-      </c>
       <c r="C7" s="5" t="s">
-        <v>58</v>
+        <v>608</v>
       </c>
       <c r="D7" s="6"/>
       <c r="E7" s="6"/>
@@ -2596,7 +2591,7 @@
         <v>50</v>
       </c>
       <c r="N7" s="7" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="O7" s="8"/>
       <c r="P7" s="8"/>
@@ -2609,13 +2604,13 @@
     </row>
     <row r="8" spans="1:18" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="C8" s="5" t="s">
         <v>60</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>62</v>
       </c>
       <c r="D8" s="6"/>
       <c r="E8" s="6"/>
@@ -2631,10 +2626,10 @@
         <v>50</v>
       </c>
       <c r="N8" s="7" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="O8" s="8" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="P8" s="8"/>
       <c r="Q8" s="8">
@@ -2646,13 +2641,13 @@
     </row>
     <row r="9" spans="1:18" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="C9" s="5" t="s">
         <v>65</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>67</v>
       </c>
       <c r="D9" s="6"/>
       <c r="E9" s="6"/>
@@ -2668,7 +2663,7 @@
         <v>50</v>
       </c>
       <c r="N9" s="7" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="O9" s="8"/>
       <c r="P9" s="8"/>
@@ -2681,13 +2676,13 @@
     </row>
     <row r="10" spans="1:18" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C10" s="5" t="s">
         <v>69</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>71</v>
       </c>
       <c r="D10" s="6"/>
       <c r="E10" s="6"/>
@@ -2703,7 +2698,7 @@
         <v>50</v>
       </c>
       <c r="N10" s="7" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="O10" s="8"/>
       <c r="P10" s="8"/>
@@ -2716,13 +2711,13 @@
     </row>
     <row r="11" spans="1:18" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="C11" s="5" t="s">
         <v>73</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>75</v>
       </c>
       <c r="D11" s="6"/>
       <c r="E11" s="6"/>
@@ -2738,10 +2733,10 @@
         <v>50</v>
       </c>
       <c r="N11" s="7" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="O11" s="8" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="P11" s="8"/>
       <c r="Q11" s="8">
@@ -2753,13 +2748,13 @@
     </row>
     <row r="12" spans="1:18" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="C12" s="5" t="s">
         <v>78</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>80</v>
       </c>
       <c r="D12" s="6"/>
       <c r="E12" s="6"/>
@@ -2775,10 +2770,10 @@
         <v>50</v>
       </c>
       <c r="N12" s="7" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="O12" s="8" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="P12" s="8"/>
       <c r="Q12" s="8">
@@ -2790,13 +2785,13 @@
     </row>
     <row r="13" spans="1:18" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="C13" s="5" t="s">
         <v>83</v>
-      </c>
-      <c r="B13" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>85</v>
       </c>
       <c r="D13" s="6"/>
       <c r="E13" s="6"/>
@@ -2812,7 +2807,7 @@
         <v>50</v>
       </c>
       <c r="N13" s="7" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="O13" s="8"/>
       <c r="P13" s="8"/>
@@ -2825,19 +2820,19 @@
     </row>
     <row r="14" spans="1:18" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="4" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="D14" s="6"/>
       <c r="E14" s="6"/>
       <c r="F14" s="6"/>
       <c r="G14" s="6" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="H14" s="6"/>
       <c r="I14" s="6"/>
@@ -2849,7 +2844,7 @@
         <v>50</v>
       </c>
       <c r="N14" s="7" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="O14" s="8"/>
       <c r="P14" s="8"/>
@@ -2862,13 +2857,13 @@
     </row>
     <row r="15" spans="1:18" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="C15" s="5" t="s">
         <v>91</v>
-      </c>
-      <c r="B15" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>93</v>
       </c>
       <c r="D15" s="6"/>
       <c r="E15" s="6"/>
@@ -2884,10 +2879,10 @@
         <v>50</v>
       </c>
       <c r="N15" s="7" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="O15" s="8" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="P15" s="8"/>
       <c r="Q15" s="8">
@@ -2899,13 +2894,13 @@
     </row>
     <row r="16" spans="1:18" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="C16" s="5" t="s">
         <v>96</v>
-      </c>
-      <c r="B16" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>98</v>
       </c>
       <c r="D16" s="6"/>
       <c r="E16" s="6"/>
@@ -2920,16 +2915,25 @@
       <c r="L16" s="6" t="s">
         <v>50</v>
       </c>
+      <c r="N16" t="s">
+        <v>609</v>
+      </c>
+      <c r="Q16">
+        <v>1</v>
+      </c>
+      <c r="R16" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="17" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="C17" s="5" t="s">
         <v>99</v>
-      </c>
-      <c r="B17" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="C17" s="5" t="s">
-        <v>101</v>
       </c>
       <c r="D17" s="6"/>
       <c r="E17" s="6"/>
@@ -2947,13 +2951,13 @@
     </row>
     <row r="18" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="C18" s="5" t="s">
         <v>102</v>
-      </c>
-      <c r="B18" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="C18" s="5" t="s">
-        <v>104</v>
       </c>
       <c r="D18" s="6"/>
       <c r="E18" s="6"/>
@@ -2971,13 +2975,13 @@
     </row>
     <row r="19" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="C19" s="5" t="s">
         <v>105</v>
-      </c>
-      <c r="B19" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="C19" s="5" t="s">
-        <v>107</v>
       </c>
       <c r="D19" s="6"/>
       <c r="E19" s="6"/>
@@ -2995,13 +2999,13 @@
     </row>
     <row r="20" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="C20" s="5" t="s">
         <v>108</v>
-      </c>
-      <c r="B20" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="C20" s="5" t="s">
-        <v>110</v>
       </c>
       <c r="D20" s="6"/>
       <c r="E20" s="6"/>
@@ -3019,19 +3023,19 @@
     </row>
     <row r="21" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="C21" s="5" t="s">
         <v>111</v>
-      </c>
-      <c r="B21" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="C21" s="5" t="s">
-        <v>113</v>
       </c>
       <c r="D21" s="6"/>
       <c r="E21" s="6"/>
       <c r="F21" s="6"/>
       <c r="G21" s="6" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H21" s="6"/>
       <c r="I21" s="6"/>
@@ -3045,13 +3049,13 @@
     </row>
     <row r="22" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="C22" s="5" t="s">
         <v>115</v>
-      </c>
-      <c r="B22" s="5" t="s">
-        <v>116</v>
-      </c>
-      <c r="C22" s="5" t="s">
-        <v>117</v>
       </c>
       <c r="D22" s="6"/>
       <c r="E22" s="6"/>
@@ -3067,18 +3071,18 @@
         <v>50</v>
       </c>
       <c r="Q22" s="9" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
     <row r="23" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="C23" s="5" t="s">
         <v>119</v>
-      </c>
-      <c r="B23" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="C23" s="5" t="s">
-        <v>121</v>
       </c>
       <c r="D23" s="6"/>
       <c r="E23" s="6"/>
@@ -3096,13 +3100,13 @@
     </row>
     <row r="24" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="C24" s="5" t="s">
         <v>122</v>
-      </c>
-      <c r="B24" s="5" t="s">
-        <v>123</v>
-      </c>
-      <c r="C24" s="5" t="s">
-        <v>124</v>
       </c>
       <c r="D24" s="6"/>
       <c r="E24" s="6"/>
@@ -3120,13 +3124,13 @@
     </row>
     <row r="25" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="C25" s="5" t="s">
         <v>125</v>
-      </c>
-      <c r="B25" s="5" t="s">
-        <v>126</v>
-      </c>
-      <c r="C25" s="5" t="s">
-        <v>127</v>
       </c>
       <c r="D25" s="6"/>
       <c r="E25" s="6"/>
@@ -3144,13 +3148,13 @@
     </row>
     <row r="26" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="C26" s="5" t="s">
         <v>128</v>
-      </c>
-      <c r="B26" s="5" t="s">
-        <v>129</v>
-      </c>
-      <c r="C26" s="5" t="s">
-        <v>130</v>
       </c>
       <c r="D26" s="6"/>
       <c r="E26" s="6"/>
@@ -3168,13 +3172,13 @@
     </row>
     <row r="27" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="B27" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="C27" s="5" t="s">
         <v>131</v>
-      </c>
-      <c r="B27" s="5" t="s">
-        <v>132</v>
-      </c>
-      <c r="C27" s="5" t="s">
-        <v>133</v>
       </c>
       <c r="D27" s="6"/>
       <c r="E27" s="6"/>
@@ -3192,13 +3196,13 @@
     </row>
     <row r="28" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="C28" s="5" t="s">
         <v>134</v>
-      </c>
-      <c r="B28" s="5" t="s">
-        <v>135</v>
-      </c>
-      <c r="C28" s="5" t="s">
-        <v>136</v>
       </c>
       <c r="D28" s="6"/>
       <c r="E28" s="6"/>
@@ -3216,13 +3220,13 @@
     </row>
     <row r="29" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="B29" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="C29" s="5" t="s">
         <v>137</v>
-      </c>
-      <c r="B29" s="5" t="s">
-        <v>138</v>
-      </c>
-      <c r="C29" s="5" t="s">
-        <v>139</v>
       </c>
       <c r="D29" s="6"/>
       <c r="E29" s="6"/>
@@ -3240,13 +3244,13 @@
     </row>
     <row r="30" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="C30" s="5" t="s">
         <v>140</v>
-      </c>
-      <c r="B30" s="5" t="s">
-        <v>141</v>
-      </c>
-      <c r="C30" s="5" t="s">
-        <v>142</v>
       </c>
       <c r="D30" s="6"/>
       <c r="E30" s="6"/>
@@ -3264,19 +3268,19 @@
     </row>
     <row r="31" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="B31" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="C31" s="5" t="s">
         <v>143</v>
-      </c>
-      <c r="B31" s="5" t="s">
-        <v>144</v>
-      </c>
-      <c r="C31" s="5" t="s">
-        <v>145</v>
       </c>
       <c r="D31" s="6"/>
       <c r="E31" s="6"/>
       <c r="F31" s="6"/>
       <c r="G31" s="6" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="H31" s="6"/>
       <c r="I31" s="6"/>
@@ -3290,13 +3294,13 @@
     </row>
     <row r="32" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="B32" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="C32" s="5" t="s">
         <v>147</v>
-      </c>
-      <c r="B32" s="5" t="s">
-        <v>148</v>
-      </c>
-      <c r="C32" s="5" t="s">
-        <v>149</v>
       </c>
       <c r="D32" s="6"/>
       <c r="E32" s="6"/>
@@ -3314,13 +3318,13 @@
     </row>
     <row r="33" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="C33" s="5" t="s">
         <v>150</v>
-      </c>
-      <c r="B33" s="5" t="s">
-        <v>151</v>
-      </c>
-      <c r="C33" s="5" t="s">
-        <v>152</v>
       </c>
       <c r="D33" s="6"/>
       <c r="E33" s="6"/>
@@ -3338,13 +3342,13 @@
     </row>
     <row r="34" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="B34" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C34" s="5" t="s">
         <v>153</v>
-      </c>
-      <c r="B34" s="5" t="s">
-        <v>154</v>
-      </c>
-      <c r="C34" s="5" t="s">
-        <v>155</v>
       </c>
       <c r="D34" s="6"/>
       <c r="E34" s="6"/>
@@ -3362,13 +3366,13 @@
     </row>
     <row r="35" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="C35" s="5" t="s">
         <v>156</v>
-      </c>
-      <c r="B35" s="5" t="s">
-        <v>157</v>
-      </c>
-      <c r="C35" s="5" t="s">
-        <v>158</v>
       </c>
       <c r="D35" s="6"/>
       <c r="E35" s="6"/>
@@ -3386,13 +3390,13 @@
     </row>
     <row r="36" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="B36" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="C36" s="5" t="s">
         <v>159</v>
-      </c>
-      <c r="B36" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="C36" s="5" t="s">
-        <v>161</v>
       </c>
       <c r="D36" s="6"/>
       <c r="E36" s="6"/>
@@ -3410,13 +3414,13 @@
     </row>
     <row r="37" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="B37" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="C37" s="5" t="s">
         <v>162</v>
-      </c>
-      <c r="B37" s="5" t="s">
-        <v>163</v>
-      </c>
-      <c r="C37" s="5" t="s">
-        <v>164</v>
       </c>
       <c r="D37" s="6"/>
       <c r="E37" s="6"/>
@@ -3434,13 +3438,13 @@
     </row>
     <row r="38" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="B38" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="C38" s="5" t="s">
         <v>165</v>
-      </c>
-      <c r="B38" s="5" t="s">
-        <v>166</v>
-      </c>
-      <c r="C38" s="5" t="s">
-        <v>167</v>
       </c>
       <c r="D38" s="6"/>
       <c r="E38" s="6"/>
@@ -3458,19 +3462,19 @@
     </row>
     <row r="39" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="B39" s="5" t="s">
+        <v>167</v>
+      </c>
+      <c r="C39" s="5" t="s">
         <v>168</v>
-      </c>
-      <c r="B39" s="5" t="s">
-        <v>169</v>
-      </c>
-      <c r="C39" s="5" t="s">
-        <v>170</v>
       </c>
       <c r="D39" s="6"/>
       <c r="E39" s="6"/>
       <c r="F39" s="6"/>
       <c r="G39" s="6" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="H39" s="6"/>
       <c r="I39" s="6"/>
@@ -3484,13 +3488,13 @@
     </row>
     <row r="40" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="B40" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="C40" s="5" t="s">
         <v>172</v>
-      </c>
-      <c r="B40" s="5" t="s">
-        <v>173</v>
-      </c>
-      <c r="C40" s="5" t="s">
-        <v>174</v>
       </c>
       <c r="D40" s="6"/>
       <c r="E40" s="6"/>
@@ -3508,13 +3512,13 @@
     </row>
     <row r="41" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="B41" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="C41" s="5" t="s">
         <v>175</v>
-      </c>
-      <c r="B41" s="5" t="s">
-        <v>176</v>
-      </c>
-      <c r="C41" s="5" t="s">
-        <v>177</v>
       </c>
       <c r="D41" s="6"/>
       <c r="E41" s="6"/>
@@ -3532,13 +3536,13 @@
     </row>
     <row r="42" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="B42" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="C42" s="5" t="s">
         <v>178</v>
-      </c>
-      <c r="B42" s="5" t="s">
-        <v>179</v>
-      </c>
-      <c r="C42" s="5" t="s">
-        <v>180</v>
       </c>
       <c r="D42" s="6"/>
       <c r="E42" s="6"/>
@@ -3556,13 +3560,13 @@
     </row>
     <row r="43" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="B43" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="C43" s="5" t="s">
         <v>181</v>
-      </c>
-      <c r="B43" s="5" t="s">
-        <v>182</v>
-      </c>
-      <c r="C43" s="5" t="s">
-        <v>183</v>
       </c>
       <c r="D43" s="6"/>
       <c r="E43" s="6"/>
@@ -3580,13 +3584,13 @@
     </row>
     <row r="44" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="B44" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="C44" s="5" t="s">
         <v>184</v>
-      </c>
-      <c r="B44" s="5" t="s">
-        <v>185</v>
-      </c>
-      <c r="C44" s="5" t="s">
-        <v>186</v>
       </c>
       <c r="D44" s="6"/>
       <c r="E44" s="6"/>
@@ -3604,13 +3608,13 @@
     </row>
     <row r="45" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="B45" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="C45" s="5" t="s">
         <v>187</v>
-      </c>
-      <c r="B45" s="5" t="s">
-        <v>188</v>
-      </c>
-      <c r="C45" s="5" t="s">
-        <v>189</v>
       </c>
       <c r="D45" s="6"/>
       <c r="E45" s="6"/>
@@ -3628,13 +3632,13 @@
     </row>
     <row r="46" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="B46" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="C46" s="5" t="s">
         <v>190</v>
-      </c>
-      <c r="B46" s="5" t="s">
-        <v>191</v>
-      </c>
-      <c r="C46" s="5" t="s">
-        <v>192</v>
       </c>
       <c r="D46" s="6"/>
       <c r="E46" s="6"/>
@@ -3652,13 +3656,13 @@
     </row>
     <row r="47" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="B47" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="C47" s="5" t="s">
         <v>193</v>
-      </c>
-      <c r="B47" s="5" t="s">
-        <v>194</v>
-      </c>
-      <c r="C47" s="5" t="s">
-        <v>195</v>
       </c>
       <c r="D47" s="6"/>
       <c r="E47" s="6"/>
@@ -3676,13 +3680,13 @@
     </row>
     <row r="48" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="B48" s="5" t="s">
+        <v>195</v>
+      </c>
+      <c r="C48" s="5" t="s">
         <v>196</v>
-      </c>
-      <c r="B48" s="5" t="s">
-        <v>197</v>
-      </c>
-      <c r="C48" s="5" t="s">
-        <v>198</v>
       </c>
       <c r="D48" s="6"/>
       <c r="E48" s="6"/>
@@ -3700,13 +3704,13 @@
     </row>
     <row r="49" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="B49" s="5" t="s">
+        <v>198</v>
+      </c>
+      <c r="C49" s="5" t="s">
         <v>199</v>
-      </c>
-      <c r="B49" s="5" t="s">
-        <v>200</v>
-      </c>
-      <c r="C49" s="5" t="s">
-        <v>201</v>
       </c>
       <c r="D49" s="6"/>
       <c r="E49" s="6"/>
@@ -3724,13 +3728,13 @@
     </row>
     <row r="50" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="B50" s="5" t="s">
+        <v>201</v>
+      </c>
+      <c r="C50" s="5" t="s">
         <v>202</v>
-      </c>
-      <c r="B50" s="5" t="s">
-        <v>203</v>
-      </c>
-      <c r="C50" s="5" t="s">
-        <v>204</v>
       </c>
       <c r="D50" s="6"/>
       <c r="E50" s="6"/>
@@ -3748,13 +3752,13 @@
     </row>
     <row r="51" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="B51" s="5" t="s">
+        <v>204</v>
+      </c>
+      <c r="C51" s="5" t="s">
         <v>205</v>
-      </c>
-      <c r="B51" s="5" t="s">
-        <v>206</v>
-      </c>
-      <c r="C51" s="5" t="s">
-        <v>207</v>
       </c>
       <c r="D51" s="6"/>
       <c r="E51" s="6"/>
@@ -3772,13 +3776,13 @@
     </row>
     <row r="52" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="B52" s="5" t="s">
+        <v>207</v>
+      </c>
+      <c r="C52" s="5" t="s">
         <v>208</v>
-      </c>
-      <c r="B52" s="5" t="s">
-        <v>209</v>
-      </c>
-      <c r="C52" s="5" t="s">
-        <v>210</v>
       </c>
       <c r="D52" s="6"/>
       <c r="E52" s="6"/>
@@ -3796,13 +3800,13 @@
     </row>
     <row r="53" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="B53" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="C53" s="5" t="s">
         <v>211</v>
-      </c>
-      <c r="B53" s="5" t="s">
-        <v>212</v>
-      </c>
-      <c r="C53" s="5" t="s">
-        <v>213</v>
       </c>
       <c r="D53" s="6"/>
       <c r="E53" s="6"/>
@@ -3820,13 +3824,13 @@
     </row>
     <row r="54" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="B54" s="5" t="s">
+        <v>213</v>
+      </c>
+      <c r="C54" s="5" t="s">
         <v>214</v>
-      </c>
-      <c r="B54" s="5" t="s">
-        <v>215</v>
-      </c>
-      <c r="C54" s="5" t="s">
-        <v>216</v>
       </c>
       <c r="D54" s="6"/>
       <c r="E54" s="6"/>
@@ -3844,13 +3848,13 @@
     </row>
     <row r="55" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="B55" s="5" t="s">
+        <v>216</v>
+      </c>
+      <c r="C55" s="5" t="s">
         <v>217</v>
-      </c>
-      <c r="B55" s="5" t="s">
-        <v>218</v>
-      </c>
-      <c r="C55" s="5" t="s">
-        <v>219</v>
       </c>
       <c r="D55" s="6"/>
       <c r="E55" s="6"/>
@@ -3868,13 +3872,13 @@
     </row>
     <row r="56" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="4" t="s">
+        <v>218</v>
+      </c>
+      <c r="B56" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="C56" s="5" t="s">
         <v>220</v>
-      </c>
-      <c r="B56" s="5" t="s">
-        <v>221</v>
-      </c>
-      <c r="C56" s="5" t="s">
-        <v>222</v>
       </c>
       <c r="D56" s="6"/>
       <c r="E56" s="6"/>
@@ -3892,13 +3896,13 @@
     </row>
     <row r="57" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="B57" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="C57" s="5" t="s">
         <v>223</v>
-      </c>
-      <c r="B57" s="5" t="s">
-        <v>224</v>
-      </c>
-      <c r="C57" s="5" t="s">
-        <v>225</v>
       </c>
       <c r="D57" s="6"/>
       <c r="E57" s="6"/>
@@ -3916,13 +3920,13 @@
     </row>
     <row r="58" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="B58" s="5" t="s">
+        <v>225</v>
+      </c>
+      <c r="C58" s="5" t="s">
         <v>226</v>
-      </c>
-      <c r="B58" s="5" t="s">
-        <v>227</v>
-      </c>
-      <c r="C58" s="5" t="s">
-        <v>228</v>
       </c>
       <c r="D58" s="6"/>
       <c r="E58" s="6"/>
@@ -3940,13 +3944,13 @@
     </row>
     <row r="59" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="B59" s="5" t="s">
+        <v>228</v>
+      </c>
+      <c r="C59" s="5" t="s">
         <v>229</v>
-      </c>
-      <c r="B59" s="5" t="s">
-        <v>230</v>
-      </c>
-      <c r="C59" s="5" t="s">
-        <v>231</v>
       </c>
       <c r="D59" s="6"/>
       <c r="E59" s="6"/>
@@ -3964,13 +3968,13 @@
     </row>
     <row r="60" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="4" t="s">
+        <v>230</v>
+      </c>
+      <c r="B60" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="C60" s="5" t="s">
         <v>232</v>
-      </c>
-      <c r="B60" s="5" t="s">
-        <v>233</v>
-      </c>
-      <c r="C60" s="5" t="s">
-        <v>234</v>
       </c>
       <c r="D60" s="6"/>
       <c r="E60" s="6"/>
@@ -3988,13 +3992,13 @@
     </row>
     <row r="61" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="4" t="s">
+        <v>233</v>
+      </c>
+      <c r="B61" s="5" t="s">
+        <v>234</v>
+      </c>
+      <c r="C61" s="5" t="s">
         <v>235</v>
-      </c>
-      <c r="B61" s="5" t="s">
-        <v>236</v>
-      </c>
-      <c r="C61" s="5" t="s">
-        <v>237</v>
       </c>
       <c r="D61" s="6"/>
       <c r="E61" s="6"/>
@@ -4012,13 +4016,13 @@
     </row>
     <row r="62" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="B62" s="5" t="s">
+        <v>237</v>
+      </c>
+      <c r="C62" s="5" t="s">
         <v>238</v>
-      </c>
-      <c r="B62" s="5" t="s">
-        <v>239</v>
-      </c>
-      <c r="C62" s="5" t="s">
-        <v>240</v>
       </c>
       <c r="D62" s="6"/>
       <c r="E62" s="6"/>
@@ -4036,13 +4040,13 @@
     </row>
     <row r="63" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="B63" s="5" t="s">
+        <v>240</v>
+      </c>
+      <c r="C63" s="5" t="s">
         <v>241</v>
-      </c>
-      <c r="B63" s="5" t="s">
-        <v>242</v>
-      </c>
-      <c r="C63" s="5" t="s">
-        <v>243</v>
       </c>
       <c r="D63" s="6"/>
       <c r="E63" s="6"/>
@@ -4060,13 +4064,13 @@
     </row>
     <row r="64" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="4" t="s">
+        <v>242</v>
+      </c>
+      <c r="B64" s="5" t="s">
+        <v>243</v>
+      </c>
+      <c r="C64" s="5" t="s">
         <v>244</v>
-      </c>
-      <c r="B64" s="5" t="s">
-        <v>245</v>
-      </c>
-      <c r="C64" s="5" t="s">
-        <v>246</v>
       </c>
       <c r="D64" s="6"/>
       <c r="E64" s="6"/>
@@ -4084,13 +4088,13 @@
     </row>
     <row r="65" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="B65" s="5" t="s">
+        <v>246</v>
+      </c>
+      <c r="C65" s="5" t="s">
         <v>247</v>
-      </c>
-      <c r="B65" s="5" t="s">
-        <v>248</v>
-      </c>
-      <c r="C65" s="5" t="s">
-        <v>249</v>
       </c>
       <c r="D65" s="6"/>
       <c r="E65" s="6"/>
@@ -4108,13 +4112,13 @@
     </row>
     <row r="66" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="B66" s="5" t="s">
+        <v>249</v>
+      </c>
+      <c r="C66" s="5" t="s">
         <v>250</v>
-      </c>
-      <c r="B66" s="5" t="s">
-        <v>251</v>
-      </c>
-      <c r="C66" s="5" t="s">
-        <v>252</v>
       </c>
       <c r="D66" s="6"/>
       <c r="E66" s="6"/>
@@ -4132,13 +4136,13 @@
     </row>
     <row r="67" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="B67" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="C67" s="5" t="s">
         <v>253</v>
-      </c>
-      <c r="B67" s="5" t="s">
-        <v>254</v>
-      </c>
-      <c r="C67" s="5" t="s">
-        <v>255</v>
       </c>
       <c r="D67" s="6"/>
       <c r="E67" s="6"/>
@@ -4156,13 +4160,13 @@
     </row>
     <row r="68" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="4" t="s">
+        <v>254</v>
+      </c>
+      <c r="B68" s="5" t="s">
+        <v>255</v>
+      </c>
+      <c r="C68" s="5" t="s">
         <v>256</v>
-      </c>
-      <c r="B68" s="5" t="s">
-        <v>257</v>
-      </c>
-      <c r="C68" s="5" t="s">
-        <v>258</v>
       </c>
       <c r="D68" s="6"/>
       <c r="E68" s="6"/>
@@ -4180,19 +4184,19 @@
     </row>
     <row r="69" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="4" t="s">
+        <v>257</v>
+      </c>
+      <c r="B69" s="5" t="s">
+        <v>258</v>
+      </c>
+      <c r="C69" s="5" t="s">
         <v>259</v>
-      </c>
-      <c r="B69" s="5" t="s">
-        <v>260</v>
-      </c>
-      <c r="C69" s="5" t="s">
-        <v>261</v>
       </c>
       <c r="D69" s="6"/>
       <c r="E69" s="6"/>
       <c r="F69" s="6"/>
       <c r="G69" s="6" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="H69" s="6"/>
       <c r="I69" s="6"/>
@@ -4206,13 +4210,13 @@
     </row>
     <row r="70" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="4" t="s">
+        <v>261</v>
+      </c>
+      <c r="B70" s="5" t="s">
+        <v>262</v>
+      </c>
+      <c r="C70" s="5" t="s">
         <v>263</v>
-      </c>
-      <c r="B70" s="5" t="s">
-        <v>264</v>
-      </c>
-      <c r="C70" s="5" t="s">
-        <v>265</v>
       </c>
       <c r="D70" s="6"/>
       <c r="E70" s="6"/>
@@ -4230,13 +4234,13 @@
     </row>
     <row r="71" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="B71" s="5" t="s">
+        <v>265</v>
+      </c>
+      <c r="C71" s="5" t="s">
         <v>266</v>
-      </c>
-      <c r="B71" s="5" t="s">
-        <v>267</v>
-      </c>
-      <c r="C71" s="5" t="s">
-        <v>268</v>
       </c>
       <c r="D71" s="6"/>
       <c r="E71" s="6"/>
@@ -4254,13 +4258,13 @@
     </row>
     <row r="72" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="4" t="s">
+        <v>267</v>
+      </c>
+      <c r="B72" s="5" t="s">
+        <v>268</v>
+      </c>
+      <c r="C72" s="5" t="s">
         <v>269</v>
-      </c>
-      <c r="B72" s="5" t="s">
-        <v>270</v>
-      </c>
-      <c r="C72" s="5" t="s">
-        <v>271</v>
       </c>
       <c r="D72" s="6"/>
       <c r="E72" s="6"/>
@@ -4278,13 +4282,13 @@
     </row>
     <row r="73" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="4" t="s">
+        <v>270</v>
+      </c>
+      <c r="B73" s="5" t="s">
+        <v>271</v>
+      </c>
+      <c r="C73" s="5" t="s">
         <v>272</v>
-      </c>
-      <c r="B73" s="5" t="s">
-        <v>273</v>
-      </c>
-      <c r="C73" s="5" t="s">
-        <v>274</v>
       </c>
       <c r="D73" s="6"/>
       <c r="E73" s="6"/>
@@ -4302,13 +4306,13 @@
     </row>
     <row r="74" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="4" t="s">
+        <v>273</v>
+      </c>
+      <c r="B74" s="5" t="s">
+        <v>274</v>
+      </c>
+      <c r="C74" s="5" t="s">
         <v>275</v>
-      </c>
-      <c r="B74" s="5" t="s">
-        <v>276</v>
-      </c>
-      <c r="C74" s="5" t="s">
-        <v>277</v>
       </c>
       <c r="D74" s="6"/>
       <c r="E74" s="6"/>
@@ -4326,13 +4330,13 @@
     </row>
     <row r="75" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="4" t="s">
+        <v>276</v>
+      </c>
+      <c r="B75" s="5" t="s">
+        <v>277</v>
+      </c>
+      <c r="C75" s="5" t="s">
         <v>278</v>
-      </c>
-      <c r="B75" s="5" t="s">
-        <v>279</v>
-      </c>
-      <c r="C75" s="5" t="s">
-        <v>280</v>
       </c>
       <c r="D75" s="6"/>
       <c r="E75" s="6"/>
@@ -4350,13 +4354,13 @@
     </row>
     <row r="76" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" s="4" t="s">
+        <v>279</v>
+      </c>
+      <c r="B76" s="5" t="s">
+        <v>280</v>
+      </c>
+      <c r="C76" s="5" t="s">
         <v>281</v>
-      </c>
-      <c r="B76" s="5" t="s">
-        <v>282</v>
-      </c>
-      <c r="C76" s="5" t="s">
-        <v>283</v>
       </c>
       <c r="D76" s="6"/>
       <c r="E76" s="6"/>
@@ -4374,13 +4378,13 @@
     </row>
     <row r="77" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A77" s="4" t="s">
+        <v>282</v>
+      </c>
+      <c r="B77" s="5" t="s">
+        <v>283</v>
+      </c>
+      <c r="C77" s="5" t="s">
         <v>284</v>
-      </c>
-      <c r="B77" s="5" t="s">
-        <v>285</v>
-      </c>
-      <c r="C77" s="5" t="s">
-        <v>286</v>
       </c>
       <c r="D77" s="6"/>
       <c r="E77" s="6"/>
@@ -4398,13 +4402,13 @@
     </row>
     <row r="78" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A78" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="B78" s="5" t="s">
+        <v>286</v>
+      </c>
+      <c r="C78" s="5" t="s">
         <v>287</v>
-      </c>
-      <c r="B78" s="5" t="s">
-        <v>288</v>
-      </c>
-      <c r="C78" s="5" t="s">
-        <v>289</v>
       </c>
       <c r="D78" s="6"/>
       <c r="E78" s="6"/>
@@ -4422,13 +4426,13 @@
     </row>
     <row r="79" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79" s="4" t="s">
+        <v>288</v>
+      </c>
+      <c r="B79" s="5" t="s">
+        <v>289</v>
+      </c>
+      <c r="C79" s="5" t="s">
         <v>290</v>
-      </c>
-      <c r="B79" s="5" t="s">
-        <v>291</v>
-      </c>
-      <c r="C79" s="5" t="s">
-        <v>292</v>
       </c>
       <c r="D79" s="6"/>
       <c r="E79" s="6"/>
@@ -4446,13 +4450,13 @@
     </row>
     <row r="80" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A80" s="4" t="s">
+        <v>291</v>
+      </c>
+      <c r="B80" s="5" t="s">
+        <v>292</v>
+      </c>
+      <c r="C80" s="5" t="s">
         <v>293</v>
-      </c>
-      <c r="B80" s="5" t="s">
-        <v>294</v>
-      </c>
-      <c r="C80" s="5" t="s">
-        <v>295</v>
       </c>
       <c r="D80" s="6"/>
       <c r="E80" s="6"/>
@@ -4470,13 +4474,13 @@
     </row>
     <row r="81" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" s="4" t="s">
+        <v>294</v>
+      </c>
+      <c r="B81" s="5" t="s">
+        <v>295</v>
+      </c>
+      <c r="C81" s="5" t="s">
         <v>296</v>
-      </c>
-      <c r="B81" s="5" t="s">
-        <v>297</v>
-      </c>
-      <c r="C81" s="5" t="s">
-        <v>298</v>
       </c>
       <c r="D81" s="6"/>
       <c r="E81" s="6"/>
@@ -4494,13 +4498,13 @@
     </row>
     <row r="82" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A82" s="4" t="s">
+        <v>297</v>
+      </c>
+      <c r="B82" s="5" t="s">
+        <v>298</v>
+      </c>
+      <c r="C82" s="5" t="s">
         <v>299</v>
-      </c>
-      <c r="B82" s="5" t="s">
-        <v>300</v>
-      </c>
-      <c r="C82" s="5" t="s">
-        <v>301</v>
       </c>
       <c r="D82" s="6"/>
       <c r="E82" s="6"/>
@@ -4518,13 +4522,13 @@
     </row>
     <row r="83" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" s="4" t="s">
+        <v>300</v>
+      </c>
+      <c r="B83" s="5" t="s">
+        <v>301</v>
+      </c>
+      <c r="C83" s="5" t="s">
         <v>302</v>
-      </c>
-      <c r="B83" s="5" t="s">
-        <v>303</v>
-      </c>
-      <c r="C83" s="5" t="s">
-        <v>304</v>
       </c>
       <c r="D83" s="6"/>
       <c r="E83" s="6"/>
@@ -4542,13 +4546,13 @@
     </row>
     <row r="84" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A84" s="4" t="s">
+        <v>303</v>
+      </c>
+      <c r="B84" s="5" t="s">
+        <v>304</v>
+      </c>
+      <c r="C84" s="5" t="s">
         <v>305</v>
-      </c>
-      <c r="B84" s="5" t="s">
-        <v>306</v>
-      </c>
-      <c r="C84" s="5" t="s">
-        <v>307</v>
       </c>
       <c r="D84" s="6"/>
       <c r="E84" s="6"/>
@@ -4566,13 +4570,13 @@
     </row>
     <row r="85" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A85" s="4" t="s">
+        <v>306</v>
+      </c>
+      <c r="B85" s="5" t="s">
+        <v>307</v>
+      </c>
+      <c r="C85" s="5" t="s">
         <v>308</v>
-      </c>
-      <c r="B85" s="5" t="s">
-        <v>309</v>
-      </c>
-      <c r="C85" s="5" t="s">
-        <v>310</v>
       </c>
       <c r="D85" s="6"/>
       <c r="E85" s="6"/>
@@ -4590,13 +4594,13 @@
     </row>
     <row r="86" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A86" s="4" t="s">
+        <v>309</v>
+      </c>
+      <c r="B86" s="5" t="s">
+        <v>310</v>
+      </c>
+      <c r="C86" s="5" t="s">
         <v>311</v>
-      </c>
-      <c r="B86" s="5" t="s">
-        <v>312</v>
-      </c>
-      <c r="C86" s="5" t="s">
-        <v>313</v>
       </c>
       <c r="D86" s="6"/>
       <c r="E86" s="6"/>
@@ -4614,13 +4618,13 @@
     </row>
     <row r="87" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A87" s="4" t="s">
+        <v>312</v>
+      </c>
+      <c r="B87" s="5" t="s">
+        <v>313</v>
+      </c>
+      <c r="C87" s="5" t="s">
         <v>314</v>
-      </c>
-      <c r="B87" s="5" t="s">
-        <v>315</v>
-      </c>
-      <c r="C87" s="5" t="s">
-        <v>316</v>
       </c>
       <c r="D87" s="6"/>
       <c r="E87" s="6"/>
@@ -4638,13 +4642,13 @@
     </row>
     <row r="88" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A88" s="4" t="s">
+        <v>315</v>
+      </c>
+      <c r="B88" s="5" t="s">
+        <v>316</v>
+      </c>
+      <c r="C88" s="5" t="s">
         <v>317</v>
-      </c>
-      <c r="B88" s="5" t="s">
-        <v>318</v>
-      </c>
-      <c r="C88" s="5" t="s">
-        <v>319</v>
       </c>
       <c r="D88" s="6"/>
       <c r="E88" s="6"/>
@@ -4662,13 +4666,13 @@
     </row>
     <row r="89" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A89" s="4" t="s">
+        <v>318</v>
+      </c>
+      <c r="B89" s="5" t="s">
+        <v>319</v>
+      </c>
+      <c r="C89" s="5" t="s">
         <v>320</v>
-      </c>
-      <c r="B89" s="5" t="s">
-        <v>321</v>
-      </c>
-      <c r="C89" s="5" t="s">
-        <v>322</v>
       </c>
       <c r="D89" s="6"/>
       <c r="E89" s="6"/>
@@ -4686,13 +4690,13 @@
     </row>
     <row r="90" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A90" s="4" t="s">
+        <v>321</v>
+      </c>
+      <c r="B90" s="5" t="s">
+        <v>322</v>
+      </c>
+      <c r="C90" s="5" t="s">
         <v>323</v>
-      </c>
-      <c r="B90" s="5" t="s">
-        <v>324</v>
-      </c>
-      <c r="C90" s="5" t="s">
-        <v>325</v>
       </c>
       <c r="D90" s="6"/>
       <c r="E90" s="6"/>
@@ -4710,13 +4714,13 @@
     </row>
     <row r="91" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A91" s="4" t="s">
+        <v>324</v>
+      </c>
+      <c r="B91" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="C91" s="5" t="s">
         <v>326</v>
-      </c>
-      <c r="B91" s="5" t="s">
-        <v>327</v>
-      </c>
-      <c r="C91" s="5" t="s">
-        <v>328</v>
       </c>
       <c r="D91" s="6"/>
       <c r="E91" s="6"/>
@@ -4734,19 +4738,19 @@
     </row>
     <row r="92" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A92" s="4" t="s">
+        <v>327</v>
+      </c>
+      <c r="B92" s="5" t="s">
+        <v>328</v>
+      </c>
+      <c r="C92" s="5" t="s">
         <v>329</v>
-      </c>
-      <c r="B92" s="5" t="s">
-        <v>330</v>
-      </c>
-      <c r="C92" s="5" t="s">
-        <v>331</v>
       </c>
       <c r="D92" s="6"/>
       <c r="E92" s="6"/>
       <c r="F92" s="6"/>
       <c r="G92" s="6" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="H92" s="6"/>
       <c r="I92" s="6"/>
@@ -4760,13 +4764,13 @@
     </row>
     <row r="93" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A93" s="4" t="s">
+        <v>331</v>
+      </c>
+      <c r="B93" s="5" t="s">
+        <v>332</v>
+      </c>
+      <c r="C93" s="5" t="s">
         <v>333</v>
-      </c>
-      <c r="B93" s="5" t="s">
-        <v>334</v>
-      </c>
-      <c r="C93" s="5" t="s">
-        <v>335</v>
       </c>
       <c r="D93" s="6"/>
       <c r="E93" s="6"/>
@@ -4784,13 +4788,13 @@
     </row>
     <row r="94" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A94" s="4" t="s">
+        <v>334</v>
+      </c>
+      <c r="B94" s="5" t="s">
+        <v>335</v>
+      </c>
+      <c r="C94" s="5" t="s">
         <v>336</v>
-      </c>
-      <c r="B94" s="5" t="s">
-        <v>337</v>
-      </c>
-      <c r="C94" s="5" t="s">
-        <v>338</v>
       </c>
       <c r="D94" s="6"/>
       <c r="E94" s="6"/>
@@ -4808,13 +4812,13 @@
     </row>
     <row r="95" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A95" s="4" t="s">
+        <v>337</v>
+      </c>
+      <c r="B95" s="5" t="s">
+        <v>338</v>
+      </c>
+      <c r="C95" s="5" t="s">
         <v>339</v>
-      </c>
-      <c r="B95" s="5" t="s">
-        <v>340</v>
-      </c>
-      <c r="C95" s="5" t="s">
-        <v>341</v>
       </c>
       <c r="D95" s="6"/>
       <c r="E95" s="6"/>
@@ -4832,13 +4836,13 @@
     </row>
     <row r="96" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A96" s="4" t="s">
+        <v>340</v>
+      </c>
+      <c r="B96" s="5" t="s">
+        <v>341</v>
+      </c>
+      <c r="C96" s="5" t="s">
         <v>342</v>
-      </c>
-      <c r="B96" s="5" t="s">
-        <v>343</v>
-      </c>
-      <c r="C96" s="5" t="s">
-        <v>344</v>
       </c>
       <c r="D96" s="6"/>
       <c r="E96" s="6"/>
@@ -4856,13 +4860,13 @@
     </row>
     <row r="97" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A97" s="4" t="s">
+        <v>343</v>
+      </c>
+      <c r="B97" s="5" t="s">
+        <v>344</v>
+      </c>
+      <c r="C97" s="5" t="s">
         <v>345</v>
-      </c>
-      <c r="B97" s="5" t="s">
-        <v>346</v>
-      </c>
-      <c r="C97" s="5" t="s">
-        <v>347</v>
       </c>
       <c r="D97" s="6"/>
       <c r="E97" s="6"/>
@@ -4880,13 +4884,13 @@
     </row>
     <row r="98" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A98" s="4" t="s">
+        <v>346</v>
+      </c>
+      <c r="B98" s="5" t="s">
+        <v>347</v>
+      </c>
+      <c r="C98" s="5" t="s">
         <v>348</v>
-      </c>
-      <c r="B98" s="5" t="s">
-        <v>349</v>
-      </c>
-      <c r="C98" s="5" t="s">
-        <v>350</v>
       </c>
       <c r="D98" s="6"/>
       <c r="E98" s="6"/>
@@ -4904,13 +4908,13 @@
     </row>
     <row r="99" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A99" s="4" t="s">
+        <v>349</v>
+      </c>
+      <c r="B99" s="5" t="s">
+        <v>350</v>
+      </c>
+      <c r="C99" s="5" t="s">
         <v>351</v>
-      </c>
-      <c r="B99" s="5" t="s">
-        <v>352</v>
-      </c>
-      <c r="C99" s="5" t="s">
-        <v>353</v>
       </c>
       <c r="D99" s="6"/>
       <c r="E99" s="6"/>
@@ -4928,13 +4932,13 @@
     </row>
     <row r="100" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A100" s="4" t="s">
+        <v>352</v>
+      </c>
+      <c r="B100" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="C100" s="5" t="s">
         <v>354</v>
-      </c>
-      <c r="B100" s="5" t="s">
-        <v>355</v>
-      </c>
-      <c r="C100" s="5" t="s">
-        <v>356</v>
       </c>
       <c r="D100" s="6"/>
       <c r="E100" s="6"/>
@@ -4952,13 +4956,13 @@
     </row>
     <row r="101" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A101" s="4" t="s">
+        <v>355</v>
+      </c>
+      <c r="B101" s="5" t="s">
+        <v>356</v>
+      </c>
+      <c r="C101" s="5" t="s">
         <v>357</v>
-      </c>
-      <c r="B101" s="5" t="s">
-        <v>358</v>
-      </c>
-      <c r="C101" s="5" t="s">
-        <v>359</v>
       </c>
       <c r="D101" s="6"/>
       <c r="E101" s="6"/>
@@ -4974,13 +4978,13 @@
     </row>
     <row r="102" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A102" s="4" t="s">
+        <v>358</v>
+      </c>
+      <c r="B102" s="5" t="s">
+        <v>359</v>
+      </c>
+      <c r="C102" s="5" t="s">
         <v>360</v>
-      </c>
-      <c r="B102" s="5" t="s">
-        <v>361</v>
-      </c>
-      <c r="C102" s="5" t="s">
-        <v>362</v>
       </c>
       <c r="D102" s="6"/>
       <c r="E102" s="6"/>
@@ -4996,13 +5000,13 @@
     </row>
     <row r="103" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A103" s="4" t="s">
+        <v>361</v>
+      </c>
+      <c r="B103" s="5" t="s">
+        <v>362</v>
+      </c>
+      <c r="C103" s="5" t="s">
         <v>363</v>
-      </c>
-      <c r="B103" s="5" t="s">
-        <v>364</v>
-      </c>
-      <c r="C103" s="5" t="s">
-        <v>365</v>
       </c>
       <c r="D103" s="6"/>
       <c r="E103" s="6"/>
@@ -5018,13 +5022,13 @@
     </row>
     <row r="104" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A104" s="4" t="s">
+        <v>364</v>
+      </c>
+      <c r="B104" s="5" t="s">
+        <v>365</v>
+      </c>
+      <c r="C104" s="5" t="s">
         <v>366</v>
-      </c>
-      <c r="B104" s="5" t="s">
-        <v>367</v>
-      </c>
-      <c r="C104" s="5" t="s">
-        <v>368</v>
       </c>
       <c r="D104" s="6"/>
       <c r="E104" s="6"/>
@@ -5040,13 +5044,13 @@
     </row>
     <row r="105" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A105" s="4" t="s">
+        <v>367</v>
+      </c>
+      <c r="B105" s="5" t="s">
+        <v>368</v>
+      </c>
+      <c r="C105" s="5" t="s">
         <v>369</v>
-      </c>
-      <c r="B105" s="5" t="s">
-        <v>370</v>
-      </c>
-      <c r="C105" s="5" t="s">
-        <v>371</v>
       </c>
       <c r="D105" s="6"/>
       <c r="E105" s="6"/>
@@ -5062,13 +5066,13 @@
     </row>
     <row r="106" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A106" s="4" t="s">
+        <v>370</v>
+      </c>
+      <c r="B106" s="5" t="s">
+        <v>371</v>
+      </c>
+      <c r="C106" s="5" t="s">
         <v>372</v>
-      </c>
-      <c r="B106" s="5" t="s">
-        <v>373</v>
-      </c>
-      <c r="C106" s="5" t="s">
-        <v>374</v>
       </c>
       <c r="D106" s="6"/>
       <c r="E106" s="6"/>
@@ -5084,13 +5088,13 @@
     </row>
     <row r="107" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A107" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="B107" s="5" t="s">
+        <v>374</v>
+      </c>
+      <c r="C107" s="5" t="s">
         <v>375</v>
-      </c>
-      <c r="B107" s="5" t="s">
-        <v>376</v>
-      </c>
-      <c r="C107" s="5" t="s">
-        <v>377</v>
       </c>
       <c r="D107" s="6"/>
       <c r="E107" s="6"/>
@@ -5106,13 +5110,13 @@
     </row>
     <row r="108" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A108" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="B108" s="5" t="s">
+        <v>377</v>
+      </c>
+      <c r="C108" s="5" t="s">
         <v>378</v>
-      </c>
-      <c r="B108" s="5" t="s">
-        <v>379</v>
-      </c>
-      <c r="C108" s="5" t="s">
-        <v>380</v>
       </c>
       <c r="D108" s="6"/>
       <c r="E108" s="6"/>
@@ -5128,13 +5132,13 @@
     </row>
     <row r="109" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A109" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="B109" s="5" t="s">
+        <v>380</v>
+      </c>
+      <c r="C109" s="5" t="s">
         <v>381</v>
-      </c>
-      <c r="B109" s="5" t="s">
-        <v>382</v>
-      </c>
-      <c r="C109" s="5" t="s">
-        <v>383</v>
       </c>
       <c r="D109" s="6"/>
       <c r="E109" s="6"/>
@@ -5150,13 +5154,13 @@
     </row>
     <row r="110" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A110" s="4" t="s">
+        <v>382</v>
+      </c>
+      <c r="B110" s="5" t="s">
+        <v>383</v>
+      </c>
+      <c r="C110" s="5" t="s">
         <v>384</v>
-      </c>
-      <c r="B110" s="5" t="s">
-        <v>385</v>
-      </c>
-      <c r="C110" s="5" t="s">
-        <v>386</v>
       </c>
       <c r="D110" s="6"/>
       <c r="E110" s="6"/>
@@ -5172,13 +5176,13 @@
     </row>
     <row r="111" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A111" s="4" t="s">
+        <v>385</v>
+      </c>
+      <c r="B111" s="5" t="s">
+        <v>386</v>
+      </c>
+      <c r="C111" s="5" t="s">
         <v>387</v>
-      </c>
-      <c r="B111" s="5" t="s">
-        <v>388</v>
-      </c>
-      <c r="C111" s="5" t="s">
-        <v>389</v>
       </c>
       <c r="D111" s="6"/>
       <c r="E111" s="6"/>
@@ -5194,13 +5198,13 @@
     </row>
     <row r="112" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A112" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="B112" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="C112" s="5" t="s">
         <v>390</v>
-      </c>
-      <c r="B112" s="5" t="s">
-        <v>391</v>
-      </c>
-      <c r="C112" s="5" t="s">
-        <v>392</v>
       </c>
       <c r="D112" s="6"/>
       <c r="E112" s="6"/>
@@ -5216,13 +5220,13 @@
     </row>
     <row r="113" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A113" s="4" t="s">
+        <v>391</v>
+      </c>
+      <c r="B113" s="5" t="s">
+        <v>392</v>
+      </c>
+      <c r="C113" s="5" t="s">
         <v>393</v>
-      </c>
-      <c r="B113" s="5" t="s">
-        <v>394</v>
-      </c>
-      <c r="C113" s="5" t="s">
-        <v>395</v>
       </c>
       <c r="D113" s="6"/>
       <c r="E113" s="6"/>
@@ -5238,13 +5242,13 @@
     </row>
     <row r="114" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A114" s="4" t="s">
+        <v>394</v>
+      </c>
+      <c r="B114" s="5" t="s">
+        <v>395</v>
+      </c>
+      <c r="C114" s="5" t="s">
         <v>396</v>
-      </c>
-      <c r="B114" s="5" t="s">
-        <v>397</v>
-      </c>
-      <c r="C114" s="5" t="s">
-        <v>398</v>
       </c>
       <c r="D114" s="6"/>
       <c r="E114" s="6"/>
@@ -5260,13 +5264,13 @@
     </row>
     <row r="115" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A115" s="4" t="s">
+        <v>397</v>
+      </c>
+      <c r="B115" s="5" t="s">
+        <v>398</v>
+      </c>
+      <c r="C115" s="5" t="s">
         <v>399</v>
-      </c>
-      <c r="B115" s="5" t="s">
-        <v>400</v>
-      </c>
-      <c r="C115" s="5" t="s">
-        <v>401</v>
       </c>
       <c r="D115" s="6"/>
       <c r="E115" s="6"/>
@@ -5282,13 +5286,13 @@
     </row>
     <row r="116" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A116" s="4" t="s">
+        <v>400</v>
+      </c>
+      <c r="B116" s="5" t="s">
+        <v>401</v>
+      </c>
+      <c r="C116" s="5" t="s">
         <v>402</v>
-      </c>
-      <c r="B116" s="5" t="s">
-        <v>403</v>
-      </c>
-      <c r="C116" s="5" t="s">
-        <v>404</v>
       </c>
       <c r="D116" s="6"/>
       <c r="E116" s="6"/>
@@ -5304,13 +5308,13 @@
     </row>
     <row r="117" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A117" s="4" t="s">
+        <v>403</v>
+      </c>
+      <c r="B117" s="5" t="s">
+        <v>404</v>
+      </c>
+      <c r="C117" s="5" t="s">
         <v>405</v>
-      </c>
-      <c r="B117" s="5" t="s">
-        <v>406</v>
-      </c>
-      <c r="C117" s="5" t="s">
-        <v>407</v>
       </c>
       <c r="D117" s="6"/>
       <c r="E117" s="6"/>
@@ -5326,13 +5330,13 @@
     </row>
     <row r="118" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A118" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="B118" s="5" t="s">
+        <v>407</v>
+      </c>
+      <c r="C118" s="5" t="s">
         <v>408</v>
-      </c>
-      <c r="B118" s="5" t="s">
-        <v>409</v>
-      </c>
-      <c r="C118" s="5" t="s">
-        <v>410</v>
       </c>
       <c r="D118" s="6"/>
       <c r="E118" s="6"/>
@@ -5348,13 +5352,13 @@
     </row>
     <row r="119" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A119" s="4" t="s">
+        <v>409</v>
+      </c>
+      <c r="B119" s="5" t="s">
+        <v>410</v>
+      </c>
+      <c r="C119" s="5" t="s">
         <v>411</v>
-      </c>
-      <c r="B119" s="5" t="s">
-        <v>412</v>
-      </c>
-      <c r="C119" s="5" t="s">
-        <v>413</v>
       </c>
       <c r="D119" s="6"/>
       <c r="E119" s="6"/>
@@ -5370,13 +5374,13 @@
     </row>
     <row r="120" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A120" s="4" t="s">
+        <v>412</v>
+      </c>
+      <c r="B120" s="5" t="s">
+        <v>413</v>
+      </c>
+      <c r="C120" s="5" t="s">
         <v>414</v>
-      </c>
-      <c r="B120" s="5" t="s">
-        <v>415</v>
-      </c>
-      <c r="C120" s="5" t="s">
-        <v>416</v>
       </c>
       <c r="D120" s="6"/>
       <c r="E120" s="6"/>
@@ -5392,13 +5396,13 @@
     </row>
     <row r="121" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A121" s="4" t="s">
+        <v>415</v>
+      </c>
+      <c r="B121" s="5" t="s">
+        <v>416</v>
+      </c>
+      <c r="C121" s="5" t="s">
         <v>417</v>
-      </c>
-      <c r="B121" s="5" t="s">
-        <v>418</v>
-      </c>
-      <c r="C121" s="5" t="s">
-        <v>419</v>
       </c>
       <c r="D121" s="6"/>
       <c r="E121" s="6"/>
@@ -5414,13 +5418,13 @@
     </row>
     <row r="122" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A122" s="4" t="s">
+        <v>418</v>
+      </c>
+      <c r="B122" s="5" t="s">
+        <v>419</v>
+      </c>
+      <c r="C122" s="5" t="s">
         <v>420</v>
-      </c>
-      <c r="B122" s="5" t="s">
-        <v>421</v>
-      </c>
-      <c r="C122" s="5" t="s">
-        <v>422</v>
       </c>
       <c r="D122" s="6"/>
       <c r="E122" s="6"/>
@@ -5436,13 +5440,13 @@
     </row>
     <row r="123" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A123" s="4" t="s">
+        <v>421</v>
+      </c>
+      <c r="B123" s="5" t="s">
+        <v>422</v>
+      </c>
+      <c r="C123" s="5" t="s">
         <v>423</v>
-      </c>
-      <c r="B123" s="5" t="s">
-        <v>424</v>
-      </c>
-      <c r="C123" s="5" t="s">
-        <v>425</v>
       </c>
       <c r="D123" s="6"/>
       <c r="E123" s="6"/>
@@ -5458,13 +5462,13 @@
     </row>
     <row r="124" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A124" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="B124" s="5" t="s">
+        <v>425</v>
+      </c>
+      <c r="C124" s="5" t="s">
         <v>426</v>
-      </c>
-      <c r="B124" s="5" t="s">
-        <v>427</v>
-      </c>
-      <c r="C124" s="5" t="s">
-        <v>428</v>
       </c>
       <c r="D124" s="6"/>
       <c r="E124" s="6"/>
@@ -5480,13 +5484,13 @@
     </row>
     <row r="125" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A125" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="B125" s="5" t="s">
+        <v>428</v>
+      </c>
+      <c r="C125" s="5" t="s">
         <v>429</v>
-      </c>
-      <c r="B125" s="5" t="s">
-        <v>430</v>
-      </c>
-      <c r="C125" s="5" t="s">
-        <v>431</v>
       </c>
       <c r="D125" s="6"/>
       <c r="E125" s="6"/>
@@ -5502,13 +5506,13 @@
     </row>
     <row r="126" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A126" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="B126" s="5" t="s">
+        <v>431</v>
+      </c>
+      <c r="C126" s="5" t="s">
         <v>432</v>
-      </c>
-      <c r="B126" s="5" t="s">
-        <v>433</v>
-      </c>
-      <c r="C126" s="5" t="s">
-        <v>434</v>
       </c>
       <c r="D126" s="6"/>
       <c r="E126" s="6"/>
@@ -5524,13 +5528,13 @@
     </row>
     <row r="127" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A127" s="4" t="s">
+        <v>433</v>
+      </c>
+      <c r="B127" s="5" t="s">
+        <v>434</v>
+      </c>
+      <c r="C127" s="5" t="s">
         <v>435</v>
-      </c>
-      <c r="B127" s="5" t="s">
-        <v>436</v>
-      </c>
-      <c r="C127" s="5" t="s">
-        <v>437</v>
       </c>
       <c r="D127" s="6"/>
       <c r="E127" s="6"/>
@@ -5546,13 +5550,13 @@
     </row>
     <row r="128" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A128" s="4" t="s">
+        <v>436</v>
+      </c>
+      <c r="B128" s="5" t="s">
+        <v>437</v>
+      </c>
+      <c r="C128" s="5" t="s">
         <v>438</v>
-      </c>
-      <c r="B128" s="5" t="s">
-        <v>439</v>
-      </c>
-      <c r="C128" s="5" t="s">
-        <v>440</v>
       </c>
       <c r="D128" s="6"/>
       <c r="E128" s="6"/>
@@ -5568,13 +5572,13 @@
     </row>
     <row r="129" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A129" s="4" t="s">
+        <v>439</v>
+      </c>
+      <c r="B129" s="5" t="s">
+        <v>440</v>
+      </c>
+      <c r="C129" s="5" t="s">
         <v>441</v>
-      </c>
-      <c r="B129" s="5" t="s">
-        <v>442</v>
-      </c>
-      <c r="C129" s="5" t="s">
-        <v>443</v>
       </c>
       <c r="D129" s="6"/>
       <c r="E129" s="6"/>
@@ -5590,13 +5594,13 @@
     </row>
     <row r="130" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A130" s="4" t="s">
+        <v>442</v>
+      </c>
+      <c r="B130" s="5" t="s">
+        <v>443</v>
+      </c>
+      <c r="C130" s="5" t="s">
         <v>444</v>
-      </c>
-      <c r="B130" s="5" t="s">
-        <v>445</v>
-      </c>
-      <c r="C130" s="5" t="s">
-        <v>446</v>
       </c>
       <c r="D130" s="6"/>
       <c r="E130" s="6"/>
@@ -5612,13 +5616,13 @@
     </row>
     <row r="131" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A131" s="4" t="s">
+        <v>445</v>
+      </c>
+      <c r="B131" s="5" t="s">
+        <v>446</v>
+      </c>
+      <c r="C131" s="5" t="s">
         <v>447</v>
-      </c>
-      <c r="B131" s="5" t="s">
-        <v>448</v>
-      </c>
-      <c r="C131" s="5" t="s">
-        <v>449</v>
       </c>
       <c r="D131" s="6"/>
       <c r="E131" s="6"/>
@@ -5634,13 +5638,13 @@
     </row>
     <row r="132" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A132" s="4" t="s">
+        <v>448</v>
+      </c>
+      <c r="B132" s="5" t="s">
+        <v>449</v>
+      </c>
+      <c r="C132" s="5" t="s">
         <v>450</v>
-      </c>
-      <c r="B132" s="5" t="s">
-        <v>451</v>
-      </c>
-      <c r="C132" s="5" t="s">
-        <v>452</v>
       </c>
       <c r="D132" s="6"/>
       <c r="E132" s="6"/>
@@ -5656,13 +5660,13 @@
     </row>
     <row r="133" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A133" s="4" t="s">
+        <v>451</v>
+      </c>
+      <c r="B133" s="5" t="s">
+        <v>452</v>
+      </c>
+      <c r="C133" s="5" t="s">
         <v>453</v>
-      </c>
-      <c r="B133" s="5" t="s">
-        <v>454</v>
-      </c>
-      <c r="C133" s="5" t="s">
-        <v>455</v>
       </c>
       <c r="D133" s="6"/>
       <c r="E133" s="6"/>
@@ -5678,13 +5682,13 @@
     </row>
     <row r="134" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A134" s="4" t="s">
+        <v>454</v>
+      </c>
+      <c r="B134" s="5" t="s">
+        <v>455</v>
+      </c>
+      <c r="C134" s="5" t="s">
         <v>456</v>
-      </c>
-      <c r="B134" s="5" t="s">
-        <v>457</v>
-      </c>
-      <c r="C134" s="5" t="s">
-        <v>458</v>
       </c>
       <c r="D134" s="6"/>
       <c r="E134" s="6"/>
@@ -5700,13 +5704,13 @@
     </row>
     <row r="135" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A135" s="4" t="s">
+        <v>457</v>
+      </c>
+      <c r="B135" s="5" t="s">
+        <v>458</v>
+      </c>
+      <c r="C135" s="5" t="s">
         <v>459</v>
-      </c>
-      <c r="B135" s="5" t="s">
-        <v>460</v>
-      </c>
-      <c r="C135" s="5" t="s">
-        <v>461</v>
       </c>
       <c r="D135" s="6"/>
       <c r="E135" s="6"/>
@@ -5722,13 +5726,13 @@
     </row>
     <row r="136" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A136" s="4" t="s">
+        <v>460</v>
+      </c>
+      <c r="B136" s="5" t="s">
+        <v>461</v>
+      </c>
+      <c r="C136" s="5" t="s">
         <v>462</v>
-      </c>
-      <c r="B136" s="5" t="s">
-        <v>463</v>
-      </c>
-      <c r="C136" s="5" t="s">
-        <v>464</v>
       </c>
       <c r="D136" s="6"/>
       <c r="E136" s="6"/>
@@ -5744,13 +5748,13 @@
     </row>
     <row r="137" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A137" s="4" t="s">
+        <v>463</v>
+      </c>
+      <c r="B137" s="5" t="s">
+        <v>464</v>
+      </c>
+      <c r="C137" s="5" t="s">
         <v>465</v>
-      </c>
-      <c r="B137" s="5" t="s">
-        <v>466</v>
-      </c>
-      <c r="C137" s="5" t="s">
-        <v>467</v>
       </c>
       <c r="D137" s="6"/>
       <c r="E137" s="6"/>
@@ -5766,13 +5770,13 @@
     </row>
     <row r="138" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A138" s="4" t="s">
+        <v>466</v>
+      </c>
+      <c r="B138" s="5" t="s">
+        <v>467</v>
+      </c>
+      <c r="C138" s="5" t="s">
         <v>468</v>
-      </c>
-      <c r="B138" s="5" t="s">
-        <v>469</v>
-      </c>
-      <c r="C138" s="5" t="s">
-        <v>470</v>
       </c>
       <c r="D138" s="6"/>
       <c r="E138" s="6"/>
@@ -5788,13 +5792,13 @@
     </row>
     <row r="139" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A139" s="4" t="s">
+        <v>469</v>
+      </c>
+      <c r="B139" s="5" t="s">
+        <v>470</v>
+      </c>
+      <c r="C139" s="5" t="s">
         <v>471</v>
-      </c>
-      <c r="B139" s="5" t="s">
-        <v>472</v>
-      </c>
-      <c r="C139" s="5" t="s">
-        <v>473</v>
       </c>
       <c r="D139" s="6"/>
       <c r="E139" s="6"/>
@@ -5810,13 +5814,13 @@
     </row>
     <row r="140" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A140" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="B140" s="5" t="s">
+        <v>473</v>
+      </c>
+      <c r="C140" s="5" t="s">
         <v>474</v>
-      </c>
-      <c r="B140" s="5" t="s">
-        <v>475</v>
-      </c>
-      <c r="C140" s="5" t="s">
-        <v>476</v>
       </c>
       <c r="D140" s="6"/>
       <c r="E140" s="6"/>
@@ -5832,13 +5836,13 @@
     </row>
     <row r="141" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A141" s="4" t="s">
+        <v>475</v>
+      </c>
+      <c r="B141" s="5" t="s">
+        <v>476</v>
+      </c>
+      <c r="C141" s="5" t="s">
         <v>477</v>
-      </c>
-      <c r="B141" s="5" t="s">
-        <v>478</v>
-      </c>
-      <c r="C141" s="5" t="s">
-        <v>479</v>
       </c>
       <c r="D141" s="6"/>
       <c r="E141" s="6"/>
@@ -5854,13 +5858,13 @@
     </row>
     <row r="142" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A142" s="4" t="s">
+        <v>478</v>
+      </c>
+      <c r="B142" s="5" t="s">
+        <v>479</v>
+      </c>
+      <c r="C142" s="5" t="s">
         <v>480</v>
-      </c>
-      <c r="B142" s="5" t="s">
-        <v>481</v>
-      </c>
-      <c r="C142" s="5" t="s">
-        <v>482</v>
       </c>
       <c r="D142" s="6"/>
       <c r="E142" s="6"/>
@@ -5876,13 +5880,13 @@
     </row>
     <row r="143" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A143" s="4" t="s">
+        <v>481</v>
+      </c>
+      <c r="B143" s="5" t="s">
+        <v>482</v>
+      </c>
+      <c r="C143" s="5" t="s">
         <v>483</v>
-      </c>
-      <c r="B143" s="5" t="s">
-        <v>484</v>
-      </c>
-      <c r="C143" s="5" t="s">
-        <v>485</v>
       </c>
       <c r="D143" s="6"/>
       <c r="E143" s="6"/>
@@ -5898,13 +5902,13 @@
     </row>
     <row r="144" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A144" s="4" t="s">
+        <v>484</v>
+      </c>
+      <c r="B144" s="5" t="s">
+        <v>485</v>
+      </c>
+      <c r="C144" s="5" t="s">
         <v>486</v>
-      </c>
-      <c r="B144" s="5" t="s">
-        <v>487</v>
-      </c>
-      <c r="C144" s="5" t="s">
-        <v>488</v>
       </c>
       <c r="D144" s="6"/>
       <c r="E144" s="6"/>
@@ -5920,13 +5924,13 @@
     </row>
     <row r="145" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A145" s="4" t="s">
+        <v>487</v>
+      </c>
+      <c r="B145" s="5" t="s">
+        <v>488</v>
+      </c>
+      <c r="C145" s="5" t="s">
         <v>489</v>
-      </c>
-      <c r="B145" s="5" t="s">
-        <v>490</v>
-      </c>
-      <c r="C145" s="5" t="s">
-        <v>491</v>
       </c>
       <c r="D145" s="6"/>
       <c r="E145" s="6"/>
@@ -5942,13 +5946,13 @@
     </row>
     <row r="146" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A146" s="4" t="s">
+        <v>490</v>
+      </c>
+      <c r="B146" s="5" t="s">
+        <v>491</v>
+      </c>
+      <c r="C146" s="5" t="s">
         <v>492</v>
-      </c>
-      <c r="B146" s="5" t="s">
-        <v>493</v>
-      </c>
-      <c r="C146" s="5" t="s">
-        <v>494</v>
       </c>
       <c r="D146" s="6"/>
       <c r="E146" s="6"/>
@@ -5964,13 +5968,13 @@
     </row>
     <row r="147" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A147" s="4" t="s">
+        <v>493</v>
+      </c>
+      <c r="B147" s="5" t="s">
+        <v>494</v>
+      </c>
+      <c r="C147" s="5" t="s">
         <v>495</v>
-      </c>
-      <c r="B147" s="5" t="s">
-        <v>496</v>
-      </c>
-      <c r="C147" s="5" t="s">
-        <v>497</v>
       </c>
       <c r="D147" s="6"/>
       <c r="E147" s="6"/>
@@ -5986,13 +5990,13 @@
     </row>
     <row r="148" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A148" s="4" t="s">
+        <v>496</v>
+      </c>
+      <c r="B148" s="5" t="s">
+        <v>497</v>
+      </c>
+      <c r="C148" s="5" t="s">
         <v>498</v>
-      </c>
-      <c r="B148" s="5" t="s">
-        <v>499</v>
-      </c>
-      <c r="C148" s="5" t="s">
-        <v>500</v>
       </c>
       <c r="D148" s="6"/>
       <c r="E148" s="6"/>
@@ -6008,13 +6012,13 @@
     </row>
     <row r="149" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A149" s="4" t="s">
+        <v>499</v>
+      </c>
+      <c r="B149" s="5" t="s">
+        <v>500</v>
+      </c>
+      <c r="C149" s="5" t="s">
         <v>501</v>
-      </c>
-      <c r="B149" s="5" t="s">
-        <v>502</v>
-      </c>
-      <c r="C149" s="5" t="s">
-        <v>503</v>
       </c>
       <c r="D149" s="6"/>
       <c r="E149" s="6"/>
@@ -6030,13 +6034,13 @@
     </row>
     <row r="150" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A150" s="4" t="s">
+        <v>502</v>
+      </c>
+      <c r="B150" s="5" t="s">
+        <v>503</v>
+      </c>
+      <c r="C150" s="5" t="s">
         <v>504</v>
-      </c>
-      <c r="B150" s="5" t="s">
-        <v>505</v>
-      </c>
-      <c r="C150" s="5" t="s">
-        <v>506</v>
       </c>
       <c r="D150" s="6"/>
       <c r="E150" s="6"/>
@@ -6052,13 +6056,13 @@
     </row>
     <row r="151" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A151" s="4" t="s">
+        <v>505</v>
+      </c>
+      <c r="B151" s="5" t="s">
+        <v>506</v>
+      </c>
+      <c r="C151" s="5" t="s">
         <v>507</v>
-      </c>
-      <c r="B151" s="5" t="s">
-        <v>508</v>
-      </c>
-      <c r="C151" s="5" t="s">
-        <v>509</v>
       </c>
       <c r="D151" s="6"/>
       <c r="E151" s="6"/>
@@ -6074,19 +6078,19 @@
     </row>
     <row r="152" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A152" s="4" t="s">
+        <v>508</v>
+      </c>
+      <c r="B152" s="5" t="s">
+        <v>509</v>
+      </c>
+      <c r="C152" s="5" t="s">
         <v>510</v>
-      </c>
-      <c r="B152" s="5" t="s">
-        <v>511</v>
-      </c>
-      <c r="C152" s="5" t="s">
-        <v>512</v>
       </c>
       <c r="D152" s="6"/>
       <c r="E152" s="6"/>
       <c r="F152" s="6"/>
       <c r="G152" s="6" t="s">
-        <v>513</v>
+        <v>511</v>
       </c>
       <c r="H152" s="6"/>
       <c r="I152" s="6"/>
@@ -6098,13 +6102,13 @@
     </row>
     <row r="153" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A153" s="4" t="s">
+        <v>512</v>
+      </c>
+      <c r="B153" s="5" t="s">
+        <v>513</v>
+      </c>
+      <c r="C153" s="5" t="s">
         <v>514</v>
-      </c>
-      <c r="B153" s="5" t="s">
-        <v>515</v>
-      </c>
-      <c r="C153" s="5" t="s">
-        <v>516</v>
       </c>
       <c r="D153" s="6"/>
       <c r="E153" s="6"/>
@@ -6120,13 +6124,13 @@
     </row>
     <row r="154" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A154" s="4" t="s">
+        <v>515</v>
+      </c>
+      <c r="B154" s="5" t="s">
+        <v>516</v>
+      </c>
+      <c r="C154" s="5" t="s">
         <v>517</v>
-      </c>
-      <c r="B154" s="5" t="s">
-        <v>518</v>
-      </c>
-      <c r="C154" s="5" t="s">
-        <v>519</v>
       </c>
       <c r="D154" s="6"/>
       <c r="E154" s="6"/>
@@ -6142,13 +6146,13 @@
     </row>
     <row r="155" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A155" s="4" t="s">
+        <v>518</v>
+      </c>
+      <c r="B155" s="5" t="s">
+        <v>519</v>
+      </c>
+      <c r="C155" s="5" t="s">
         <v>520</v>
-      </c>
-      <c r="B155" s="5" t="s">
-        <v>521</v>
-      </c>
-      <c r="C155" s="5" t="s">
-        <v>522</v>
       </c>
       <c r="D155" s="6"/>
       <c r="E155" s="6"/>
@@ -6164,13 +6168,13 @@
     </row>
     <row r="156" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A156" s="4" t="s">
+        <v>521</v>
+      </c>
+      <c r="B156" s="5" t="s">
+        <v>522</v>
+      </c>
+      <c r="C156" s="5" t="s">
         <v>523</v>
-      </c>
-      <c r="B156" s="5" t="s">
-        <v>524</v>
-      </c>
-      <c r="C156" s="5" t="s">
-        <v>525</v>
       </c>
       <c r="D156" s="6"/>
       <c r="E156" s="6"/>
@@ -6186,13 +6190,13 @@
     </row>
     <row r="157" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A157" s="4" t="s">
+        <v>524</v>
+      </c>
+      <c r="B157" s="5" t="s">
+        <v>525</v>
+      </c>
+      <c r="C157" s="5" t="s">
         <v>526</v>
-      </c>
-      <c r="B157" s="5" t="s">
-        <v>527</v>
-      </c>
-      <c r="C157" s="5" t="s">
-        <v>528</v>
       </c>
       <c r="D157" s="6"/>
       <c r="E157" s="6"/>
@@ -6208,13 +6212,13 @@
     </row>
     <row r="158" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A158" s="4" t="s">
+        <v>527</v>
+      </c>
+      <c r="B158" s="5" t="s">
+        <v>528</v>
+      </c>
+      <c r="C158" s="5" t="s">
         <v>529</v>
-      </c>
-      <c r="B158" s="5" t="s">
-        <v>530</v>
-      </c>
-      <c r="C158" s="5" t="s">
-        <v>531</v>
       </c>
       <c r="D158" s="6"/>
       <c r="E158" s="6"/>
@@ -6230,13 +6234,13 @@
     </row>
     <row r="159" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A159" s="4" t="s">
+        <v>530</v>
+      </c>
+      <c r="B159" s="5" t="s">
+        <v>531</v>
+      </c>
+      <c r="C159" s="5" t="s">
         <v>532</v>
-      </c>
-      <c r="B159" s="5" t="s">
-        <v>533</v>
-      </c>
-      <c r="C159" s="5" t="s">
-        <v>534</v>
       </c>
       <c r="D159" s="6"/>
       <c r="E159" s="6"/>
@@ -6252,13 +6256,13 @@
     </row>
     <row r="160" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A160" s="4" t="s">
+        <v>533</v>
+      </c>
+      <c r="B160" s="5" t="s">
+        <v>534</v>
+      </c>
+      <c r="C160" s="5" t="s">
         <v>535</v>
-      </c>
-      <c r="B160" s="5" t="s">
-        <v>536</v>
-      </c>
-      <c r="C160" s="5" t="s">
-        <v>537</v>
       </c>
       <c r="D160" s="6"/>
       <c r="E160" s="6"/>
@@ -6274,13 +6278,13 @@
     </row>
     <row r="161" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A161" s="4" t="s">
+        <v>536</v>
+      </c>
+      <c r="B161" s="5" t="s">
+        <v>537</v>
+      </c>
+      <c r="C161" s="5" t="s">
         <v>538</v>
-      </c>
-      <c r="B161" s="5" t="s">
-        <v>539</v>
-      </c>
-      <c r="C161" s="5" t="s">
-        <v>540</v>
       </c>
       <c r="D161" s="6"/>
       <c r="E161" s="6"/>
@@ -6296,19 +6300,19 @@
     </row>
     <row r="162" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A162" s="4" t="s">
+        <v>539</v>
+      </c>
+      <c r="B162" s="5" t="s">
+        <v>540</v>
+      </c>
+      <c r="C162" s="5" t="s">
         <v>541</v>
-      </c>
-      <c r="B162" s="5" t="s">
-        <v>542</v>
-      </c>
-      <c r="C162" s="5" t="s">
-        <v>543</v>
       </c>
       <c r="D162" s="6"/>
       <c r="E162" s="6"/>
       <c r="F162" s="6"/>
       <c r="G162" s="6" t="s">
-        <v>544</v>
+        <v>542</v>
       </c>
       <c r="H162" s="6"/>
       <c r="I162" s="6"/>
@@ -6320,13 +6324,13 @@
     </row>
     <row r="163" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A163" s="4" t="s">
+        <v>543</v>
+      </c>
+      <c r="B163" s="5" t="s">
+        <v>544</v>
+      </c>
+      <c r="C163" s="5" t="s">
         <v>545</v>
-      </c>
-      <c r="B163" s="5" t="s">
-        <v>546</v>
-      </c>
-      <c r="C163" s="5" t="s">
-        <v>547</v>
       </c>
       <c r="D163" s="6"/>
       <c r="E163" s="6"/>
@@ -6342,13 +6346,13 @@
     </row>
     <row r="164" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A164" s="4" t="s">
+        <v>546</v>
+      </c>
+      <c r="B164" s="5" t="s">
+        <v>547</v>
+      </c>
+      <c r="C164" s="5" t="s">
         <v>548</v>
-      </c>
-      <c r="B164" s="5" t="s">
-        <v>549</v>
-      </c>
-      <c r="C164" s="5" t="s">
-        <v>550</v>
       </c>
       <c r="D164" s="6"/>
       <c r="E164" s="6"/>
@@ -6364,13 +6368,13 @@
     </row>
     <row r="165" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A165" s="4" t="s">
+        <v>549</v>
+      </c>
+      <c r="B165" s="5" t="s">
+        <v>550</v>
+      </c>
+      <c r="C165" s="5" t="s">
         <v>551</v>
-      </c>
-      <c r="B165" s="5" t="s">
-        <v>552</v>
-      </c>
-      <c r="C165" s="5" t="s">
-        <v>553</v>
       </c>
       <c r="D165" s="6"/>
       <c r="E165" s="6"/>
@@ -6386,13 +6390,13 @@
     </row>
     <row r="166" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A166" s="4" t="s">
+        <v>552</v>
+      </c>
+      <c r="B166" s="5" t="s">
+        <v>553</v>
+      </c>
+      <c r="C166" s="5" t="s">
         <v>554</v>
-      </c>
-      <c r="B166" s="5" t="s">
-        <v>555</v>
-      </c>
-      <c r="C166" s="5" t="s">
-        <v>556</v>
       </c>
       <c r="D166" s="6"/>
       <c r="E166" s="6"/>
@@ -6408,13 +6412,13 @@
     </row>
     <row r="167" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A167" s="4" t="s">
+        <v>555</v>
+      </c>
+      <c r="B167" s="5" t="s">
+        <v>556</v>
+      </c>
+      <c r="C167" s="5" t="s">
         <v>557</v>
-      </c>
-      <c r="B167" s="5" t="s">
-        <v>558</v>
-      </c>
-      <c r="C167" s="5" t="s">
-        <v>559</v>
       </c>
       <c r="D167" s="6"/>
       <c r="E167" s="6"/>
@@ -6433,10 +6437,10 @@
     <row r="168" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A168" s="5"/>
       <c r="B168" s="5" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="C168" s="5" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="D168" s="6"/>
       <c r="E168" s="6"/>
@@ -6451,10 +6455,10 @@
     <row r="169" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A169" s="5"/>
       <c r="B169" s="5" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="C169" s="5" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="D169" s="6"/>
       <c r="E169" s="6"/>
@@ -6469,10 +6473,10 @@
     <row r="170" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A170" s="5"/>
       <c r="B170" s="5" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
       <c r="C170" s="5" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="D170" s="6"/>
       <c r="E170" s="6"/>
@@ -6487,10 +6491,10 @@
     <row r="171" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A171" s="5"/>
       <c r="B171" s="5" t="s">
-        <v>566</v>
+        <v>564</v>
       </c>
       <c r="C171" s="5" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
       <c r="D171" s="6"/>
       <c r="E171" s="6"/>
@@ -6505,10 +6509,10 @@
     <row r="172" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A172" s="5"/>
       <c r="B172" s="5" t="s">
-        <v>568</v>
+        <v>566</v>
       </c>
       <c r="C172" s="5" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="D172" s="6"/>
       <c r="E172" s="6"/>
@@ -6523,16 +6527,16 @@
     <row r="173" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A173" s="5"/>
       <c r="B173" s="5" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="C173" s="5" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="D173" s="6"/>
       <c r="E173" s="6"/>
       <c r="F173" s="6"/>
       <c r="G173" s="6" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="H173" s="6"/>
       <c r="I173" s="6"/>
@@ -6543,10 +6547,10 @@
     <row r="174" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A174" s="5"/>
       <c r="B174" s="5" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
       <c r="C174" s="5" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
       <c r="D174" s="6"/>
       <c r="E174" s="6"/>
@@ -6561,10 +6565,10 @@
     <row r="175" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A175" s="5"/>
       <c r="B175" s="5" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="C175" s="5" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="D175" s="6"/>
       <c r="E175" s="6"/>
@@ -6579,10 +6583,10 @@
     <row r="176" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A176" s="5"/>
       <c r="B176" s="5" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="C176" s="5" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="D176" s="6"/>
       <c r="E176" s="6"/>
@@ -6597,10 +6601,10 @@
     <row r="177" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A177" s="5"/>
       <c r="B177" s="5" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="C177" s="5" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="D177" s="6"/>
       <c r="E177" s="6"/>
@@ -6615,10 +6619,10 @@
     <row r="178" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A178" s="5"/>
       <c r="B178" s="5" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="C178" s="5" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="D178" s="6"/>
       <c r="E178" s="6"/>
@@ -6633,10 +6637,10 @@
     <row r="179" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A179" s="5"/>
       <c r="B179" s="5" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="C179" s="5" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="D179" s="6"/>
       <c r="E179" s="6"/>
@@ -6651,10 +6655,10 @@
     <row r="180" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A180" s="5"/>
       <c r="B180" s="5" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="C180" s="5" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="D180" s="6"/>
       <c r="E180" s="6"/>
@@ -6669,10 +6673,10 @@
     <row r="181" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A181" s="5"/>
       <c r="B181" s="5" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="C181" s="5" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
       <c r="D181" s="6"/>
       <c r="E181" s="6"/>
@@ -6687,10 +6691,10 @@
     <row r="182" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A182" s="5"/>
       <c r="B182" s="5" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
       <c r="C182" s="5" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="D182" s="6"/>
       <c r="E182" s="6"/>
@@ -6705,10 +6709,10 @@
     <row r="183" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A183" s="5"/>
       <c r="B183" s="5" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
       <c r="C183" s="5" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="D183" s="6"/>
       <c r="E183" s="6"/>
@@ -18370,13 +18374,13 @@
     </row>
     <row r="1016" spans="1:12" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1016" s="5" t="s">
+        <v>596</v>
+      </c>
+      <c r="B1016" s="5" t="s">
+        <v>597</v>
+      </c>
+      <c r="C1016" s="5" t="s">
         <v>598</v>
-      </c>
-      <c r="B1016" s="5" t="s">
-        <v>599</v>
-      </c>
-      <c r="C1016" s="5" t="s">
-        <v>600</v>
       </c>
       <c r="D1016" s="6"/>
       <c r="E1016" s="6"/>
@@ -18385,24 +18389,24 @@
       <c r="H1016" s="6"/>
       <c r="I1016" s="6"/>
       <c r="J1016" s="6" t="s">
+        <v>599</v>
+      </c>
+      <c r="K1016" s="6" t="s">
+        <v>600</v>
+      </c>
+      <c r="L1016" s="6" t="s">
         <v>601</v>
-      </c>
-      <c r="K1016" s="6" t="s">
-        <v>602</v>
-      </c>
-      <c r="L1016" s="6" t="s">
-        <v>603</v>
       </c>
     </row>
     <row r="1017" spans="1:12" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1017" s="5" t="s">
+        <v>602</v>
+      </c>
+      <c r="B1017" s="5" t="s">
+        <v>603</v>
+      </c>
+      <c r="C1017" s="5" t="s">
         <v>604</v>
-      </c>
-      <c r="B1017" s="5" t="s">
-        <v>605</v>
-      </c>
-      <c r="C1017" s="5" t="s">
-        <v>606</v>
       </c>
       <c r="D1017" s="6"/>
       <c r="E1017" s="6"/>
@@ -18411,13 +18415,13 @@
       <c r="H1017" s="6"/>
       <c r="I1017" s="6"/>
       <c r="J1017" s="6" t="s">
+        <v>599</v>
+      </c>
+      <c r="K1017" s="6" t="s">
+        <v>600</v>
+      </c>
+      <c r="L1017" s="6" t="s">
         <v>601</v>
-      </c>
-      <c r="K1017" s="6" t="s">
-        <v>602</v>
-      </c>
-      <c r="L1017" s="6" t="s">
-        <v>603</v>
       </c>
     </row>
   </sheetData>
@@ -18425,14 +18429,14 @@
     <dataValidation type="list" allowBlank="1" sqref="K2:K1017" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Minor Repeatable,Minor Fire-Once,Major"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="Q2:Q15" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" allowBlank="1" sqref="Q2:Q16" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"1,2,3,4,5"</formula1>
     </dataValidation>
-    <dataValidation allowBlank="1" showDropDown="1" sqref="N2:N15 A2:C1017" xr:uid="{00000000-0002-0000-0000-000002000000}"/>
+    <dataValidation allowBlank="1" showDropDown="1" sqref="N2:N16 A2:C1017" xr:uid="{00000000-0002-0000-0000-000002000000}"/>
     <dataValidation type="list" allowBlank="1" sqref="L2:L1017" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>"Implemented,New,In progress,To Be Reworked,Buggy,Needs Testing"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="R2:R15" xr:uid="{00000000-0002-0000-0000-000004000000}">
+    <dataValidation type="list" allowBlank="1" sqref="R2:R16" xr:uid="{00000000-0002-0000-0000-000004000000}">
       <formula1>"Implemented,New,In progress,Under review,Buggy"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
fixed a crash, cleaned the project
</commit_message>
<xml_diff>
--- a/docs/spreadsheets/chaos_redux_events_catalog.xlsx
+++ b/docs/spreadsheets/chaos_redux_events_catalog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\home\klim\projects\chaos_redux\docs\spreadsheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{654CBF13-214A-458E-AFA9-9C0DD2C2BB93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B9DC280-3EAE-48C3-A93C-CFD43DD36E07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="892" uniqueCount="610">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="895" uniqueCount="611">
   <si>
     <t>ID</t>
   </si>
@@ -172,30 +172,63 @@
     <t>Random War</t>
   </si>
   <si>
+    <t>A random eligible country declares war on another eligible country. Higher chaos stages create larger linked war webs. Compatible special countries can appear in later stages.</t>
+  </si>
+  <si>
+    <t>Gathering Storm: Triangular Incident. Three declarations fire in one linked dispute.</t>
+  </si>
+  <si>
+    <t>Rising Chaos: Four Fronts. Four declarations fire in one conflict web, with a small chance for a compatible special country to appear.</t>
+  </si>
+  <si>
+    <t>Chaos Tier: Contagious Ultimatums. Five declarations fire, major countries and faction members become more likely, and special-country involvement becomes more common.</t>
+  </si>
+  <si>
+    <t>Totalen Chaos: The War Week. Six declarations fire in a short chain, with a strong chance of one compatible special country participating.</t>
+  </si>
+  <si>
+    <t>World Collapse: Open Season. Seven to eight declarations fire while normal random events still run. Compatible special countries are strongly favored when available.</t>
+  </si>
+  <si>
     <t>Minor Repeatable</t>
   </si>
   <si>
+    <t>Wars</t>
+  </si>
+  <si>
+    <t>Repeatable Wars cluster.</t>
+  </si>
+  <si>
+    <t>4, (later add more)</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>Soviet Union Collapse</t>
+  </si>
+  <si>
+    <t>Needs Final Review</t>
+  </si>
+  <si>
+    <t>Liberations</t>
+  </si>
+  <si>
+    <t>Liberation and breakaway shocks centered on a collapsing Soviet Union. Republics can seek recognition, arms, volunteers, intelligence contacts, economic help, or regional partners while the old union tries to hold together.</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>Independence Wave</t>
+  </si>
+  <si>
+    <t>to be reworked</t>
+  </si>
+  <si>
     <t>To Be Reworked</t>
   </si>
   <si>
-    <t>Wars</t>
-  </si>
-  <si>
-    <t>5</t>
-  </si>
-  <si>
-    <t>Soviet Union Collapse</t>
-  </si>
-  <si>
-    <t>Diseases</t>
-  </si>
-  <si>
-    <t>6</t>
-  </si>
-  <si>
-    <t>Independence Wave</t>
-  </si>
-  <si>
     <t>Aliens</t>
   </si>
   <si>
@@ -373,7 +406,7 @@
     <t>random country gets a civil war.</t>
   </si>
   <si>
-    <t xml:space="preserve"> </t>
+    <t/>
   </si>
   <si>
     <t>22</t>
@@ -1798,21 +1831,6 @@
     <t>Happens on a friday,  everything is heavely discounted for one day. A rare event</t>
   </si>
   <si>
-    <t>Gathering Storm: Triangular Incident. Three declarations fire in one linked dispute.</t>
-  </si>
-  <si>
-    <t>Rising Chaos: Four Fronts. Four declarations fire in one conflict web, with a small chance for a compatible special country to appear.</t>
-  </si>
-  <si>
-    <t>Chaos Tier: Contagious Ultimatums. Five declarations fire, major countries and faction members become more likely, and special-country involvement becomes more common.</t>
-  </si>
-  <si>
-    <t>Totalen Chaos: The War Week. Six declarations fire in a short chain, with a strong chance of one compatible special country participating.</t>
-  </si>
-  <si>
-    <t>World Collapse: Open Season. Seven to eight declarations fire while normal random events still run. Compatible special countries are strongly favored when available.</t>
-  </si>
-  <si>
     <t>SCN-001</t>
   </si>
   <si>
@@ -1838,21 +1856,6 @@
   </si>
   <si>
     <t>Triggerable scenario. Manual setup launched from the Chaos Redux scenario window. Type switches between the standard clone army and the stronger Aryan variant; intensity controls starting territory, division count, army strength, equipment, and neighboring pressure.</t>
-  </si>
-  <si>
-    <t>A random eligible country declares war on another eligible country. Higher chaos stages create larger linked war webs. Compatible special countries can appear in later stages.</t>
-  </si>
-  <si>
-    <t>Repeatable Wars cluster.</t>
-  </si>
-  <si>
-    <t>4, (later add more)</t>
-  </si>
-  <si>
-    <t>to be reworked</t>
-  </si>
-  <si>
-    <t>Liberations</t>
   </si>
 </sst>
 </file>
@@ -2013,7 +2016,7 @@
       </border>
     </dxf>
   </dxfs>
-  <tableStyles count="2">
+  <tableStyles count="2" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="Main Sheet-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
       <tableStyleElement type="wholeTable" size="0" dxfId="7"/>
       <tableStyleElement type="headerRow" dxfId="6"/>
@@ -2491,39 +2494,39 @@
         <v>48</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>605</v>
+        <v>49</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>591</v>
+        <v>50</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>592</v>
+        <v>51</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>593</v>
+        <v>52</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>594</v>
+        <v>53</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>595</v>
+        <v>54</v>
       </c>
       <c r="I5" s="6"/>
       <c r="J5" s="6"/>
       <c r="K5" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L5" s="6" t="s">
         <v>23</v>
       </c>
       <c r="N5" s="7" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="O5" s="8" t="s">
-        <v>606</v>
+        <v>57</v>
       </c>
       <c r="P5" s="8" t="s">
-        <v>607</v>
+        <v>58</v>
       </c>
       <c r="Q5" s="8">
         <v>2</v>
@@ -2534,13 +2537,13 @@
     </row>
     <row r="6" spans="1:18" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>608</v>
+        <v>66</v>
       </c>
       <c r="D6" s="6"/>
       <c r="E6" s="6"/>
@@ -2553,29 +2556,33 @@
         <v>22</v>
       </c>
       <c r="L6" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
       <c r="N6" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="O6" s="8"/>
-      <c r="P6" s="8"/>
-      <c r="Q6" s="8">
-        <v>3</v>
+        <v>62</v>
+      </c>
+      <c r="O6" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="P6" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="Q6" s="8" t="s">
+        <v>59</v>
       </c>
       <c r="R6" s="8" t="s">
-        <v>26</v>
+        <v>61</v>
       </c>
     </row>
     <row r="7" spans="1:18" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>608</v>
+        <v>66</v>
       </c>
       <c r="D7" s="6"/>
       <c r="E7" s="6"/>
@@ -2585,13 +2592,13 @@
       <c r="I7" s="6"/>
       <c r="J7" s="6"/>
       <c r="K7" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L7" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
       <c r="N7" s="7" t="s">
-        <v>57</v>
+        <v>68</v>
       </c>
       <c r="O7" s="8"/>
       <c r="P7" s="8"/>
@@ -2604,13 +2611,13 @@
     </row>
     <row r="8" spans="1:18" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>59</v>
+        <v>70</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="D8" s="6"/>
       <c r="E8" s="6"/>
@@ -2620,16 +2627,16 @@
       <c r="I8" s="6"/>
       <c r="J8" s="6"/>
       <c r="K8" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L8" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
       <c r="N8" s="7" t="s">
-        <v>61</v>
+        <v>72</v>
       </c>
       <c r="O8" s="8" t="s">
-        <v>62</v>
+        <v>73</v>
       </c>
       <c r="P8" s="8"/>
       <c r="Q8" s="8">
@@ -2641,13 +2648,13 @@
     </row>
     <row r="9" spans="1:18" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
-        <v>63</v>
+        <v>74</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>64</v>
+        <v>75</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>65</v>
+        <v>76</v>
       </c>
       <c r="D9" s="6"/>
       <c r="E9" s="6"/>
@@ -2657,13 +2664,13 @@
       <c r="I9" s="6"/>
       <c r="J9" s="6"/>
       <c r="K9" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L9" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
       <c r="N9" s="7" t="s">
-        <v>66</v>
+        <v>77</v>
       </c>
       <c r="O9" s="8"/>
       <c r="P9" s="8"/>
@@ -2676,13 +2683,13 @@
     </row>
     <row r="10" spans="1:18" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
-        <v>67</v>
+        <v>78</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>68</v>
+        <v>79</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="D10" s="6"/>
       <c r="E10" s="6"/>
@@ -2692,13 +2699,13 @@
       <c r="I10" s="6"/>
       <c r="J10" s="6"/>
       <c r="K10" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L10" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
       <c r="N10" s="7" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="O10" s="8"/>
       <c r="P10" s="8"/>
@@ -2711,13 +2718,13 @@
     </row>
     <row r="11" spans="1:18" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
-        <v>71</v>
+        <v>82</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="D11" s="6"/>
       <c r="E11" s="6"/>
@@ -2730,13 +2737,13 @@
         <v>22</v>
       </c>
       <c r="L11" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
       <c r="N11" s="7" t="s">
-        <v>74</v>
+        <v>85</v>
       </c>
       <c r="O11" s="8" t="s">
-        <v>75</v>
+        <v>86</v>
       </c>
       <c r="P11" s="8"/>
       <c r="Q11" s="8">
@@ -2748,13 +2755,13 @@
     </row>
     <row r="12" spans="1:18" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="s">
-        <v>76</v>
+        <v>87</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="D12" s="6"/>
       <c r="E12" s="6"/>
@@ -2767,13 +2774,13 @@
         <v>22</v>
       </c>
       <c r="L12" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
       <c r="N12" s="7" t="s">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="O12" s="8" t="s">
-        <v>80</v>
+        <v>91</v>
       </c>
       <c r="P12" s="8"/>
       <c r="Q12" s="8">
@@ -2785,13 +2792,13 @@
     </row>
     <row r="13" spans="1:18" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="4" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>83</v>
+        <v>94</v>
       </c>
       <c r="D13" s="6"/>
       <c r="E13" s="6"/>
@@ -2804,10 +2811,10 @@
         <v>22</v>
       </c>
       <c r="L13" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
       <c r="N13" s="7" t="s">
-        <v>84</v>
+        <v>95</v>
       </c>
       <c r="O13" s="8"/>
       <c r="P13" s="8"/>
@@ -2820,31 +2827,31 @@
     </row>
     <row r="14" spans="1:18" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B14" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="B14" s="5" t="s">
-        <v>74</v>
-      </c>
       <c r="C14" s="5" t="s">
-        <v>86</v>
+        <v>97</v>
       </c>
       <c r="D14" s="6"/>
       <c r="E14" s="6"/>
       <c r="F14" s="6"/>
       <c r="G14" s="6" t="s">
-        <v>87</v>
+        <v>98</v>
       </c>
       <c r="H14" s="6"/>
       <c r="I14" s="6"/>
       <c r="J14" s="6"/>
       <c r="K14" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L14" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
       <c r="N14" s="7" t="s">
-        <v>88</v>
+        <v>99</v>
       </c>
       <c r="O14" s="8"/>
       <c r="P14" s="8"/>
@@ -2857,13 +2864,13 @@
     </row>
     <row r="15" spans="1:18" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="4" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>91</v>
+        <v>102</v>
       </c>
       <c r="D15" s="6"/>
       <c r="E15" s="6"/>
@@ -2873,16 +2880,16 @@
       <c r="I15" s="6"/>
       <c r="J15" s="6"/>
       <c r="K15" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L15" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
       <c r="N15" s="7" t="s">
-        <v>92</v>
+        <v>103</v>
       </c>
       <c r="O15" s="8" t="s">
-        <v>93</v>
+        <v>104</v>
       </c>
       <c r="P15" s="8"/>
       <c r="Q15" s="8">
@@ -2894,13 +2901,13 @@
     </row>
     <row r="16" spans="1:18" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="4" t="s">
-        <v>94</v>
+        <v>105</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>95</v>
+        <v>106</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>96</v>
+        <v>107</v>
       </c>
       <c r="D16" s="6"/>
       <c r="E16" s="6"/>
@@ -2910,13 +2917,13 @@
       <c r="I16" s="6"/>
       <c r="J16" s="6"/>
       <c r="K16" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L16" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
       <c r="N16" t="s">
-        <v>609</v>
+        <v>62</v>
       </c>
       <c r="Q16">
         <v>1</v>
@@ -2927,13 +2934,13 @@
     </row>
     <row r="17" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
-        <v>97</v>
+        <v>108</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>98</v>
+        <v>109</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>99</v>
+        <v>110</v>
       </c>
       <c r="D17" s="6"/>
       <c r="E17" s="6"/>
@@ -2946,18 +2953,18 @@
         <v>22</v>
       </c>
       <c r="L17" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="18" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="4" t="s">
-        <v>100</v>
+        <v>111</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>101</v>
+        <v>112</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>102</v>
+        <v>113</v>
       </c>
       <c r="D18" s="6"/>
       <c r="E18" s="6"/>
@@ -2967,21 +2974,21 @@
       <c r="I18" s="6"/>
       <c r="J18" s="6"/>
       <c r="K18" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L18" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="19" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="4" t="s">
-        <v>103</v>
+        <v>114</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>104</v>
+        <v>115</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>105</v>
+        <v>116</v>
       </c>
       <c r="D19" s="6"/>
       <c r="E19" s="6"/>
@@ -2991,21 +2998,21 @@
       <c r="I19" s="6"/>
       <c r="J19" s="6"/>
       <c r="K19" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L19" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="20" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="4" t="s">
-        <v>106</v>
+        <v>117</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>107</v>
+        <v>118</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>108</v>
+        <v>119</v>
       </c>
       <c r="D20" s="6"/>
       <c r="E20" s="6"/>
@@ -3015,27 +3022,27 @@
       <c r="I20" s="6"/>
       <c r="J20" s="6"/>
       <c r="K20" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L20" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="21" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="4" t="s">
-        <v>109</v>
+        <v>120</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>110</v>
+        <v>121</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>111</v>
+        <v>122</v>
       </c>
       <c r="D21" s="6"/>
       <c r="E21" s="6"/>
       <c r="F21" s="6"/>
       <c r="G21" s="6" t="s">
-        <v>112</v>
+        <v>123</v>
       </c>
       <c r="H21" s="6"/>
       <c r="I21" s="6"/>
@@ -3044,18 +3051,18 @@
         <v>22</v>
       </c>
       <c r="L21" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="22" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="4" t="s">
-        <v>113</v>
+        <v>124</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>114</v>
+        <v>125</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="D22" s="6"/>
       <c r="E22" s="6"/>
@@ -3065,24 +3072,24 @@
       <c r="I22" s="6"/>
       <c r="J22" s="6"/>
       <c r="K22" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L22" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
       <c r="Q22" s="9" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
     </row>
     <row r="23" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="4" t="s">
-        <v>117</v>
+        <v>128</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="D23" s="6"/>
       <c r="E23" s="6"/>
@@ -3095,18 +3102,18 @@
         <v>22</v>
       </c>
       <c r="L23" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="24" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="4" t="s">
-        <v>120</v>
+        <v>131</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>122</v>
+        <v>133</v>
       </c>
       <c r="D24" s="6"/>
       <c r="E24" s="6"/>
@@ -3119,18 +3126,18 @@
         <v>22</v>
       </c>
       <c r="L24" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="25" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="4" t="s">
-        <v>123</v>
+        <v>134</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>125</v>
+        <v>136</v>
       </c>
       <c r="D25" s="6"/>
       <c r="E25" s="6"/>
@@ -3143,18 +3150,18 @@
         <v>22</v>
       </c>
       <c r="L25" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="26" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="4" t="s">
-        <v>126</v>
+        <v>137</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>127</v>
+        <v>138</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>128</v>
+        <v>139</v>
       </c>
       <c r="D26" s="6"/>
       <c r="E26" s="6"/>
@@ -3167,18 +3174,18 @@
         <v>34</v>
       </c>
       <c r="L26" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="27" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="4" t="s">
-        <v>129</v>
+        <v>140</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>130</v>
+        <v>141</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>131</v>
+        <v>142</v>
       </c>
       <c r="D27" s="6"/>
       <c r="E27" s="6"/>
@@ -3191,18 +3198,18 @@
         <v>22</v>
       </c>
       <c r="L27" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="28" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="4" t="s">
-        <v>132</v>
+        <v>143</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>133</v>
+        <v>144</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>134</v>
+        <v>145</v>
       </c>
       <c r="D28" s="6"/>
       <c r="E28" s="6"/>
@@ -3215,18 +3222,18 @@
         <v>22</v>
       </c>
       <c r="L28" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="29" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="4" t="s">
-        <v>135</v>
+        <v>146</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>136</v>
+        <v>147</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>137</v>
+        <v>148</v>
       </c>
       <c r="D29" s="6"/>
       <c r="E29" s="6"/>
@@ -3236,21 +3243,21 @@
       <c r="I29" s="6"/>
       <c r="J29" s="6"/>
       <c r="K29" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L29" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="30" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="4" t="s">
-        <v>138</v>
+        <v>149</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>139</v>
+        <v>150</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>140</v>
+        <v>151</v>
       </c>
       <c r="D30" s="6"/>
       <c r="E30" s="6"/>
@@ -3260,27 +3267,27 @@
       <c r="I30" s="6"/>
       <c r="J30" s="6"/>
       <c r="K30" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L30" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="31" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="4" t="s">
-        <v>141</v>
+        <v>152</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>142</v>
+        <v>153</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>143</v>
+        <v>154</v>
       </c>
       <c r="D31" s="6"/>
       <c r="E31" s="6"/>
       <c r="F31" s="6"/>
       <c r="G31" s="6" t="s">
-        <v>144</v>
+        <v>155</v>
       </c>
       <c r="H31" s="6"/>
       <c r="I31" s="6"/>
@@ -3289,18 +3296,18 @@
         <v>34</v>
       </c>
       <c r="L31" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="32" spans="1:17" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="4" t="s">
-        <v>145</v>
+        <v>156</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>146</v>
+        <v>157</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>147</v>
+        <v>158</v>
       </c>
       <c r="D32" s="6"/>
       <c r="E32" s="6"/>
@@ -3310,21 +3317,21 @@
       <c r="I32" s="6"/>
       <c r="J32" s="6"/>
       <c r="K32" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L32" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="33" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="4" t="s">
-        <v>148</v>
+        <v>159</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>149</v>
+        <v>160</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>150</v>
+        <v>161</v>
       </c>
       <c r="D33" s="6"/>
       <c r="E33" s="6"/>
@@ -3334,21 +3341,21 @@
       <c r="I33" s="6"/>
       <c r="J33" s="6"/>
       <c r="K33" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L33" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="34" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="4" t="s">
-        <v>151</v>
+        <v>162</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>152</v>
+        <v>163</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>153</v>
+        <v>164</v>
       </c>
       <c r="D34" s="6"/>
       <c r="E34" s="6"/>
@@ -3358,21 +3365,21 @@
       <c r="I34" s="6"/>
       <c r="J34" s="6"/>
       <c r="K34" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L34" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="35" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="4" t="s">
-        <v>154</v>
+        <v>165</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>155</v>
+        <v>166</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>156</v>
+        <v>167</v>
       </c>
       <c r="D35" s="6"/>
       <c r="E35" s="6"/>
@@ -3382,21 +3389,21 @@
       <c r="I35" s="6"/>
       <c r="J35" s="6"/>
       <c r="K35" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L35" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="36" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="4" t="s">
-        <v>157</v>
+        <v>168</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>158</v>
+        <v>169</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>159</v>
+        <v>170</v>
       </c>
       <c r="D36" s="6"/>
       <c r="E36" s="6"/>
@@ -3406,21 +3413,21 @@
       <c r="I36" s="6"/>
       <c r="J36" s="6"/>
       <c r="K36" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L36" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="37" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="4" t="s">
-        <v>160</v>
+        <v>171</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>161</v>
+        <v>172</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>162</v>
+        <v>173</v>
       </c>
       <c r="D37" s="6"/>
       <c r="E37" s="6"/>
@@ -3430,21 +3437,21 @@
       <c r="I37" s="6"/>
       <c r="J37" s="6"/>
       <c r="K37" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L37" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="38" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="4" t="s">
-        <v>163</v>
+        <v>174</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>164</v>
+        <v>175</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>165</v>
+        <v>176</v>
       </c>
       <c r="D38" s="6"/>
       <c r="E38" s="6"/>
@@ -3454,27 +3461,27 @@
       <c r="I38" s="6"/>
       <c r="J38" s="6"/>
       <c r="K38" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L38" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="39" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="4" t="s">
-        <v>166</v>
+        <v>177</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>167</v>
+        <v>178</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>168</v>
+        <v>179</v>
       </c>
       <c r="D39" s="6"/>
       <c r="E39" s="6"/>
       <c r="F39" s="6"/>
       <c r="G39" s="6" t="s">
-        <v>169</v>
+        <v>180</v>
       </c>
       <c r="H39" s="6"/>
       <c r="I39" s="6"/>
@@ -3483,18 +3490,18 @@
         <v>22</v>
       </c>
       <c r="L39" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="40" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="4" t="s">
-        <v>170</v>
+        <v>181</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>171</v>
+        <v>182</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>172</v>
+        <v>183</v>
       </c>
       <c r="D40" s="6"/>
       <c r="E40" s="6"/>
@@ -3504,21 +3511,21 @@
       <c r="I40" s="6"/>
       <c r="J40" s="6"/>
       <c r="K40" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L40" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="41" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="4" t="s">
-        <v>173</v>
+        <v>184</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>174</v>
+        <v>185</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>175</v>
+        <v>186</v>
       </c>
       <c r="D41" s="6"/>
       <c r="E41" s="6"/>
@@ -3528,21 +3535,21 @@
       <c r="I41" s="6"/>
       <c r="J41" s="6"/>
       <c r="K41" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L41" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="42" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="4" t="s">
-        <v>176</v>
+        <v>187</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>177</v>
+        <v>188</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>178</v>
+        <v>189</v>
       </c>
       <c r="D42" s="6"/>
       <c r="E42" s="6"/>
@@ -3552,21 +3559,21 @@
       <c r="I42" s="6"/>
       <c r="J42" s="6"/>
       <c r="K42" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L42" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="43" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="4" t="s">
-        <v>179</v>
+        <v>190</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>180</v>
+        <v>191</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>181</v>
+        <v>192</v>
       </c>
       <c r="D43" s="6"/>
       <c r="E43" s="6"/>
@@ -3576,21 +3583,21 @@
       <c r="I43" s="6"/>
       <c r="J43" s="6"/>
       <c r="K43" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L43" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="44" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="4" t="s">
-        <v>182</v>
+        <v>193</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>183</v>
+        <v>194</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>184</v>
+        <v>195</v>
       </c>
       <c r="D44" s="6"/>
       <c r="E44" s="6"/>
@@ -3600,21 +3607,21 @@
       <c r="I44" s="6"/>
       <c r="J44" s="6"/>
       <c r="K44" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L44" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="45" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="4" t="s">
-        <v>185</v>
+        <v>196</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>186</v>
+        <v>197</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>187</v>
+        <v>198</v>
       </c>
       <c r="D45" s="6"/>
       <c r="E45" s="6"/>
@@ -3627,18 +3634,18 @@
         <v>34</v>
       </c>
       <c r="L45" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="46" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="4" t="s">
-        <v>188</v>
+        <v>199</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>189</v>
+        <v>200</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>190</v>
+        <v>201</v>
       </c>
       <c r="D46" s="6"/>
       <c r="E46" s="6"/>
@@ -3651,18 +3658,18 @@
         <v>22</v>
       </c>
       <c r="L46" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="47" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="4" t="s">
-        <v>191</v>
+        <v>202</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>193</v>
+        <v>204</v>
       </c>
       <c r="D47" s="6"/>
       <c r="E47" s="6"/>
@@ -3672,21 +3679,21 @@
       <c r="I47" s="6"/>
       <c r="J47" s="6"/>
       <c r="K47" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L47" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="48" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="4" t="s">
-        <v>194</v>
+        <v>205</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>195</v>
+        <v>206</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>196</v>
+        <v>207</v>
       </c>
       <c r="D48" s="6"/>
       <c r="E48" s="6"/>
@@ -3696,21 +3703,21 @@
       <c r="I48" s="6"/>
       <c r="J48" s="6"/>
       <c r="K48" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L48" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="49" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="4" t="s">
-        <v>197</v>
+        <v>208</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>198</v>
+        <v>209</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>199</v>
+        <v>210</v>
       </c>
       <c r="D49" s="6"/>
       <c r="E49" s="6"/>
@@ -3723,18 +3730,18 @@
         <v>22</v>
       </c>
       <c r="L49" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="50" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="4" t="s">
-        <v>200</v>
+        <v>211</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>201</v>
+        <v>212</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>202</v>
+        <v>213</v>
       </c>
       <c r="D50" s="6"/>
       <c r="E50" s="6"/>
@@ -3747,18 +3754,18 @@
         <v>34</v>
       </c>
       <c r="L50" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="51" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="4" t="s">
-        <v>203</v>
+        <v>214</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>204</v>
+        <v>215</v>
       </c>
       <c r="C51" s="5" t="s">
-        <v>205</v>
+        <v>216</v>
       </c>
       <c r="D51" s="6"/>
       <c r="E51" s="6"/>
@@ -3768,21 +3775,21 @@
       <c r="I51" s="6"/>
       <c r="J51" s="6"/>
       <c r="K51" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L51" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="52" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="4" t="s">
-        <v>206</v>
+        <v>217</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>207</v>
+        <v>218</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>208</v>
+        <v>219</v>
       </c>
       <c r="D52" s="6"/>
       <c r="E52" s="6"/>
@@ -3795,18 +3802,18 @@
         <v>22</v>
       </c>
       <c r="L52" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="53" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="4" t="s">
-        <v>209</v>
+        <v>220</v>
       </c>
       <c r="B53" s="5" t="s">
-        <v>210</v>
+        <v>221</v>
       </c>
       <c r="C53" s="5" t="s">
-        <v>211</v>
+        <v>222</v>
       </c>
       <c r="D53" s="6"/>
       <c r="E53" s="6"/>
@@ -3816,21 +3823,21 @@
       <c r="I53" s="6"/>
       <c r="J53" s="6"/>
       <c r="K53" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L53" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="54" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="4" t="s">
-        <v>212</v>
+        <v>223</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>213</v>
+        <v>224</v>
       </c>
       <c r="C54" s="5" t="s">
-        <v>214</v>
+        <v>225</v>
       </c>
       <c r="D54" s="6"/>
       <c r="E54" s="6"/>
@@ -3843,18 +3850,18 @@
         <v>22</v>
       </c>
       <c r="L54" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="55" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="4" t="s">
-        <v>215</v>
+        <v>226</v>
       </c>
       <c r="B55" s="5" t="s">
-        <v>216</v>
+        <v>227</v>
       </c>
       <c r="C55" s="5" t="s">
-        <v>217</v>
+        <v>228</v>
       </c>
       <c r="D55" s="6"/>
       <c r="E55" s="6"/>
@@ -3864,21 +3871,21 @@
       <c r="I55" s="6"/>
       <c r="J55" s="6"/>
       <c r="K55" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L55" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="56" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="4" t="s">
-        <v>218</v>
+        <v>229</v>
       </c>
       <c r="B56" s="5" t="s">
-        <v>219</v>
+        <v>230</v>
       </c>
       <c r="C56" s="5" t="s">
-        <v>220</v>
+        <v>231</v>
       </c>
       <c r="D56" s="6"/>
       <c r="E56" s="6"/>
@@ -3888,21 +3895,21 @@
       <c r="I56" s="6"/>
       <c r="J56" s="6"/>
       <c r="K56" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L56" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="57" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="4" t="s">
-        <v>221</v>
+        <v>232</v>
       </c>
       <c r="B57" s="5" t="s">
-        <v>222</v>
+        <v>233</v>
       </c>
       <c r="C57" s="5" t="s">
-        <v>223</v>
+        <v>234</v>
       </c>
       <c r="D57" s="6"/>
       <c r="E57" s="6"/>
@@ -3912,21 +3919,21 @@
       <c r="I57" s="6"/>
       <c r="J57" s="6"/>
       <c r="K57" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L57" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="58" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="4" t="s">
-        <v>224</v>
+        <v>235</v>
       </c>
       <c r="B58" s="5" t="s">
-        <v>225</v>
+        <v>236</v>
       </c>
       <c r="C58" s="5" t="s">
-        <v>226</v>
+        <v>237</v>
       </c>
       <c r="D58" s="6"/>
       <c r="E58" s="6"/>
@@ -3936,21 +3943,21 @@
       <c r="I58" s="6"/>
       <c r="J58" s="6"/>
       <c r="K58" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L58" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="59" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="4" t="s">
-        <v>227</v>
+        <v>238</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>228</v>
+        <v>239</v>
       </c>
       <c r="C59" s="5" t="s">
-        <v>229</v>
+        <v>240</v>
       </c>
       <c r="D59" s="6"/>
       <c r="E59" s="6"/>
@@ -3960,21 +3967,21 @@
       <c r="I59" s="6"/>
       <c r="J59" s="6"/>
       <c r="K59" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L59" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="60" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="4" t="s">
-        <v>230</v>
+        <v>241</v>
       </c>
       <c r="B60" s="5" t="s">
-        <v>231</v>
+        <v>242</v>
       </c>
       <c r="C60" s="5" t="s">
-        <v>232</v>
+        <v>243</v>
       </c>
       <c r="D60" s="6"/>
       <c r="E60" s="6"/>
@@ -3987,18 +3994,18 @@
         <v>22</v>
       </c>
       <c r="L60" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="61" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="4" t="s">
-        <v>233</v>
+        <v>244</v>
       </c>
       <c r="B61" s="5" t="s">
-        <v>234</v>
+        <v>245</v>
       </c>
       <c r="C61" s="5" t="s">
-        <v>235</v>
+        <v>246</v>
       </c>
       <c r="D61" s="6"/>
       <c r="E61" s="6"/>
@@ -4008,21 +4015,21 @@
       <c r="I61" s="6"/>
       <c r="J61" s="6"/>
       <c r="K61" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L61" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="62" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="4" t="s">
-        <v>236</v>
+        <v>247</v>
       </c>
       <c r="B62" s="5" t="s">
-        <v>237</v>
+        <v>248</v>
       </c>
       <c r="C62" s="5" t="s">
-        <v>238</v>
+        <v>249</v>
       </c>
       <c r="D62" s="6"/>
       <c r="E62" s="6"/>
@@ -4032,21 +4039,21 @@
       <c r="I62" s="6"/>
       <c r="J62" s="6"/>
       <c r="K62" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L62" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="63" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="4" t="s">
-        <v>239</v>
+        <v>250</v>
       </c>
       <c r="B63" s="5" t="s">
-        <v>240</v>
+        <v>251</v>
       </c>
       <c r="C63" s="5" t="s">
-        <v>241</v>
+        <v>252</v>
       </c>
       <c r="D63" s="6"/>
       <c r="E63" s="6"/>
@@ -4056,21 +4063,21 @@
       <c r="I63" s="6"/>
       <c r="J63" s="6"/>
       <c r="K63" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L63" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="64" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="4" t="s">
-        <v>242</v>
+        <v>253</v>
       </c>
       <c r="B64" s="5" t="s">
-        <v>243</v>
+        <v>254</v>
       </c>
       <c r="C64" s="5" t="s">
-        <v>244</v>
+        <v>255</v>
       </c>
       <c r="D64" s="6"/>
       <c r="E64" s="6"/>
@@ -4080,21 +4087,21 @@
       <c r="I64" s="6"/>
       <c r="J64" s="6"/>
       <c r="K64" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L64" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="65" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="4" t="s">
-        <v>245</v>
+        <v>256</v>
       </c>
       <c r="B65" s="5" t="s">
-        <v>246</v>
+        <v>257</v>
       </c>
       <c r="C65" s="5" t="s">
-        <v>247</v>
+        <v>258</v>
       </c>
       <c r="D65" s="6"/>
       <c r="E65" s="6"/>
@@ -4104,21 +4111,21 @@
       <c r="I65" s="6"/>
       <c r="J65" s="6"/>
       <c r="K65" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L65" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="66" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="4" t="s">
-        <v>248</v>
+        <v>259</v>
       </c>
       <c r="B66" s="5" t="s">
-        <v>249</v>
+        <v>260</v>
       </c>
       <c r="C66" s="5" t="s">
-        <v>250</v>
+        <v>261</v>
       </c>
       <c r="D66" s="6"/>
       <c r="E66" s="6"/>
@@ -4128,21 +4135,21 @@
       <c r="I66" s="6"/>
       <c r="J66" s="6"/>
       <c r="K66" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L66" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="67" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="4" t="s">
-        <v>251</v>
+        <v>262</v>
       </c>
       <c r="B67" s="5" t="s">
-        <v>252</v>
+        <v>263</v>
       </c>
       <c r="C67" s="5" t="s">
-        <v>253</v>
+        <v>264</v>
       </c>
       <c r="D67" s="6"/>
       <c r="E67" s="6"/>
@@ -4152,21 +4159,21 @@
       <c r="I67" s="6"/>
       <c r="J67" s="6"/>
       <c r="K67" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L67" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="68" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="4" t="s">
-        <v>254</v>
+        <v>265</v>
       </c>
       <c r="B68" s="5" t="s">
-        <v>255</v>
+        <v>266</v>
       </c>
       <c r="C68" s="5" t="s">
-        <v>256</v>
+        <v>267</v>
       </c>
       <c r="D68" s="6"/>
       <c r="E68" s="6"/>
@@ -4179,24 +4186,24 @@
         <v>22</v>
       </c>
       <c r="L68" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="69" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="4" t="s">
-        <v>257</v>
+        <v>268</v>
       </c>
       <c r="B69" s="5" t="s">
-        <v>258</v>
+        <v>269</v>
       </c>
       <c r="C69" s="5" t="s">
-        <v>259</v>
+        <v>270</v>
       </c>
       <c r="D69" s="6"/>
       <c r="E69" s="6"/>
       <c r="F69" s="6"/>
       <c r="G69" s="6" t="s">
-        <v>260</v>
+        <v>271</v>
       </c>
       <c r="H69" s="6"/>
       <c r="I69" s="6"/>
@@ -4205,18 +4212,18 @@
         <v>22</v>
       </c>
       <c r="L69" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="70" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="4" t="s">
-        <v>261</v>
+        <v>272</v>
       </c>
       <c r="B70" s="5" t="s">
-        <v>262</v>
+        <v>273</v>
       </c>
       <c r="C70" s="5" t="s">
-        <v>263</v>
+        <v>274</v>
       </c>
       <c r="D70" s="6"/>
       <c r="E70" s="6"/>
@@ -4229,18 +4236,18 @@
         <v>22</v>
       </c>
       <c r="L70" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="71" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="4" t="s">
-        <v>264</v>
+        <v>275</v>
       </c>
       <c r="B71" s="5" t="s">
-        <v>265</v>
+        <v>276</v>
       </c>
       <c r="C71" s="5" t="s">
-        <v>266</v>
+        <v>277</v>
       </c>
       <c r="D71" s="6"/>
       <c r="E71" s="6"/>
@@ -4253,18 +4260,18 @@
         <v>34</v>
       </c>
       <c r="L71" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="72" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="4" t="s">
-        <v>267</v>
+        <v>278</v>
       </c>
       <c r="B72" s="5" t="s">
-        <v>268</v>
+        <v>279</v>
       </c>
       <c r="C72" s="5" t="s">
-        <v>269</v>
+        <v>280</v>
       </c>
       <c r="D72" s="6"/>
       <c r="E72" s="6"/>
@@ -4277,18 +4284,18 @@
         <v>22</v>
       </c>
       <c r="L72" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="73" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="4" t="s">
-        <v>270</v>
+        <v>281</v>
       </c>
       <c r="B73" s="5" t="s">
-        <v>271</v>
+        <v>282</v>
       </c>
       <c r="C73" s="5" t="s">
-        <v>272</v>
+        <v>283</v>
       </c>
       <c r="D73" s="6"/>
       <c r="E73" s="6"/>
@@ -4301,18 +4308,18 @@
         <v>22</v>
       </c>
       <c r="L73" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="74" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="4" t="s">
-        <v>273</v>
+        <v>284</v>
       </c>
       <c r="B74" s="5" t="s">
-        <v>274</v>
+        <v>285</v>
       </c>
       <c r="C74" s="5" t="s">
-        <v>275</v>
+        <v>286</v>
       </c>
       <c r="D74" s="6"/>
       <c r="E74" s="6"/>
@@ -4325,18 +4332,18 @@
         <v>22</v>
       </c>
       <c r="L74" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="75" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="4" t="s">
-        <v>276</v>
+        <v>287</v>
       </c>
       <c r="B75" s="5" t="s">
-        <v>277</v>
+        <v>288</v>
       </c>
       <c r="C75" s="5" t="s">
-        <v>278</v>
+        <v>289</v>
       </c>
       <c r="D75" s="6"/>
       <c r="E75" s="6"/>
@@ -4349,18 +4356,18 @@
         <v>22</v>
       </c>
       <c r="L75" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="76" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" s="4" t="s">
-        <v>279</v>
+        <v>290</v>
       </c>
       <c r="B76" s="5" t="s">
-        <v>280</v>
+        <v>291</v>
       </c>
       <c r="C76" s="5" t="s">
-        <v>281</v>
+        <v>292</v>
       </c>
       <c r="D76" s="6"/>
       <c r="E76" s="6"/>
@@ -4373,18 +4380,18 @@
         <v>22</v>
       </c>
       <c r="L76" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="77" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A77" s="4" t="s">
-        <v>282</v>
+        <v>293</v>
       </c>
       <c r="B77" s="5" t="s">
-        <v>283</v>
+        <v>294</v>
       </c>
       <c r="C77" s="5" t="s">
-        <v>284</v>
+        <v>295</v>
       </c>
       <c r="D77" s="6"/>
       <c r="E77" s="6"/>
@@ -4394,21 +4401,21 @@
       <c r="I77" s="6"/>
       <c r="J77" s="6"/>
       <c r="K77" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L77" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="78" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A78" s="4" t="s">
-        <v>285</v>
+        <v>296</v>
       </c>
       <c r="B78" s="5" t="s">
-        <v>286</v>
+        <v>297</v>
       </c>
       <c r="C78" s="5" t="s">
-        <v>287</v>
+        <v>298</v>
       </c>
       <c r="D78" s="6"/>
       <c r="E78" s="6"/>
@@ -4418,21 +4425,21 @@
       <c r="I78" s="6"/>
       <c r="J78" s="6"/>
       <c r="K78" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L78" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="79" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79" s="4" t="s">
-        <v>288</v>
+        <v>299</v>
       </c>
       <c r="B79" s="5" t="s">
-        <v>289</v>
+        <v>300</v>
       </c>
       <c r="C79" s="5" t="s">
-        <v>290</v>
+        <v>301</v>
       </c>
       <c r="D79" s="6"/>
       <c r="E79" s="6"/>
@@ -4442,21 +4449,21 @@
       <c r="I79" s="6"/>
       <c r="J79" s="6"/>
       <c r="K79" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L79" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="80" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A80" s="4" t="s">
-        <v>291</v>
+        <v>302</v>
       </c>
       <c r="B80" s="5" t="s">
-        <v>292</v>
+        <v>303</v>
       </c>
       <c r="C80" s="5" t="s">
-        <v>293</v>
+        <v>304</v>
       </c>
       <c r="D80" s="6"/>
       <c r="E80" s="6"/>
@@ -4466,21 +4473,21 @@
       <c r="I80" s="6"/>
       <c r="J80" s="6"/>
       <c r="K80" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L80" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="81" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" s="4" t="s">
-        <v>294</v>
+        <v>305</v>
       </c>
       <c r="B81" s="5" t="s">
-        <v>295</v>
+        <v>306</v>
       </c>
       <c r="C81" s="5" t="s">
-        <v>296</v>
+        <v>307</v>
       </c>
       <c r="D81" s="6"/>
       <c r="E81" s="6"/>
@@ -4493,18 +4500,18 @@
         <v>34</v>
       </c>
       <c r="L81" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="82" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A82" s="4" t="s">
-        <v>297</v>
+        <v>308</v>
       </c>
       <c r="B82" s="5" t="s">
-        <v>298</v>
+        <v>309</v>
       </c>
       <c r="C82" s="5" t="s">
-        <v>299</v>
+        <v>310</v>
       </c>
       <c r="D82" s="6"/>
       <c r="E82" s="6"/>
@@ -4517,18 +4524,18 @@
         <v>22</v>
       </c>
       <c r="L82" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="83" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" s="4" t="s">
-        <v>300</v>
+        <v>311</v>
       </c>
       <c r="B83" s="5" t="s">
-        <v>301</v>
+        <v>312</v>
       </c>
       <c r="C83" s="5" t="s">
-        <v>302</v>
+        <v>313</v>
       </c>
       <c r="D83" s="6"/>
       <c r="E83" s="6"/>
@@ -4538,21 +4545,21 @@
       <c r="I83" s="6"/>
       <c r="J83" s="6"/>
       <c r="K83" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L83" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="84" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A84" s="4" t="s">
-        <v>303</v>
+        <v>314</v>
       </c>
       <c r="B84" s="5" t="s">
-        <v>304</v>
+        <v>315</v>
       </c>
       <c r="C84" s="5" t="s">
-        <v>305</v>
+        <v>316</v>
       </c>
       <c r="D84" s="6"/>
       <c r="E84" s="6"/>
@@ -4562,21 +4569,21 @@
       <c r="I84" s="6"/>
       <c r="J84" s="6"/>
       <c r="K84" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L84" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="85" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A85" s="4" t="s">
-        <v>306</v>
+        <v>317</v>
       </c>
       <c r="B85" s="5" t="s">
-        <v>307</v>
+        <v>318</v>
       </c>
       <c r="C85" s="5" t="s">
-        <v>308</v>
+        <v>319</v>
       </c>
       <c r="D85" s="6"/>
       <c r="E85" s="6"/>
@@ -4586,21 +4593,21 @@
       <c r="I85" s="6"/>
       <c r="J85" s="6"/>
       <c r="K85" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L85" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="86" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A86" s="4" t="s">
-        <v>309</v>
+        <v>320</v>
       </c>
       <c r="B86" s="5" t="s">
-        <v>310</v>
+        <v>321</v>
       </c>
       <c r="C86" s="5" t="s">
-        <v>311</v>
+        <v>322</v>
       </c>
       <c r="D86" s="6"/>
       <c r="E86" s="6"/>
@@ -4610,21 +4617,21 @@
       <c r="I86" s="6"/>
       <c r="J86" s="6"/>
       <c r="K86" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L86" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="87" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A87" s="4" t="s">
-        <v>312</v>
+        <v>323</v>
       </c>
       <c r="B87" s="5" t="s">
-        <v>313</v>
+        <v>324</v>
       </c>
       <c r="C87" s="5" t="s">
-        <v>314</v>
+        <v>325</v>
       </c>
       <c r="D87" s="6"/>
       <c r="E87" s="6"/>
@@ -4637,18 +4644,18 @@
         <v>22</v>
       </c>
       <c r="L87" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="88" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A88" s="4" t="s">
-        <v>315</v>
+        <v>326</v>
       </c>
       <c r="B88" s="5" t="s">
-        <v>316</v>
+        <v>327</v>
       </c>
       <c r="C88" s="5" t="s">
-        <v>317</v>
+        <v>328</v>
       </c>
       <c r="D88" s="6"/>
       <c r="E88" s="6"/>
@@ -4658,21 +4665,21 @@
       <c r="I88" s="6"/>
       <c r="J88" s="6"/>
       <c r="K88" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L88" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="89" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A89" s="4" t="s">
-        <v>318</v>
+        <v>329</v>
       </c>
       <c r="B89" s="5" t="s">
-        <v>319</v>
+        <v>330</v>
       </c>
       <c r="C89" s="5" t="s">
-        <v>320</v>
+        <v>331</v>
       </c>
       <c r="D89" s="6"/>
       <c r="E89" s="6"/>
@@ -4685,18 +4692,18 @@
         <v>22</v>
       </c>
       <c r="L89" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="90" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A90" s="4" t="s">
-        <v>321</v>
+        <v>332</v>
       </c>
       <c r="B90" s="5" t="s">
-        <v>322</v>
+        <v>333</v>
       </c>
       <c r="C90" s="5" t="s">
-        <v>323</v>
+        <v>334</v>
       </c>
       <c r="D90" s="6"/>
       <c r="E90" s="6"/>
@@ -4709,18 +4716,18 @@
         <v>22</v>
       </c>
       <c r="L90" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="91" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A91" s="4" t="s">
-        <v>324</v>
+        <v>335</v>
       </c>
       <c r="B91" s="5" t="s">
-        <v>325</v>
+        <v>336</v>
       </c>
       <c r="C91" s="5" t="s">
-        <v>326</v>
+        <v>337</v>
       </c>
       <c r="D91" s="6"/>
       <c r="E91" s="6"/>
@@ -4733,24 +4740,24 @@
         <v>22</v>
       </c>
       <c r="L91" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="92" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A92" s="4" t="s">
-        <v>327</v>
+        <v>338</v>
       </c>
       <c r="B92" s="5" t="s">
-        <v>328</v>
+        <v>339</v>
       </c>
       <c r="C92" s="5" t="s">
-        <v>329</v>
+        <v>340</v>
       </c>
       <c r="D92" s="6"/>
       <c r="E92" s="6"/>
       <c r="F92" s="6"/>
       <c r="G92" s="6" t="s">
-        <v>330</v>
+        <v>341</v>
       </c>
       <c r="H92" s="6"/>
       <c r="I92" s="6"/>
@@ -4759,18 +4766,18 @@
         <v>34</v>
       </c>
       <c r="L92" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="93" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A93" s="4" t="s">
-        <v>331</v>
+        <v>342</v>
       </c>
       <c r="B93" s="5" t="s">
-        <v>332</v>
+        <v>343</v>
       </c>
       <c r="C93" s="5" t="s">
-        <v>333</v>
+        <v>344</v>
       </c>
       <c r="D93" s="6"/>
       <c r="E93" s="6"/>
@@ -4783,18 +4790,18 @@
         <v>22</v>
       </c>
       <c r="L93" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="94" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A94" s="4" t="s">
-        <v>334</v>
+        <v>345</v>
       </c>
       <c r="B94" s="5" t="s">
-        <v>335</v>
+        <v>346</v>
       </c>
       <c r="C94" s="5" t="s">
-        <v>336</v>
+        <v>347</v>
       </c>
       <c r="D94" s="6"/>
       <c r="E94" s="6"/>
@@ -4807,18 +4814,18 @@
         <v>22</v>
       </c>
       <c r="L94" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="95" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A95" s="4" t="s">
-        <v>337</v>
+        <v>348</v>
       </c>
       <c r="B95" s="5" t="s">
-        <v>338</v>
+        <v>349</v>
       </c>
       <c r="C95" s="5" t="s">
-        <v>339</v>
+        <v>350</v>
       </c>
       <c r="D95" s="6"/>
       <c r="E95" s="6"/>
@@ -4828,21 +4835,21 @@
       <c r="I95" s="6"/>
       <c r="J95" s="6"/>
       <c r="K95" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L95" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="96" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A96" s="4" t="s">
-        <v>340</v>
+        <v>351</v>
       </c>
       <c r="B96" s="5" t="s">
-        <v>341</v>
+        <v>352</v>
       </c>
       <c r="C96" s="5" t="s">
-        <v>342</v>
+        <v>353</v>
       </c>
       <c r="D96" s="6"/>
       <c r="E96" s="6"/>
@@ -4852,21 +4859,21 @@
       <c r="I96" s="6"/>
       <c r="J96" s="6"/>
       <c r="K96" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L96" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="97" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A97" s="4" t="s">
-        <v>343</v>
+        <v>354</v>
       </c>
       <c r="B97" s="5" t="s">
-        <v>344</v>
+        <v>355</v>
       </c>
       <c r="C97" s="5" t="s">
-        <v>345</v>
+        <v>356</v>
       </c>
       <c r="D97" s="6"/>
       <c r="E97" s="6"/>
@@ -4876,21 +4883,21 @@
       <c r="I97" s="6"/>
       <c r="J97" s="6"/>
       <c r="K97" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L97" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="98" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A98" s="4" t="s">
-        <v>346</v>
+        <v>357</v>
       </c>
       <c r="B98" s="5" t="s">
-        <v>347</v>
+        <v>358</v>
       </c>
       <c r="C98" s="5" t="s">
-        <v>348</v>
+        <v>359</v>
       </c>
       <c r="D98" s="6"/>
       <c r="E98" s="6"/>
@@ -4900,21 +4907,21 @@
       <c r="I98" s="6"/>
       <c r="J98" s="6"/>
       <c r="K98" s="6" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L98" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="99" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A99" s="4" t="s">
-        <v>349</v>
+        <v>360</v>
       </c>
       <c r="B99" s="5" t="s">
-        <v>350</v>
+        <v>361</v>
       </c>
       <c r="C99" s="5" t="s">
-        <v>351</v>
+        <v>362</v>
       </c>
       <c r="D99" s="6"/>
       <c r="E99" s="6"/>
@@ -4927,18 +4934,18 @@
         <v>22</v>
       </c>
       <c r="L99" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="100" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A100" s="4" t="s">
-        <v>352</v>
+        <v>363</v>
       </c>
       <c r="B100" s="5" t="s">
-        <v>353</v>
+        <v>364</v>
       </c>
       <c r="C100" s="5" t="s">
-        <v>354</v>
+        <v>365</v>
       </c>
       <c r="D100" s="6"/>
       <c r="E100" s="6"/>
@@ -4951,18 +4958,18 @@
         <v>22</v>
       </c>
       <c r="L100" s="6" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="101" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A101" s="4" t="s">
-        <v>355</v>
+        <v>366</v>
       </c>
       <c r="B101" s="5" t="s">
-        <v>356</v>
+        <v>367</v>
       </c>
       <c r="C101" s="5" t="s">
-        <v>357</v>
+        <v>368</v>
       </c>
       <c r="D101" s="6"/>
       <c r="E101" s="6"/>
@@ -4978,13 +4985,13 @@
     </row>
     <row r="102" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A102" s="4" t="s">
-        <v>358</v>
+        <v>369</v>
       </c>
       <c r="B102" s="5" t="s">
-        <v>359</v>
+        <v>370</v>
       </c>
       <c r="C102" s="5" t="s">
-        <v>360</v>
+        <v>371</v>
       </c>
       <c r="D102" s="6"/>
       <c r="E102" s="6"/>
@@ -5000,13 +5007,13 @@
     </row>
     <row r="103" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A103" s="4" t="s">
-        <v>361</v>
+        <v>372</v>
       </c>
       <c r="B103" s="5" t="s">
-        <v>362</v>
+        <v>373</v>
       </c>
       <c r="C103" s="5" t="s">
-        <v>363</v>
+        <v>374</v>
       </c>
       <c r="D103" s="6"/>
       <c r="E103" s="6"/>
@@ -5022,13 +5029,13 @@
     </row>
     <row r="104" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A104" s="4" t="s">
-        <v>364</v>
+        <v>375</v>
       </c>
       <c r="B104" s="5" t="s">
-        <v>365</v>
+        <v>376</v>
       </c>
       <c r="C104" s="5" t="s">
-        <v>366</v>
+        <v>377</v>
       </c>
       <c r="D104" s="6"/>
       <c r="E104" s="6"/>
@@ -5044,13 +5051,13 @@
     </row>
     <row r="105" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A105" s="4" t="s">
-        <v>367</v>
+        <v>378</v>
       </c>
       <c r="B105" s="5" t="s">
-        <v>368</v>
+        <v>379</v>
       </c>
       <c r="C105" s="5" t="s">
-        <v>369</v>
+        <v>380</v>
       </c>
       <c r="D105" s="6"/>
       <c r="E105" s="6"/>
@@ -5066,13 +5073,13 @@
     </row>
     <row r="106" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A106" s="4" t="s">
-        <v>370</v>
+        <v>381</v>
       </c>
       <c r="B106" s="5" t="s">
-        <v>371</v>
+        <v>382</v>
       </c>
       <c r="C106" s="5" t="s">
-        <v>372</v>
+        <v>383</v>
       </c>
       <c r="D106" s="6"/>
       <c r="E106" s="6"/>
@@ -5088,13 +5095,13 @@
     </row>
     <row r="107" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A107" s="4" t="s">
-        <v>373</v>
+        <v>384</v>
       </c>
       <c r="B107" s="5" t="s">
-        <v>374</v>
+        <v>385</v>
       </c>
       <c r="C107" s="5" t="s">
-        <v>375</v>
+        <v>386</v>
       </c>
       <c r="D107" s="6"/>
       <c r="E107" s="6"/>
@@ -5110,13 +5117,13 @@
     </row>
     <row r="108" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A108" s="4" t="s">
-        <v>376</v>
+        <v>387</v>
       </c>
       <c r="B108" s="5" t="s">
-        <v>377</v>
+        <v>388</v>
       </c>
       <c r="C108" s="5" t="s">
-        <v>378</v>
+        <v>389</v>
       </c>
       <c r="D108" s="6"/>
       <c r="E108" s="6"/>
@@ -5132,13 +5139,13 @@
     </row>
     <row r="109" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A109" s="4" t="s">
-        <v>379</v>
+        <v>390</v>
       </c>
       <c r="B109" s="5" t="s">
-        <v>380</v>
+        <v>391</v>
       </c>
       <c r="C109" s="5" t="s">
-        <v>381</v>
+        <v>392</v>
       </c>
       <c r="D109" s="6"/>
       <c r="E109" s="6"/>
@@ -5154,13 +5161,13 @@
     </row>
     <row r="110" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A110" s="4" t="s">
-        <v>382</v>
+        <v>393</v>
       </c>
       <c r="B110" s="5" t="s">
-        <v>383</v>
+        <v>394</v>
       </c>
       <c r="C110" s="5" t="s">
-        <v>384</v>
+        <v>395</v>
       </c>
       <c r="D110" s="6"/>
       <c r="E110" s="6"/>
@@ -5176,13 +5183,13 @@
     </row>
     <row r="111" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A111" s="4" t="s">
-        <v>385</v>
+        <v>396</v>
       </c>
       <c r="B111" s="5" t="s">
-        <v>386</v>
+        <v>397</v>
       </c>
       <c r="C111" s="5" t="s">
-        <v>387</v>
+        <v>398</v>
       </c>
       <c r="D111" s="6"/>
       <c r="E111" s="6"/>
@@ -5198,13 +5205,13 @@
     </row>
     <row r="112" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A112" s="4" t="s">
-        <v>388</v>
+        <v>399</v>
       </c>
       <c r="B112" s="5" t="s">
-        <v>389</v>
+        <v>400</v>
       </c>
       <c r="C112" s="5" t="s">
-        <v>390</v>
+        <v>401</v>
       </c>
       <c r="D112" s="6"/>
       <c r="E112" s="6"/>
@@ -5220,13 +5227,13 @@
     </row>
     <row r="113" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A113" s="4" t="s">
-        <v>391</v>
+        <v>402</v>
       </c>
       <c r="B113" s="5" t="s">
-        <v>392</v>
+        <v>403</v>
       </c>
       <c r="C113" s="5" t="s">
-        <v>393</v>
+        <v>404</v>
       </c>
       <c r="D113" s="6"/>
       <c r="E113" s="6"/>
@@ -5242,13 +5249,13 @@
     </row>
     <row r="114" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A114" s="4" t="s">
-        <v>394</v>
+        <v>405</v>
       </c>
       <c r="B114" s="5" t="s">
-        <v>395</v>
+        <v>406</v>
       </c>
       <c r="C114" s="5" t="s">
-        <v>396</v>
+        <v>407</v>
       </c>
       <c r="D114" s="6"/>
       <c r="E114" s="6"/>
@@ -5264,13 +5271,13 @@
     </row>
     <row r="115" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A115" s="4" t="s">
-        <v>397</v>
+        <v>408</v>
       </c>
       <c r="B115" s="5" t="s">
-        <v>398</v>
+        <v>409</v>
       </c>
       <c r="C115" s="5" t="s">
-        <v>399</v>
+        <v>410</v>
       </c>
       <c r="D115" s="6"/>
       <c r="E115" s="6"/>
@@ -5286,13 +5293,13 @@
     </row>
     <row r="116" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A116" s="4" t="s">
-        <v>400</v>
+        <v>411</v>
       </c>
       <c r="B116" s="5" t="s">
-        <v>401</v>
+        <v>412</v>
       </c>
       <c r="C116" s="5" t="s">
-        <v>402</v>
+        <v>413</v>
       </c>
       <c r="D116" s="6"/>
       <c r="E116" s="6"/>
@@ -5308,13 +5315,13 @@
     </row>
     <row r="117" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A117" s="4" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="B117" s="5" t="s">
-        <v>404</v>
+        <v>415</v>
       </c>
       <c r="C117" s="5" t="s">
-        <v>405</v>
+        <v>416</v>
       </c>
       <c r="D117" s="6"/>
       <c r="E117" s="6"/>
@@ -5330,13 +5337,13 @@
     </row>
     <row r="118" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A118" s="4" t="s">
-        <v>406</v>
+        <v>417</v>
       </c>
       <c r="B118" s="5" t="s">
-        <v>407</v>
+        <v>418</v>
       </c>
       <c r="C118" s="5" t="s">
-        <v>408</v>
+        <v>419</v>
       </c>
       <c r="D118" s="6"/>
       <c r="E118" s="6"/>
@@ -5352,13 +5359,13 @@
     </row>
     <row r="119" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A119" s="4" t="s">
-        <v>409</v>
+        <v>420</v>
       </c>
       <c r="B119" s="5" t="s">
-        <v>410</v>
+        <v>421</v>
       </c>
       <c r="C119" s="5" t="s">
-        <v>411</v>
+        <v>422</v>
       </c>
       <c r="D119" s="6"/>
       <c r="E119" s="6"/>
@@ -5374,13 +5381,13 @@
     </row>
     <row r="120" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A120" s="4" t="s">
-        <v>412</v>
+        <v>423</v>
       </c>
       <c r="B120" s="5" t="s">
-        <v>413</v>
+        <v>424</v>
       </c>
       <c r="C120" s="5" t="s">
-        <v>414</v>
+        <v>425</v>
       </c>
       <c r="D120" s="6"/>
       <c r="E120" s="6"/>
@@ -5396,13 +5403,13 @@
     </row>
     <row r="121" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A121" s="4" t="s">
-        <v>415</v>
+        <v>426</v>
       </c>
       <c r="B121" s="5" t="s">
-        <v>416</v>
+        <v>427</v>
       </c>
       <c r="C121" s="5" t="s">
-        <v>417</v>
+        <v>428</v>
       </c>
       <c r="D121" s="6"/>
       <c r="E121" s="6"/>
@@ -5418,13 +5425,13 @@
     </row>
     <row r="122" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A122" s="4" t="s">
-        <v>418</v>
+        <v>429</v>
       </c>
       <c r="B122" s="5" t="s">
-        <v>419</v>
+        <v>430</v>
       </c>
       <c r="C122" s="5" t="s">
-        <v>420</v>
+        <v>431</v>
       </c>
       <c r="D122" s="6"/>
       <c r="E122" s="6"/>
@@ -5440,13 +5447,13 @@
     </row>
     <row r="123" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A123" s="4" t="s">
-        <v>421</v>
+        <v>432</v>
       </c>
       <c r="B123" s="5" t="s">
-        <v>422</v>
+        <v>433</v>
       </c>
       <c r="C123" s="5" t="s">
-        <v>423</v>
+        <v>434</v>
       </c>
       <c r="D123" s="6"/>
       <c r="E123" s="6"/>
@@ -5462,13 +5469,13 @@
     </row>
     <row r="124" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A124" s="4" t="s">
-        <v>424</v>
+        <v>435</v>
       </c>
       <c r="B124" s="5" t="s">
-        <v>425</v>
+        <v>436</v>
       </c>
       <c r="C124" s="5" t="s">
-        <v>426</v>
+        <v>437</v>
       </c>
       <c r="D124" s="6"/>
       <c r="E124" s="6"/>
@@ -5484,13 +5491,13 @@
     </row>
     <row r="125" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A125" s="4" t="s">
-        <v>427</v>
+        <v>438</v>
       </c>
       <c r="B125" s="5" t="s">
-        <v>428</v>
+        <v>439</v>
       </c>
       <c r="C125" s="5" t="s">
-        <v>429</v>
+        <v>440</v>
       </c>
       <c r="D125" s="6"/>
       <c r="E125" s="6"/>
@@ -5506,13 +5513,13 @@
     </row>
     <row r="126" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A126" s="4" t="s">
-        <v>430</v>
+        <v>441</v>
       </c>
       <c r="B126" s="5" t="s">
-        <v>431</v>
+        <v>442</v>
       </c>
       <c r="C126" s="5" t="s">
-        <v>432</v>
+        <v>443</v>
       </c>
       <c r="D126" s="6"/>
       <c r="E126" s="6"/>
@@ -5528,13 +5535,13 @@
     </row>
     <row r="127" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A127" s="4" t="s">
-        <v>433</v>
+        <v>444</v>
       </c>
       <c r="B127" s="5" t="s">
-        <v>434</v>
+        <v>445</v>
       </c>
       <c r="C127" s="5" t="s">
-        <v>435</v>
+        <v>446</v>
       </c>
       <c r="D127" s="6"/>
       <c r="E127" s="6"/>
@@ -5550,13 +5557,13 @@
     </row>
     <row r="128" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A128" s="4" t="s">
-        <v>436</v>
+        <v>447</v>
       </c>
       <c r="B128" s="5" t="s">
-        <v>437</v>
+        <v>448</v>
       </c>
       <c r="C128" s="5" t="s">
-        <v>438</v>
+        <v>449</v>
       </c>
       <c r="D128" s="6"/>
       <c r="E128" s="6"/>
@@ -5572,13 +5579,13 @@
     </row>
     <row r="129" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A129" s="4" t="s">
-        <v>439</v>
+        <v>450</v>
       </c>
       <c r="B129" s="5" t="s">
-        <v>440</v>
+        <v>451</v>
       </c>
       <c r="C129" s="5" t="s">
-        <v>441</v>
+        <v>452</v>
       </c>
       <c r="D129" s="6"/>
       <c r="E129" s="6"/>
@@ -5594,13 +5601,13 @@
     </row>
     <row r="130" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A130" s="4" t="s">
-        <v>442</v>
+        <v>453</v>
       </c>
       <c r="B130" s="5" t="s">
-        <v>443</v>
+        <v>454</v>
       </c>
       <c r="C130" s="5" t="s">
-        <v>444</v>
+        <v>455</v>
       </c>
       <c r="D130" s="6"/>
       <c r="E130" s="6"/>
@@ -5616,13 +5623,13 @@
     </row>
     <row r="131" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A131" s="4" t="s">
-        <v>445</v>
+        <v>456</v>
       </c>
       <c r="B131" s="5" t="s">
-        <v>446</v>
+        <v>457</v>
       </c>
       <c r="C131" s="5" t="s">
-        <v>447</v>
+        <v>458</v>
       </c>
       <c r="D131" s="6"/>
       <c r="E131" s="6"/>
@@ -5638,13 +5645,13 @@
     </row>
     <row r="132" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A132" s="4" t="s">
-        <v>448</v>
+        <v>459</v>
       </c>
       <c r="B132" s="5" t="s">
-        <v>449</v>
+        <v>460</v>
       </c>
       <c r="C132" s="5" t="s">
-        <v>450</v>
+        <v>461</v>
       </c>
       <c r="D132" s="6"/>
       <c r="E132" s="6"/>
@@ -5660,13 +5667,13 @@
     </row>
     <row r="133" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A133" s="4" t="s">
-        <v>451</v>
+        <v>462</v>
       </c>
       <c r="B133" s="5" t="s">
-        <v>452</v>
+        <v>463</v>
       </c>
       <c r="C133" s="5" t="s">
-        <v>453</v>
+        <v>464</v>
       </c>
       <c r="D133" s="6"/>
       <c r="E133" s="6"/>
@@ -5682,13 +5689,13 @@
     </row>
     <row r="134" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A134" s="4" t="s">
-        <v>454</v>
+        <v>465</v>
       </c>
       <c r="B134" s="5" t="s">
-        <v>455</v>
+        <v>466</v>
       </c>
       <c r="C134" s="5" t="s">
-        <v>456</v>
+        <v>467</v>
       </c>
       <c r="D134" s="6"/>
       <c r="E134" s="6"/>
@@ -5704,13 +5711,13 @@
     </row>
     <row r="135" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A135" s="4" t="s">
-        <v>457</v>
+        <v>468</v>
       </c>
       <c r="B135" s="5" t="s">
-        <v>458</v>
+        <v>469</v>
       </c>
       <c r="C135" s="5" t="s">
-        <v>459</v>
+        <v>470</v>
       </c>
       <c r="D135" s="6"/>
       <c r="E135" s="6"/>
@@ -5726,13 +5733,13 @@
     </row>
     <row r="136" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A136" s="4" t="s">
-        <v>460</v>
+        <v>471</v>
       </c>
       <c r="B136" s="5" t="s">
-        <v>461</v>
+        <v>472</v>
       </c>
       <c r="C136" s="5" t="s">
-        <v>462</v>
+        <v>473</v>
       </c>
       <c r="D136" s="6"/>
       <c r="E136" s="6"/>
@@ -5748,13 +5755,13 @@
     </row>
     <row r="137" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A137" s="4" t="s">
-        <v>463</v>
+        <v>474</v>
       </c>
       <c r="B137" s="5" t="s">
-        <v>464</v>
+        <v>475</v>
       </c>
       <c r="C137" s="5" t="s">
-        <v>465</v>
+        <v>476</v>
       </c>
       <c r="D137" s="6"/>
       <c r="E137" s="6"/>
@@ -5770,13 +5777,13 @@
     </row>
     <row r="138" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A138" s="4" t="s">
-        <v>466</v>
+        <v>477</v>
       </c>
       <c r="B138" s="5" t="s">
-        <v>467</v>
+        <v>478</v>
       </c>
       <c r="C138" s="5" t="s">
-        <v>468</v>
+        <v>479</v>
       </c>
       <c r="D138" s="6"/>
       <c r="E138" s="6"/>
@@ -5792,13 +5799,13 @@
     </row>
     <row r="139" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A139" s="4" t="s">
-        <v>469</v>
+        <v>480</v>
       </c>
       <c r="B139" s="5" t="s">
-        <v>470</v>
+        <v>481</v>
       </c>
       <c r="C139" s="5" t="s">
-        <v>471</v>
+        <v>482</v>
       </c>
       <c r="D139" s="6"/>
       <c r="E139" s="6"/>
@@ -5814,13 +5821,13 @@
     </row>
     <row r="140" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A140" s="4" t="s">
-        <v>472</v>
+        <v>483</v>
       </c>
       <c r="B140" s="5" t="s">
-        <v>473</v>
+        <v>484</v>
       </c>
       <c r="C140" s="5" t="s">
-        <v>474</v>
+        <v>485</v>
       </c>
       <c r="D140" s="6"/>
       <c r="E140" s="6"/>
@@ -5836,13 +5843,13 @@
     </row>
     <row r="141" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A141" s="4" t="s">
-        <v>475</v>
+        <v>486</v>
       </c>
       <c r="B141" s="5" t="s">
-        <v>476</v>
+        <v>487</v>
       </c>
       <c r="C141" s="5" t="s">
-        <v>477</v>
+        <v>488</v>
       </c>
       <c r="D141" s="6"/>
       <c r="E141" s="6"/>
@@ -5858,13 +5865,13 @@
     </row>
     <row r="142" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A142" s="4" t="s">
-        <v>478</v>
+        <v>489</v>
       </c>
       <c r="B142" s="5" t="s">
-        <v>479</v>
+        <v>490</v>
       </c>
       <c r="C142" s="5" t="s">
-        <v>480</v>
+        <v>491</v>
       </c>
       <c r="D142" s="6"/>
       <c r="E142" s="6"/>
@@ -5880,13 +5887,13 @@
     </row>
     <row r="143" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A143" s="4" t="s">
-        <v>481</v>
+        <v>492</v>
       </c>
       <c r="B143" s="5" t="s">
-        <v>482</v>
+        <v>493</v>
       </c>
       <c r="C143" s="5" t="s">
-        <v>483</v>
+        <v>494</v>
       </c>
       <c r="D143" s="6"/>
       <c r="E143" s="6"/>
@@ -5902,13 +5909,13 @@
     </row>
     <row r="144" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A144" s="4" t="s">
-        <v>484</v>
+        <v>495</v>
       </c>
       <c r="B144" s="5" t="s">
-        <v>485</v>
+        <v>496</v>
       </c>
       <c r="C144" s="5" t="s">
-        <v>486</v>
+        <v>497</v>
       </c>
       <c r="D144" s="6"/>
       <c r="E144" s="6"/>
@@ -5924,13 +5931,13 @@
     </row>
     <row r="145" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A145" s="4" t="s">
-        <v>487</v>
+        <v>498</v>
       </c>
       <c r="B145" s="5" t="s">
-        <v>488</v>
+        <v>499</v>
       </c>
       <c r="C145" s="5" t="s">
-        <v>489</v>
+        <v>500</v>
       </c>
       <c r="D145" s="6"/>
       <c r="E145" s="6"/>
@@ -5946,13 +5953,13 @@
     </row>
     <row r="146" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A146" s="4" t="s">
-        <v>490</v>
+        <v>501</v>
       </c>
       <c r="B146" s="5" t="s">
-        <v>491</v>
+        <v>502</v>
       </c>
       <c r="C146" s="5" t="s">
-        <v>492</v>
+        <v>503</v>
       </c>
       <c r="D146" s="6"/>
       <c r="E146" s="6"/>
@@ -5968,13 +5975,13 @@
     </row>
     <row r="147" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A147" s="4" t="s">
-        <v>493</v>
+        <v>504</v>
       </c>
       <c r="B147" s="5" t="s">
-        <v>494</v>
+        <v>505</v>
       </c>
       <c r="C147" s="5" t="s">
-        <v>495</v>
+        <v>506</v>
       </c>
       <c r="D147" s="6"/>
       <c r="E147" s="6"/>
@@ -5990,13 +5997,13 @@
     </row>
     <row r="148" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A148" s="4" t="s">
-        <v>496</v>
+        <v>507</v>
       </c>
       <c r="B148" s="5" t="s">
-        <v>497</v>
+        <v>508</v>
       </c>
       <c r="C148" s="5" t="s">
-        <v>498</v>
+        <v>509</v>
       </c>
       <c r="D148" s="6"/>
       <c r="E148" s="6"/>
@@ -6012,13 +6019,13 @@
     </row>
     <row r="149" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A149" s="4" t="s">
-        <v>499</v>
+        <v>510</v>
       </c>
       <c r="B149" s="5" t="s">
-        <v>500</v>
+        <v>511</v>
       </c>
       <c r="C149" s="5" t="s">
-        <v>501</v>
+        <v>512</v>
       </c>
       <c r="D149" s="6"/>
       <c r="E149" s="6"/>
@@ -6034,13 +6041,13 @@
     </row>
     <row r="150" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A150" s="4" t="s">
-        <v>502</v>
+        <v>513</v>
       </c>
       <c r="B150" s="5" t="s">
-        <v>503</v>
+        <v>514</v>
       </c>
       <c r="C150" s="5" t="s">
-        <v>504</v>
+        <v>515</v>
       </c>
       <c r="D150" s="6"/>
       <c r="E150" s="6"/>
@@ -6056,13 +6063,13 @@
     </row>
     <row r="151" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A151" s="4" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="B151" s="5" t="s">
-        <v>506</v>
+        <v>517</v>
       </c>
       <c r="C151" s="5" t="s">
-        <v>507</v>
+        <v>518</v>
       </c>
       <c r="D151" s="6"/>
       <c r="E151" s="6"/>
@@ -6078,19 +6085,19 @@
     </row>
     <row r="152" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A152" s="4" t="s">
-        <v>508</v>
+        <v>519</v>
       </c>
       <c r="B152" s="5" t="s">
-        <v>509</v>
+        <v>520</v>
       </c>
       <c r="C152" s="5" t="s">
-        <v>510</v>
+        <v>521</v>
       </c>
       <c r="D152" s="6"/>
       <c r="E152" s="6"/>
       <c r="F152" s="6"/>
       <c r="G152" s="6" t="s">
-        <v>511</v>
+        <v>522</v>
       </c>
       <c r="H152" s="6"/>
       <c r="I152" s="6"/>
@@ -6102,13 +6109,13 @@
     </row>
     <row r="153" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A153" s="4" t="s">
-        <v>512</v>
+        <v>523</v>
       </c>
       <c r="B153" s="5" t="s">
-        <v>513</v>
+        <v>524</v>
       </c>
       <c r="C153" s="5" t="s">
-        <v>514</v>
+        <v>525</v>
       </c>
       <c r="D153" s="6"/>
       <c r="E153" s="6"/>
@@ -6124,13 +6131,13 @@
     </row>
     <row r="154" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A154" s="4" t="s">
-        <v>515</v>
+        <v>526</v>
       </c>
       <c r="B154" s="5" t="s">
-        <v>516</v>
+        <v>527</v>
       </c>
       <c r="C154" s="5" t="s">
-        <v>517</v>
+        <v>528</v>
       </c>
       <c r="D154" s="6"/>
       <c r="E154" s="6"/>
@@ -6146,13 +6153,13 @@
     </row>
     <row r="155" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A155" s="4" t="s">
-        <v>518</v>
+        <v>529</v>
       </c>
       <c r="B155" s="5" t="s">
-        <v>519</v>
+        <v>530</v>
       </c>
       <c r="C155" s="5" t="s">
-        <v>520</v>
+        <v>531</v>
       </c>
       <c r="D155" s="6"/>
       <c r="E155" s="6"/>
@@ -6168,13 +6175,13 @@
     </row>
     <row r="156" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A156" s="4" t="s">
-        <v>521</v>
+        <v>532</v>
       </c>
       <c r="B156" s="5" t="s">
-        <v>522</v>
+        <v>533</v>
       </c>
       <c r="C156" s="5" t="s">
-        <v>523</v>
+        <v>534</v>
       </c>
       <c r="D156" s="6"/>
       <c r="E156" s="6"/>
@@ -6190,13 +6197,13 @@
     </row>
     <row r="157" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A157" s="4" t="s">
-        <v>524</v>
+        <v>535</v>
       </c>
       <c r="B157" s="5" t="s">
-        <v>525</v>
+        <v>536</v>
       </c>
       <c r="C157" s="5" t="s">
-        <v>526</v>
+        <v>537</v>
       </c>
       <c r="D157" s="6"/>
       <c r="E157" s="6"/>
@@ -6212,13 +6219,13 @@
     </row>
     <row r="158" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A158" s="4" t="s">
-        <v>527</v>
+        <v>538</v>
       </c>
       <c r="B158" s="5" t="s">
-        <v>528</v>
+        <v>539</v>
       </c>
       <c r="C158" s="5" t="s">
-        <v>529</v>
+        <v>540</v>
       </c>
       <c r="D158" s="6"/>
       <c r="E158" s="6"/>
@@ -6234,13 +6241,13 @@
     </row>
     <row r="159" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A159" s="4" t="s">
-        <v>530</v>
+        <v>541</v>
       </c>
       <c r="B159" s="5" t="s">
-        <v>531</v>
+        <v>542</v>
       </c>
       <c r="C159" s="5" t="s">
-        <v>532</v>
+        <v>543</v>
       </c>
       <c r="D159" s="6"/>
       <c r="E159" s="6"/>
@@ -6256,13 +6263,13 @@
     </row>
     <row r="160" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A160" s="4" t="s">
-        <v>533</v>
+        <v>544</v>
       </c>
       <c r="B160" s="5" t="s">
-        <v>534</v>
+        <v>545</v>
       </c>
       <c r="C160" s="5" t="s">
-        <v>535</v>
+        <v>546</v>
       </c>
       <c r="D160" s="6"/>
       <c r="E160" s="6"/>
@@ -6278,13 +6285,13 @@
     </row>
     <row r="161" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A161" s="4" t="s">
-        <v>536</v>
+        <v>547</v>
       </c>
       <c r="B161" s="5" t="s">
-        <v>537</v>
+        <v>548</v>
       </c>
       <c r="C161" s="5" t="s">
-        <v>538</v>
+        <v>549</v>
       </c>
       <c r="D161" s="6"/>
       <c r="E161" s="6"/>
@@ -6300,19 +6307,19 @@
     </row>
     <row r="162" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A162" s="4" t="s">
-        <v>539</v>
+        <v>550</v>
       </c>
       <c r="B162" s="5" t="s">
-        <v>540</v>
+        <v>551</v>
       </c>
       <c r="C162" s="5" t="s">
-        <v>541</v>
+        <v>552</v>
       </c>
       <c r="D162" s="6"/>
       <c r="E162" s="6"/>
       <c r="F162" s="6"/>
       <c r="G162" s="6" t="s">
-        <v>542</v>
+        <v>553</v>
       </c>
       <c r="H162" s="6"/>
       <c r="I162" s="6"/>
@@ -6324,13 +6331,13 @@
     </row>
     <row r="163" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A163" s="4" t="s">
-        <v>543</v>
+        <v>554</v>
       </c>
       <c r="B163" s="5" t="s">
-        <v>544</v>
+        <v>555</v>
       </c>
       <c r="C163" s="5" t="s">
-        <v>545</v>
+        <v>556</v>
       </c>
       <c r="D163" s="6"/>
       <c r="E163" s="6"/>
@@ -6346,13 +6353,13 @@
     </row>
     <row r="164" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A164" s="4" t="s">
-        <v>546</v>
+        <v>557</v>
       </c>
       <c r="B164" s="5" t="s">
-        <v>547</v>
+        <v>558</v>
       </c>
       <c r="C164" s="5" t="s">
-        <v>548</v>
+        <v>559</v>
       </c>
       <c r="D164" s="6"/>
       <c r="E164" s="6"/>
@@ -6368,13 +6375,13 @@
     </row>
     <row r="165" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A165" s="4" t="s">
-        <v>549</v>
+        <v>560</v>
       </c>
       <c r="B165" s="5" t="s">
-        <v>550</v>
+        <v>561</v>
       </c>
       <c r="C165" s="5" t="s">
-        <v>551</v>
+        <v>562</v>
       </c>
       <c r="D165" s="6"/>
       <c r="E165" s="6"/>
@@ -6390,13 +6397,13 @@
     </row>
     <row r="166" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A166" s="4" t="s">
-        <v>552</v>
+        <v>563</v>
       </c>
       <c r="B166" s="5" t="s">
-        <v>553</v>
+        <v>564</v>
       </c>
       <c r="C166" s="5" t="s">
-        <v>554</v>
+        <v>565</v>
       </c>
       <c r="D166" s="6"/>
       <c r="E166" s="6"/>
@@ -6412,13 +6419,13 @@
     </row>
     <row r="167" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A167" s="4" t="s">
-        <v>555</v>
+        <v>566</v>
       </c>
       <c r="B167" s="5" t="s">
-        <v>556</v>
+        <v>567</v>
       </c>
       <c r="C167" s="5" t="s">
-        <v>557</v>
+        <v>568</v>
       </c>
       <c r="D167" s="6"/>
       <c r="E167" s="6"/>
@@ -6437,10 +6444,10 @@
     <row r="168" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A168" s="5"/>
       <c r="B168" s="5" t="s">
-        <v>558</v>
+        <v>569</v>
       </c>
       <c r="C168" s="5" t="s">
-        <v>559</v>
+        <v>570</v>
       </c>
       <c r="D168" s="6"/>
       <c r="E168" s="6"/>
@@ -6455,10 +6462,10 @@
     <row r="169" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A169" s="5"/>
       <c r="B169" s="5" t="s">
-        <v>560</v>
+        <v>571</v>
       </c>
       <c r="C169" s="5" t="s">
-        <v>561</v>
+        <v>572</v>
       </c>
       <c r="D169" s="6"/>
       <c r="E169" s="6"/>
@@ -6473,10 +6480,10 @@
     <row r="170" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A170" s="5"/>
       <c r="B170" s="5" t="s">
-        <v>562</v>
+        <v>573</v>
       </c>
       <c r="C170" s="5" t="s">
-        <v>563</v>
+        <v>574</v>
       </c>
       <c r="D170" s="6"/>
       <c r="E170" s="6"/>
@@ -6491,10 +6498,10 @@
     <row r="171" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A171" s="5"/>
       <c r="B171" s="5" t="s">
-        <v>564</v>
+        <v>575</v>
       </c>
       <c r="C171" s="5" t="s">
-        <v>565</v>
+        <v>576</v>
       </c>
       <c r="D171" s="6"/>
       <c r="E171" s="6"/>
@@ -6509,10 +6516,10 @@
     <row r="172" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A172" s="5"/>
       <c r="B172" s="5" t="s">
-        <v>566</v>
+        <v>577</v>
       </c>
       <c r="C172" s="5" t="s">
-        <v>567</v>
+        <v>578</v>
       </c>
       <c r="D172" s="6"/>
       <c r="E172" s="6"/>
@@ -6527,16 +6534,16 @@
     <row r="173" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A173" s="5"/>
       <c r="B173" s="5" t="s">
-        <v>568</v>
+        <v>579</v>
       </c>
       <c r="C173" s="5" t="s">
-        <v>569</v>
+        <v>580</v>
       </c>
       <c r="D173" s="6"/>
       <c r="E173" s="6"/>
       <c r="F173" s="6"/>
       <c r="G173" s="6" t="s">
-        <v>570</v>
+        <v>581</v>
       </c>
       <c r="H173" s="6"/>
       <c r="I173" s="6"/>
@@ -6547,10 +6554,10 @@
     <row r="174" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A174" s="5"/>
       <c r="B174" s="5" t="s">
-        <v>571</v>
+        <v>582</v>
       </c>
       <c r="C174" s="5" t="s">
-        <v>572</v>
+        <v>583</v>
       </c>
       <c r="D174" s="6"/>
       <c r="E174" s="6"/>
@@ -6565,10 +6572,10 @@
     <row r="175" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A175" s="5"/>
       <c r="B175" s="5" t="s">
-        <v>573</v>
+        <v>584</v>
       </c>
       <c r="C175" s="5" t="s">
-        <v>574</v>
+        <v>585</v>
       </c>
       <c r="D175" s="6"/>
       <c r="E175" s="6"/>
@@ -6583,10 +6590,10 @@
     <row r="176" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A176" s="5"/>
       <c r="B176" s="5" t="s">
-        <v>575</v>
+        <v>586</v>
       </c>
       <c r="C176" s="5" t="s">
-        <v>576</v>
+        <v>587</v>
       </c>
       <c r="D176" s="6"/>
       <c r="E176" s="6"/>
@@ -6601,10 +6608,10 @@
     <row r="177" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A177" s="5"/>
       <c r="B177" s="5" t="s">
-        <v>577</v>
+        <v>588</v>
       </c>
       <c r="C177" s="5" t="s">
-        <v>578</v>
+        <v>589</v>
       </c>
       <c r="D177" s="6"/>
       <c r="E177" s="6"/>
@@ -6619,10 +6626,10 @@
     <row r="178" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A178" s="5"/>
       <c r="B178" s="5" t="s">
-        <v>579</v>
+        <v>590</v>
       </c>
       <c r="C178" s="5" t="s">
-        <v>580</v>
+        <v>591</v>
       </c>
       <c r="D178" s="6"/>
       <c r="E178" s="6"/>
@@ -6637,10 +6644,10 @@
     <row r="179" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A179" s="5"/>
       <c r="B179" s="5" t="s">
-        <v>581</v>
+        <v>592</v>
       </c>
       <c r="C179" s="5" t="s">
-        <v>582</v>
+        <v>593</v>
       </c>
       <c r="D179" s="6"/>
       <c r="E179" s="6"/>
@@ -6655,10 +6662,10 @@
     <row r="180" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A180" s="5"/>
       <c r="B180" s="5" t="s">
-        <v>583</v>
+        <v>594</v>
       </c>
       <c r="C180" s="5" t="s">
-        <v>584</v>
+        <v>595</v>
       </c>
       <c r="D180" s="6"/>
       <c r="E180" s="6"/>
@@ -6673,10 +6680,10 @@
     <row r="181" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A181" s="5"/>
       <c r="B181" s="5" t="s">
-        <v>585</v>
+        <v>596</v>
       </c>
       <c r="C181" s="5" t="s">
-        <v>586</v>
+        <v>597</v>
       </c>
       <c r="D181" s="6"/>
       <c r="E181" s="6"/>
@@ -6691,10 +6698,10 @@
     <row r="182" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A182" s="5"/>
       <c r="B182" s="5" t="s">
-        <v>587</v>
+        <v>598</v>
       </c>
       <c r="C182" s="5" t="s">
-        <v>588</v>
+        <v>599</v>
       </c>
       <c r="D182" s="6"/>
       <c r="E182" s="6"/>
@@ -6709,10 +6716,10 @@
     <row r="183" spans="1:12" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A183" s="5"/>
       <c r="B183" s="5" t="s">
-        <v>589</v>
+        <v>600</v>
       </c>
       <c r="C183" s="5" t="s">
-        <v>590</v>
+        <v>601</v>
       </c>
       <c r="D183" s="6"/>
       <c r="E183" s="6"/>
@@ -18374,13 +18381,13 @@
     </row>
     <row r="1016" spans="1:12" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1016" s="5" t="s">
-        <v>596</v>
+        <v>602</v>
       </c>
       <c r="B1016" s="5" t="s">
-        <v>597</v>
+        <v>603</v>
       </c>
       <c r="C1016" s="5" t="s">
-        <v>598</v>
+        <v>604</v>
       </c>
       <c r="D1016" s="6"/>
       <c r="E1016" s="6"/>
@@ -18389,24 +18396,24 @@
       <c r="H1016" s="6"/>
       <c r="I1016" s="6"/>
       <c r="J1016" s="6" t="s">
-        <v>599</v>
+        <v>605</v>
       </c>
       <c r="K1016" s="6" t="s">
-        <v>600</v>
+        <v>606</v>
       </c>
       <c r="L1016" s="6" t="s">
-        <v>601</v>
+        <v>607</v>
       </c>
     </row>
     <row r="1017" spans="1:12" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1017" s="5" t="s">
-        <v>602</v>
+        <v>608</v>
       </c>
       <c r="B1017" s="5" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="C1017" s="5" t="s">
-        <v>604</v>
+        <v>610</v>
       </c>
       <c r="D1017" s="6"/>
       <c r="E1017" s="6"/>
@@ -18415,13 +18422,13 @@
       <c r="H1017" s="6"/>
       <c r="I1017" s="6"/>
       <c r="J1017" s="6" t="s">
-        <v>599</v>
+        <v>605</v>
       </c>
       <c r="K1017" s="6" t="s">
-        <v>600</v>
+        <v>606</v>
       </c>
       <c r="L1017" s="6" t="s">
-        <v>601</v>
+        <v>607</v>
       </c>
     </row>
   </sheetData>
@@ -18432,7 +18439,7 @@
     <dataValidation type="list" allowBlank="1" sqref="Q2:Q16" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"1,2,3,4,5"</formula1>
     </dataValidation>
-    <dataValidation allowBlank="1" showDropDown="1" sqref="N2:N16 A2:C1017" xr:uid="{00000000-0002-0000-0000-000002000000}"/>
+    <dataValidation allowBlank="1" showDropDown="1" sqref="A2:C1017 N2:N16" xr:uid="{00000000-0002-0000-0000-000002000000}"/>
     <dataValidation type="list" allowBlank="1" sqref="L2:L1017" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>"Implemented,New,In progress,To Be Reworked,Buggy,Needs Testing"</formula1>
     </dataValidation>

</xml_diff>

<commit_message>
Close Soviet collapse active source audit
</commit_message>
<xml_diff>
--- a/docs/spreadsheets/chaos_redux_events_catalog.xlsx
+++ b/docs/spreadsheets/chaos_redux_events_catalog.xlsx
@@ -2587,7 +2587,7 @@
       </c>
       <c r="L6" s="6" t="inlineStr">
         <is>
-          <t>Implemented - Final Closure Blocked</t>
+          <t>Implemented - Verified</t>
         </is>
       </c>
       <c r="N6" s="7" t="s">
@@ -2604,7 +2604,7 @@
       </c>
       <c r="R6" s="8" t="inlineStr">
         <is>
-          <t>Blocked - Missing continuation spec</t>
+          <t>Complete</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Restore chaos catalog table styling
</commit_message>
<xml_diff>
--- a/docs/spreadsheets/chaos_redux_events_catalog.xlsx
+++ b/docs/spreadsheets/chaos_redux_events_catalog.xlsx
@@ -2321,7 +2321,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="17">
+  <dxfs count="25">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -2457,7 +2457,101 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF6F8F9"/>
+          <bgColor rgb="FFF6F8F9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFFF"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF5B3F86"/>
+          <bgColor rgb="FF5B3F86"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color rgb="FF9B3642"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF9B3642"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF9B3642"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF9B3642"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF6F8F9"/>
+          <bgColor rgb="FFF6F8F9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFFF"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF9B3642"/>
+          <bgColor rgb="FF9B3642"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color rgb="FF9B3642"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF9B3642"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF9B3642"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF9B3642"/>
+        </bottom>
+      </border>
+    </dxf>
   </dxfs>
+  <tableStyles count="2" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16">
+    <tableStyle name="Main Sheet-style" pivot="0" count="4">
+      <tableStyleElement type="wholeTable" dxfId="24" size="0"/>
+      <tableStyleElement type="headerRow" dxfId="23"/>
+      <tableStyleElement type="firstRowStripe" dxfId="22"/>
+      <tableStyleElement type="secondRowStripe" dxfId="21"/>
+    </tableStyle>
+    <tableStyle name="Main Sheet-style 2" pivot="0" count="4">
+      <tableStyleElement type="wholeTable" dxfId="20" size="0"/>
+      <tableStyleElement type="headerRow" dxfId="19"/>
+      <tableStyleElement type="firstRowStripe" dxfId="18"/>
+      <tableStyleElement type="secondRowStripe" dxfId="17"/>
+    </tableStyle>
+  </tableStyles>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -2533,6 +2627,7 @@
     <tableColumn id="7" name="Chaos level"/>
     <tableColumn id="8" name="Status"/>
   </tableColumns>
+  <tableStyleInfo name="Main Sheet-style 2" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -2553,6 +2648,7 @@
     <tableColumn id="12" name="Severity"/>
     <tableColumn id="13" name="Status"/>
   </tableColumns>
+  <tableStyleInfo name="Main Sheet-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 

</xml_diff>

<commit_message>
Remove cluster ID cell coloring from catalog
</commit_message>
<xml_diff>
--- a/docs/spreadsheets/chaos_redux_events_catalog.xlsx
+++ b/docs/spreadsheets/chaos_redux_events_catalog.xlsx
@@ -2825,7 +2825,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr filterMode="false">
     <tabColor rgb="FF1C4587"/>
     <pageSetUpPr fitToPage="false"/>
@@ -3103,7 +3103,7 @@
       <c r="J5" s="19" t="s">
         <v>57</v>
       </c>
-      <c r="K5" s="20" t="s">
+      <c r="K5" s="2" t="s">
         <v>16</v>
       </c>
       <c r="L5" s="12" t="s">
@@ -3112,7 +3112,7 @@
       <c r="M5" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="O5" s="21" t="s">
+      <c r="O5" s="2" t="s">
         <v>16</v>
       </c>
       <c r="P5" s="14" t="s">
@@ -3166,7 +3166,7 @@
       <c r="J6" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="K6" s="20" t="s">
+      <c r="K6" s="2" t="s">
         <v>29</v>
       </c>
       <c r="L6" s="23" t="s">
@@ -3175,7 +3175,7 @@
       <c r="M6" s="24" t="s">
         <v>60</v>
       </c>
-      <c r="O6" s="21" t="s">
+      <c r="O6" s="2" t="s">
         <v>29</v>
       </c>
       <c r="P6" s="14" t="s">
@@ -3229,7 +3229,7 @@
       <c r="J7" s="19" t="s">
         <v>57</v>
       </c>
-      <c r="K7" s="20" t="s">
+      <c r="K7" s="2" t="s">
         <v>29</v>
       </c>
       <c r="L7" s="12" t="s">
@@ -18129,8 +18129,8 @@
     <oddFooter/>
   </headerFooter>
   <tableParts>
-    <tablePart r:id="rId1"/>
-    <tablePart r:id="rId2"/>
+    <tablePart ns1:id="rId1"/>
+    <tablePart ns1:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Fix chaos catalog data validations
</commit_message>
<xml_diff>
--- a/docs/spreadsheets/chaos_redux_events_catalog.xlsx
+++ b/docs/spreadsheets/chaos_redux_events_catalog.xlsx
@@ -18099,26 +18099,27 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="5">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J2:K1017" type="list">
-      <formula1>"Minor Repeatable,Minor Fire-Once,Major"</formula1>
-      <formula2>0</formula2>
+  <dataValidations count="7">
+    <dataValidation type="list" allowBlank="1" sqref="J2:J1017">
+      <formula1>"Minor Repeatable,Minor Fire-Once,Major,Manual Scenario"</formula1>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="P2:P16" type="list">
+    <dataValidation type="list" allowBlank="1" sqref="L2:L1017">
+      <formula1>"Low,Medium,High,Severe"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="M2:M1017">
+      <formula1>"Implemented,New,In progress,To Be Reworked,Buggy,Needs Testing"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="S2:S14">
+      <formula1>"Minor Repeatable,Minor Fire-Once,Major,Manual Scenario"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="T2:T14">
+      <formula1>"Low,Medium,High,Severe"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="U2:U14">
       <formula1>"1,2,3,4,5"</formula1>
-      <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="true" showErrorMessage="false" showInputMessage="false" sqref="A2:C1017 M2:M16" type="none">
-      <formula1>0</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="L2:L1017" type="list">
-      <formula1>"Implemented,New,In progress,To Be Reworked,Buggy,Needs Testing"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="Q2:Q16" type="list">
+    <dataValidation type="list" allowBlank="1" sqref="V2:V14">
       <formula1>"Implemented,New,In progress,Under review,Buggy"</formula1>
-      <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Add manual scenarios catalog table
</commit_message>
<xml_diff>
--- a/docs/spreadsheets/chaos_redux_events_catalog.xlsx
+++ b/docs/spreadsheets/chaos_redux_events_catalog.xlsx
@@ -2632,7 +2632,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Events" displayName="Events" ref="A1:M1017" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Events" displayName="Events" ref="A1:M1015" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <tableColumns count="13">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Event Name"/>
@@ -2649,6 +2649,22 @@
     <tableColumn id="13" name="Status"/>
   </tableColumns>
   <tableStyleInfo name="Main Sheet-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Manual_Scenarios" displayName="Manual_Scenarios" ref="W1:AD5" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <tableColumns count="8">
+    <tableColumn id="1" name="Scenario ID"/>
+    <tableColumn id="2" name="Scenario Name"/>
+    <tableColumn id="3" name="Details"/>
+    <tableColumn id="4" name="Source Event"/>
+    <tableColumn id="5" name="Type Options"/>
+    <tableColumn id="6" name="Intensity Scaling"/>
+    <tableColumn id="7" name="Launch Gate"/>
+    <tableColumn id="8" name="Status"/>
+  </tableColumns>
+  <tableStyleInfo name="Main Sheet-style 2" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -2825,12 +2841,12 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr filterMode="false">
     <tabColor rgb="FF1C4587"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:V1017"/>
+  <dimension ref="A1:AD1015"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7.15"/>
@@ -2854,6 +2870,14 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="0" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="0" width="18"/>
+    <col min="23" max="23" width="12" customWidth="1"/>
+    <col min="24" max="24" width="24" customWidth="1"/>
+    <col min="25" max="25" width="68" customWidth="1"/>
+    <col min="26" max="26" width="24" customWidth="1"/>
+    <col min="27" max="27" width="46" customWidth="1"/>
+    <col min="28" max="28" width="52" customWidth="1"/>
+    <col min="29" max="29" width="44" customWidth="1"/>
+    <col min="30" max="30" width="16" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2920,6 +2944,46 @@
       <c r="V1" s="3" t="s">
         <v>12</v>
       </c>
+      <c r="W1" s="3" t="inlineStr">
+        <is>
+          <t>Scenario ID</t>
+        </is>
+      </c>
+      <c r="X1" s="3" t="inlineStr">
+        <is>
+          <t>Scenario Name</t>
+        </is>
+      </c>
+      <c r="Y1" s="3" t="inlineStr">
+        <is>
+          <t>Details</t>
+        </is>
+      </c>
+      <c r="Z1" s="3" t="inlineStr">
+        <is>
+          <t>Source Event</t>
+        </is>
+      </c>
+      <c r="AA1" s="3" t="inlineStr">
+        <is>
+          <t>Type Options</t>
+        </is>
+      </c>
+      <c r="AB1" s="3" t="inlineStr">
+        <is>
+          <t>Intensity Scaling</t>
+        </is>
+      </c>
+      <c r="AC1" s="3" t="inlineStr">
+        <is>
+          <t>Launch Gate</t>
+        </is>
+      </c>
+      <c r="AD1" s="3" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="99.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
@@ -2971,6 +3035,46 @@
       <c r="V2" s="17" t="s">
         <v>28</v>
       </c>
+      <c r="W2" s="14" t="inlineStr">
+        <is>
+          <t>SCN-001</t>
+        </is>
+      </c>
+      <c r="X2" s="14" t="inlineStr">
+        <is>
+          <t>Zombie Apocalypse</t>
+        </is>
+      </c>
+      <c r="Y2" s="14" t="inlineStr">
+        <is>
+          <t>Manual setup launched from the Chaos Redux scenario window. Creates hostile zombie outbreaks from selected outbreak profile and structure.</t>
+        </is>
+      </c>
+      <c r="Z2" s="14" t="inlineStr">
+        <is>
+          <t>Event 002 Zombie Outbreak</t>
+        </is>
+      </c>
+      <c r="AA2" s="14" t="inlineStr">
+        <is>
+          <t>Diverse, Random, Standard, Rabid, Parasitic, Mutant, Undead, Necrotic, Demonic, Wendigo, Connected</t>
+        </is>
+      </c>
+      <c r="AB2" s="14" t="inlineStr">
+        <is>
+          <t>Low/Medium/High/Maximum controls outbreak count, starting states, spawned divisions, and early pressure.</t>
+        </is>
+      </c>
+      <c r="AC2" s="14" t="inlineStr">
+        <is>
+          <t>Available unless the launch is impossible or conflicts with an active terminal state.</t>
+        </is>
+      </c>
+      <c r="AD2" s="19" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="111.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
@@ -3020,6 +3124,46 @@
       <c r="V3" s="17" t="s">
         <v>28</v>
       </c>
+      <c r="W3" s="14" t="inlineStr">
+        <is>
+          <t>SCN-002</t>
+        </is>
+      </c>
+      <c r="X3" s="14" t="inlineStr">
+        <is>
+          <t>Army of Clones</t>
+        </is>
+      </c>
+      <c r="Y3" s="14" t="inlineStr">
+        <is>
+          <t>Manual setup launched from the Chaos Redux scenario window. Creates a hostile artificial army in Eastern Europe and the western Soviet borderlands.</t>
+        </is>
+      </c>
+      <c r="Z3" s="14" t="inlineStr">
+        <is>
+          <t>Mengele Clone Army scenario</t>
+        </is>
+      </c>
+      <c r="AA3" s="14" t="inlineStr">
+        <is>
+          <t>Standard clone army or stronger Aryan variant</t>
+        </is>
+      </c>
+      <c r="AB3" s="14" t="inlineStr">
+        <is>
+          <t>Low/Medium/High/Maximum controls starting territory, divisions, army experience, equipment stockpiles, and pressure on neighboring countries.</t>
+        </is>
+      </c>
+      <c r="AC3" s="14" t="inlineStr">
+        <is>
+          <t>Available unless the launch is impossible or conflicts with an active terminal state.</t>
+        </is>
+      </c>
+      <c r="AD3" s="19" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
@@ -3073,6 +3217,46 @@
       <c r="V4" s="17" t="s">
         <v>28</v>
       </c>
+      <c r="W4" s="14" t="inlineStr">
+        <is>
+          <t>SCN-003</t>
+        </is>
+      </c>
+      <c r="X4" s="14" t="inlineStr">
+        <is>
+          <t>Soviet Collapse</t>
+        </is>
+      </c>
+      <c r="Y4" s="14" t="inlineStr">
+        <is>
+          <t>Manual setup launched from the Chaos Redux scenario window. Forces the Event 005 Union Unmade terminal collapse immediately and releases the Soviet breakaways.</t>
+        </is>
+      </c>
+      <c r="Z4" s="14" t="inlineStr">
+        <is>
+          <t>Event 005 Soviet Collapse</t>
+        </is>
+      </c>
+      <c r="AA4" s="14" t="inlineStr">
+        <is>
+          <t>Ordinary republics or chaos republics</t>
+        </is>
+      </c>
+      <c r="AB4" s="14" t="inlineStr">
+        <is>
+          <t>Low/Medium/High/Maximum adds scaled extra breakaway armies, manpower, infantry equipment, support equipment, artillery, and motorized equipment.</t>
+        </is>
+      </c>
+      <c r="AC4" s="14" t="inlineStr">
+        <is>
+          <t>Requires a valid Soviet collapse launch state; bypasses normal chaos, evolution, and prior-super-event gates during setup.</t>
+        </is>
+      </c>
+      <c r="AD4" s="19" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
@@ -3135,6 +3319,46 @@
       </c>
       <c r="V5" s="22" t="s">
         <v>60</v>
+      </c>
+      <c r="W5" s="14" t="inlineStr">
+        <is>
+          <t>SCN-004</t>
+        </is>
+      </c>
+      <c r="X5" s="14" t="inlineStr">
+        <is>
+          <t>Final Silence</t>
+        </is>
+      </c>
+      <c r="Y5" s="14" t="inlineStr">
+        <is>
+          <t>Manual setup launched from the Chaos Redux scenario window. Starts the Holy Realm Final Silence world-end sequence from the current player country.</t>
+        </is>
+      </c>
+      <c r="Z5" s="14" t="inlineStr">
+        <is>
+          <t>Event 003 The Holy Realm</t>
+        </is>
+      </c>
+      <c r="AA5" s="14" t="inlineStr">
+        <is>
+          <t>Nuclear or thermonuclear payload</t>
+        </is>
+      </c>
+      <c r="AB5" s="14" t="inlineStr">
+        <is>
+          <t>Intensity is fixed; the scenario keeps the canonical four-wave Final Silence sequence.</t>
+        </is>
+      </c>
+      <c r="AC5" s="14" t="inlineStr">
+        <is>
+          <t>Blocked if another terminal world-end is already active or the launch is otherwise impossible.</t>
+        </is>
+      </c>
+      <c r="AD5" s="19" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
       </c>
     </row>
     <row r="6" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18048,65 +18272,15 @@
       <c r="J1015" s="29"/>
       <c r="M1015" s="29"/>
     </row>
-    <row r="1016" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1016" s="31" t="s">
-        <v>614</v>
-      </c>
-      <c r="B1016" s="5" t="s">
-        <v>615</v>
-      </c>
-      <c r="C1016" s="5" t="s">
-        <v>616</v>
-      </c>
-      <c r="D1016" s="6"/>
-      <c r="E1016" s="7"/>
-      <c r="F1016" s="8"/>
-      <c r="G1016" s="9"/>
-      <c r="H1016" s="10"/>
-      <c r="I1016" s="11" t="s">
-        <v>617</v>
-      </c>
-      <c r="J1016" s="20" t="s">
-        <v>618</v>
-      </c>
-      <c r="M1016" s="19" t="s">
-        <v>619</v>
-      </c>
-    </row>
-    <row r="1017" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1017" s="31" t="s">
-        <v>620</v>
-      </c>
-      <c r="B1017" s="5" t="s">
-        <v>621</v>
-      </c>
-      <c r="C1017" s="5" t="s">
-        <v>622</v>
-      </c>
-      <c r="D1017" s="6"/>
-      <c r="E1017" s="7"/>
-      <c r="F1017" s="8"/>
-      <c r="G1017" s="9"/>
-      <c r="H1017" s="10"/>
-      <c r="I1017" s="11" t="s">
-        <v>617</v>
-      </c>
-      <c r="J1017" s="20" t="s">
-        <v>618</v>
-      </c>
-      <c r="M1017" s="19" t="s">
-        <v>619</v>
-      </c>
-    </row>
   </sheetData>
-  <dataValidations count="7">
-    <dataValidation type="list" allowBlank="1" sqref="J2:J1017">
+  <dataValidations count="8">
+    <dataValidation type="list" allowBlank="1" sqref="J2:J1015">
       <formula1>"Minor Repeatable,Minor Fire-Once,Major,Manual Scenario"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="L2:L1017">
+    <dataValidation type="list" allowBlank="1" sqref="L2:L1015">
       <formula1>"Low,Medium,High,Severe"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="M2:M1017">
+    <dataValidation type="list" allowBlank="1" sqref="M2:M1015">
       <formula1>"Implemented,New,In progress,To Be Reworked,Buggy,Needs Testing"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="S2:S14">
@@ -18121,6 +18295,9 @@
     <dataValidation type="list" allowBlank="1" sqref="V2:V14">
       <formula1>"Implemented,New,In progress,Under review,Buggy"</formula1>
     </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="AD2:AD5">
+      <formula1>"Implemented,New,In progress,To Be Reworked,Buggy,Needs Testing"</formula1>
+    </dataValidation>
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
@@ -18129,9 +18306,10 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <tableParts>
-    <tablePart ns1:id="rId1"/>
-    <tablePart ns1:id="rId2"/>
+  <tableParts count="3">
+    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Adjust catalog cluster table layout
</commit_message>
<xml_diff>
--- a/docs/spreadsheets/chaos_redux_events_catalog.xlsx
+++ b/docs/spreadsheets/chaos_redux_events_catalog.xlsx
@@ -2047,7 +2047,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="17">
+  <fills count="22">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2144,6 +2144,36 @@
         <bgColor rgb="FFF4CCCC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFE5E5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCCCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFB3B3"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF9999"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF8080"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border diagonalUp="false" diagonalDown="false">
@@ -2179,7 +2209,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="38">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2310,6 +2340,26 @@
     </xf>
     <xf numFmtId="164" fontId="5" fillId="13" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="17" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false" applyFill="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="18" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false" applyFill="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="19" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false" applyFill="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="20" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false" applyFill="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="21" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false" applyFill="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -2616,16 +2666,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Event_Clusters" displayName="Event_Clusters" ref="O1:V14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <tableColumns count="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Event_Clusters" displayName="Event_Clusters" ref="O1:U14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <tableColumns count="7">
     <tableColumn id="1" name="Cluster ID"/>
     <tableColumn id="2" name="Cluster Name"/>
     <tableColumn id="3" name="Details"/>
     <tableColumn id="4" name="Events (ID)"/>
     <tableColumn id="5" name="Type"/>
-    <tableColumn id="6" name="Severity"/>
-    <tableColumn id="7" name="Chaos level"/>
-    <tableColumn id="8" name="Status"/>
+    <tableColumn id="6" name="Chaos level"/>
+    <tableColumn id="7" name="Status"/>
   </tableColumns>
   <tableStyleInfo name="Main Sheet-style 2" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2936,12 +2985,9 @@
         <v>9</v>
       </c>
       <c r="T1" s="3" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="U1" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="V1" s="3" t="s">
         <v>12</v>
       </c>
       <c r="W1" s="3" t="inlineStr">
@@ -3015,7 +3061,7 @@
       <c r="M2" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="O2" s="14"/>
+      <c r="O2" s="4"/>
       <c r="P2" s="14" t="s">
         <v>25</v>
       </c>
@@ -3026,13 +3072,10 @@
       <c r="S2" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="T2" s="16" t="s">
-        <v>27</v>
-      </c>
-      <c r="U2" s="14" t="s">
+      <c r="T2" s="33" t="s">
         <v>16</v>
       </c>
-      <c r="V2" s="17" t="s">
+      <c r="U2" s="17" t="s">
         <v>28</v>
       </c>
       <c r="W2" s="14" t="inlineStr">
@@ -3106,7 +3149,7 @@
       <c r="M3" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="O3" s="14"/>
+      <c r="O3" s="4"/>
       <c r="P3" s="14" t="s">
         <v>37</v>
       </c>
@@ -3115,13 +3158,10 @@
       <c r="S3" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="T3" s="16" t="s">
-        <v>27</v>
-      </c>
-      <c r="U3" s="14" t="s">
+      <c r="T3" s="33" t="s">
         <v>16</v>
       </c>
-      <c r="V3" s="17" t="s">
+      <c r="U3" s="17" t="s">
         <v>28</v>
       </c>
       <c r="W3" s="14" t="inlineStr">
@@ -3199,7 +3239,7 @@
       <c r="M4" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="O4" s="14"/>
+      <c r="O4" s="4"/>
       <c r="P4" s="14" t="s">
         <v>47</v>
       </c>
@@ -3208,13 +3248,10 @@
       <c r="S4" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="T4" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="U4" s="14" t="s">
+      <c r="T4" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="V4" s="17" t="s">
+      <c r="U4" s="17" t="s">
         <v>28</v>
       </c>
       <c r="W4" s="14" t="inlineStr">
@@ -3296,7 +3333,7 @@
       <c r="M5" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="O5" s="2" t="s">
+      <c r="O5" s="4" t="s">
         <v>16</v>
       </c>
       <c r="P5" s="14" t="s">
@@ -3311,13 +3348,10 @@
       <c r="S5" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="T5" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="U5" s="14" t="s">
+      <c r="T5" s="33" t="s">
         <v>16</v>
       </c>
-      <c r="V5" s="22" t="s">
+      <c r="U5" s="22" t="s">
         <v>60</v>
       </c>
       <c r="W5" s="14" t="inlineStr">
@@ -3399,7 +3433,7 @@
       <c r="M6" s="24" t="s">
         <v>60</v>
       </c>
-      <c r="O6" s="2" t="s">
+      <c r="O6" s="4" t="s">
         <v>29</v>
       </c>
       <c r="P6" s="14" t="s">
@@ -3414,13 +3448,10 @@
       <c r="S6" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="T6" s="25" t="s">
-        <v>69</v>
-      </c>
-      <c r="U6" s="14" t="s">
+      <c r="T6" s="33" t="s">
         <v>16</v>
       </c>
-      <c r="V6" s="22" t="s">
+      <c r="U6" s="22" t="s">
         <v>60</v>
       </c>
     </row>
@@ -3462,7 +3493,7 @@
       <c r="M7" s="24" t="s">
         <v>60</v>
       </c>
-      <c r="O7" s="14"/>
+      <c r="O7" s="4"/>
       <c r="P7" s="14" t="s">
         <v>81</v>
       </c>
@@ -3473,13 +3504,10 @@
       <c r="S7" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="T7" s="26" t="s">
-        <v>83</v>
-      </c>
-      <c r="U7" s="14" t="s">
+      <c r="T7" s="35" t="s">
         <v>38</v>
       </c>
-      <c r="V7" s="17" t="s">
+      <c r="U7" s="17" t="s">
         <v>28</v>
       </c>
     </row>
@@ -3507,7 +3535,7 @@
       <c r="M8" s="27" t="s">
         <v>87</v>
       </c>
-      <c r="O8" s="14"/>
+      <c r="O8" s="4"/>
       <c r="P8" s="14" t="s">
         <v>88</v>
       </c>
@@ -3516,13 +3544,10 @@
       <c r="S8" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="T8" s="16" t="s">
-        <v>27</v>
-      </c>
-      <c r="U8" s="14" t="s">
+      <c r="T8" s="33" t="s">
         <v>16</v>
       </c>
-      <c r="V8" s="17" t="s">
+      <c r="U8" s="17" t="s">
         <v>28</v>
       </c>
     </row>
@@ -3548,7 +3573,7 @@
       <c r="M9" s="27" t="s">
         <v>87</v>
       </c>
-      <c r="O9" s="14"/>
+      <c r="O9" s="4"/>
       <c r="P9" s="14" t="s">
         <v>92</v>
       </c>
@@ -3557,13 +3582,10 @@
       <c r="S9" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="T9" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="U9" s="14" t="s">
+      <c r="T9" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="V9" s="17" t="s">
+      <c r="U9" s="17" t="s">
         <v>28</v>
       </c>
     </row>
@@ -3589,7 +3611,7 @@
       <c r="M10" s="27" t="s">
         <v>87</v>
       </c>
-      <c r="O10" s="14"/>
+      <c r="O10" s="4"/>
       <c r="P10" s="14" t="s">
         <v>96</v>
       </c>
@@ -3600,13 +3622,10 @@
       <c r="S10" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="T10" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="U10" s="14" t="s">
+      <c r="T10" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="V10" s="17" t="s">
+      <c r="U10" s="17" t="s">
         <v>28</v>
       </c>
     </row>
@@ -3632,7 +3651,7 @@
       <c r="M11" s="27" t="s">
         <v>87</v>
       </c>
-      <c r="O11" s="14"/>
+      <c r="O11" s="4"/>
       <c r="P11" s="14" t="s">
         <v>101</v>
       </c>
@@ -3643,13 +3662,10 @@
       <c r="S11" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="T11" s="26" t="s">
-        <v>83</v>
-      </c>
-      <c r="U11" s="14" t="s">
+      <c r="T11" s="35" t="s">
         <v>38</v>
       </c>
-      <c r="V11" s="17" t="s">
+      <c r="U11" s="17" t="s">
         <v>28</v>
       </c>
     </row>
@@ -3675,7 +3691,7 @@
       <c r="M12" s="27" t="s">
         <v>87</v>
       </c>
-      <c r="O12" s="14"/>
+      <c r="O12" s="4"/>
       <c r="P12" s="14" t="s">
         <v>106</v>
       </c>
@@ -3684,13 +3700,10 @@
       <c r="S12" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="T12" s="25" t="s">
-        <v>69</v>
-      </c>
-      <c r="U12" s="14" t="s">
+      <c r="T12" s="36" t="s">
         <v>49</v>
       </c>
-      <c r="V12" s="17" t="s">
+      <c r="U12" s="17" t="s">
         <v>28</v>
       </c>
     </row>
@@ -3716,7 +3729,7 @@
       <c r="M13" s="27" t="s">
         <v>87</v>
       </c>
-      <c r="O13" s="14"/>
+      <c r="O13" s="4"/>
       <c r="P13" s="14" t="s">
         <v>110</v>
       </c>
@@ -3725,13 +3738,10 @@
       <c r="S13" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="T13" s="26" t="s">
-        <v>83</v>
-      </c>
-      <c r="U13" s="14" t="s">
+      <c r="T13" s="35" t="s">
         <v>38</v>
       </c>
-      <c r="V13" s="17" t="s">
+      <c r="U13" s="17" t="s">
         <v>28</v>
       </c>
     </row>
@@ -3759,7 +3769,7 @@
       <c r="M14" s="27" t="s">
         <v>87</v>
       </c>
-      <c r="O14" s="14"/>
+      <c r="O14" s="4"/>
       <c r="P14" s="14" t="s">
         <v>114</v>
       </c>
@@ -3770,13 +3780,10 @@
       <c r="S14" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="T14" s="25" t="s">
-        <v>69</v>
-      </c>
-      <c r="U14" s="14" t="s">
+      <c r="T14" s="36" t="s">
         <v>49</v>
       </c>
-      <c r="V14" s="17" t="s">
+      <c r="U14" s="17" t="s">
         <v>28</v>
       </c>
     </row>
@@ -18273,7 +18280,7 @@
       <c r="M1015" s="29"/>
     </row>
   </sheetData>
-  <dataValidations count="8">
+  <dataValidations count="7">
     <dataValidation type="list" allowBlank="1" sqref="J2:J1015">
       <formula1>"Minor Repeatable,Minor Fire-Once,Major,Manual Scenario"</formula1>
     </dataValidation>
@@ -18287,12 +18294,9 @@
       <formula1>"Minor Repeatable,Minor Fire-Once,Major,Manual Scenario"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="T2:T14">
-      <formula1>"Low,Medium,High,Severe"</formula1>
+      <formula1>"1,2,3,4,5"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="U2:U14">
-      <formula1>"1,2,3,4,5"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="V2:V14">
       <formula1>"Implemented,New,In progress,Under review,Buggy"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="AD2:AD5">

</xml_diff>

<commit_message>
Fix catalog conditional fill rendering
</commit_message>
<xml_diff>
--- a/docs/spreadsheets/chaos_redux_events_catalog.xlsx
+++ b/docs/spreadsheets/chaos_redux_events_catalog.xlsx
@@ -3434,7 +3434,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFFFE699"/>
-          <bgColor indexed="64"/>
+          <bgColor rgb="FFFFE699"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3442,7 +3442,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFC6EFCE"/>
-          <bgColor indexed="64"/>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3450,7 +3450,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFF4CCCC"/>
-          <bgColor indexed="64"/>
+          <bgColor rgb="FFF4CCCC"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3458,7 +3458,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFDDEBF7"/>
-          <bgColor indexed="64"/>
+          <bgColor rgb="FFDDEBF7"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3466,7 +3466,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFE7E6E6"/>
-          <bgColor indexed="64"/>
+          <bgColor rgb="FFE7E6E6"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3474,7 +3474,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFCFE2F3"/>
-          <bgColor indexed="64"/>
+          <bgColor rgb="FFCFE2F3"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3482,7 +3482,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFFCE4D6"/>
-          <bgColor indexed="64"/>
+          <bgColor rgb="FFFCE4D6"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3490,7 +3490,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFF8CBAD"/>
-          <bgColor indexed="64"/>
+          <bgColor rgb="FFF8CBAD"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3498,7 +3498,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFC6EFCE"/>
-          <bgColor indexed="64"/>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3506,7 +3506,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFF4CCCC"/>
-          <bgColor indexed="64"/>
+          <bgColor rgb="FFF4CCCC"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3514,7 +3514,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFD9D2E9"/>
-          <bgColor indexed="64"/>
+          <bgColor rgb="FFD9D2E9"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3522,7 +3522,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFC6EFCE"/>
-          <bgColor indexed="64"/>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3530,7 +3530,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFFFE699"/>
-          <bgColor indexed="64"/>
+          <bgColor rgb="FFFFE699"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3538,7 +3538,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFF4CCCC"/>
-          <bgColor indexed="64"/>
+          <bgColor rgb="FFF4CCCC"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3546,7 +3546,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFD9D2E9"/>
-          <bgColor indexed="64"/>
+          <bgColor rgb="FFD9D2E9"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3554,7 +3554,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFFFE5E5"/>
-          <bgColor indexed="64"/>
+          <bgColor rgb="FFFFE5E5"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3562,7 +3562,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFFFCCCC"/>
-          <bgColor indexed="64"/>
+          <bgColor rgb="FFFFCCCC"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3570,7 +3570,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFFFB3B3"/>
-          <bgColor indexed="64"/>
+          <bgColor rgb="FFFFB3B3"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3578,7 +3578,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFFF9999"/>
-          <bgColor indexed="64"/>
+          <bgColor rgb="FFFF9999"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3586,7 +3586,7 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFFF8080"/>
-          <bgColor indexed="64"/>
+          <bgColor rgb="FFFF8080"/>
         </patternFill>
       </fill>
     </dxf>

</xml_diff>

<commit_message>
Disperse Fury triggerable scenario actors
</commit_message>
<xml_diff>
--- a/docs/spreadsheets/chaos_redux_events_catalog.xlsx
+++ b/docs/spreadsheets/chaos_redux_events_catalog.xlsx
@@ -2554,7 +2554,7 @@
       </c>
       <c r="Y6" s="61" t="inlineStr">
         <is>
-          <t>Creates AI Fury actors from safe eligible minors, loads their Fury package, and starts the expansion loop without turning the player into Fury.</t>
+          <t>Creates dispersed AI Fury actors from safe eligible minors, loads their Fury package, and starts the expansion loop without turning the player into Fury.</t>
         </is>
       </c>
       <c r="Z6" s="47" t="inlineStr">
@@ -2564,7 +2564,7 @@
       </c>
       <c r="AA6" s="47" t="inlineStr">
         <is>
-          <t>Low/Medium/High/Maximum targets 1/3/6/10 Fury actors, capped by safe eligible countries. Maximum records the ten-fires challenge state when ten actors spawn.</t>
+          <t>Low/Medium/High/Maximum targets 2/5/9/16 dispersed Fury actors, capped by safe eligible countries. Maximum records the full-spread challenge state when the maximum actor count or every safe candidate is used.</t>
         </is>
       </c>
       <c r="AB6" s="50" t="inlineStr">

</xml_diff>

<commit_message>
Update Holy Realm event catalog row
</commit_message>
<xml_diff>
--- a/docs/spreadsheets/chaos_redux_events_catalog.xlsx
+++ b/docs/spreadsheets/chaos_redux_events_catalog.xlsx
@@ -3238,7 +3238,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr filterMode="false">
     <tabColor rgb="FF1C4587"/>
     <pageSetUpPr fitToPage="false"/>
@@ -3500,26 +3500,40 @@
       <c r="B4" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="C4" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="D4" s="10" t="s">
-        <v>56</v>
-      </c>
-      <c r="E4" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="F4" s="12" t="s">
-        <v>58</v>
-      </c>
-      <c r="G4" s="13" t="s">
-        <v>59</v>
-      </c>
-      <c r="H4" s="14" t="s">
-        <v>60</v>
-      </c>
-      <c r="I4" s="15" t="s">
-        <v>61</v>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>Transforms Tibet first, falling back to Bhutan or Nepal only if Tibet is gone and the fallback exists and is not a special chaos country. All origins use the shared Holy Realm/THR identity. The 112-focus tree builds a defensive refuge into Buddhahood play through Bodhi, Dhyana, Teaching Successes, Meditation Charge, Defilements, World Suffering, Sangha Cohesion, the Sangha Compact, anti-chaos Buddha powers, hidden False Buddha Schism outcomes, and the split Final Silence route. Twelve Holy Realm achievements and DDS icon triplets are registered.</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="inlineStr">
+        <is>
+          <t>Mountain Refuge: forms The Holy Realm, initializes Mandala and Buddhahood counters, applies fragile refuge ideas, opens the Mandala GUI/category, loads the focus tree, and starts shelter, road, refugee, early teaching, and defensive play.</t>
+        </is>
+      </c>
+      <c r="E4" s="11" t="inlineStr">
+        <is>
+          <t>Bodhisattva Teaching and Meditation: Send Dhamma Envoys, Guard the Pilgrimage Route, Translate the Wheel, teaching-under-fire, and the concentration-vow sequence raise Bodhi, Compassion, Dhyana Depth, and Meditation Charge while tracking clean-route and Defilement risks.</t>
+        </is>
+      </c>
+      <c r="F4" s="12" t="inlineStr">
+        <is>
+          <t>Governance, Sanctuary, Guardian, and Sangha Compact routes: Council/Regent/Assembly choices, infrastructure and supply works, Temple Guard and pilgrimage escort systems, compact admission, aid, anti-puppet clauses, and AI weights support defensive humanitarian play against special chaos countries.</t>
+        </is>
+      </c>
+      <c r="G4" s="13" t="inlineStr">
+        <is>
+          <t>The Unshaken Seat and Powers: Buddhahood requires 108 Bodhi, Fourth Dhyana, low Defilements, teaching successes, crisis teaching, and the focus marker. Success changes leader/stage, fires The Awakened One, unlocks the Buddha powers category, and the first anti-chaos power display fires Powers of the Awakened.</t>
+        </is>
+      </c>
+      <c r="H4" s="14" t="inlineStr">
+        <is>
+          <t>Final Silence and Schism: the hidden False Buddha branch supports debate, exile, suppression, and absorption outcomes. Extinction of Defilements, Witnesses Gather, and the final doctrine balance gate non-terminal Empty Seat aftermath versus terminal Final Silence.</t>
+        </is>
+      </c>
+      <c r="I4" s="15" t="inlineStr">
+        <is>
+          <t>Terminal Final Silence requires Buddhahood, Dhyana 4, low Defilements, Meditation Charge, a prior anti-chaos power display, final doctrine/focus gates, controlled capital, no active schism, no other world-end, and chaos above 1000. Completion sets world_end/world_end_final_silence and runs the strike-wave sequence; otherwise the non-terminal Empty Seat aftermath remains playable.</t>
+        </is>
       </c>
       <c r="J4" s="16" t="s">
         <v>27</v>
@@ -20746,9 +20760,9 @@
     <oddFooter/>
   </headerFooter>
   <tableParts>
-    <tablePart r:id="rId1"/>
-    <tablePart r:id="rId2"/>
-    <tablePart r:id="rId3"/>
+    <tablePart ns1:id="rId1"/>
+    <tablePart ns1:id="rId2"/>
+    <tablePart ns1:id="rId3"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Align Holy Realm event catalog row
</commit_message>
<xml_diff>
--- a/docs/spreadsheets/chaos_redux_events_catalog.xlsx
+++ b/docs/spreadsheets/chaos_redux_events_catalog.xlsx
@@ -191,7 +191,7 @@
     <t xml:space="preserve">The Holy Realm</t>
   </si>
   <si>
-    <t xml:space="preserve">Transforms Tibet or a Tibet-centered Himalayan state into the Holy Realm. The route begins as a defensive mountain refuge, develops into a Bodhisattva-led state, and layers Bodhi, Dhyana, Teaching Successes, Meditation Charge, Defilements, World Suffering, and Sangha Cohesion onto the older Mandala counters. The Unshaken Seat tests whether the Bodhisattva realizes Buddhahood or builds False Buddha Schism pressure; a realized Buddha unlocks Powers of the Awakened and a split Final Silence that can end as the Empty Seat aftermath or the terminal world-end.</t>
+    <t xml:space="preserve">Transforms Tibet first, falling back to Bhutan or Nepal only if Tibet is gone and the fallback exists as a valid normal country. All origins use the shared Holy Realm/THR identity. The route begins as a defensive mountain refuge, develops into a Bodhisattva-led state, and layers Bodhi, Dhyana, Teaching Successes, Meditation Charge, Defilements, World Suffering, and Sangha Cohesion onto the older Mandala counters. The Unshaken Seat tests whether the Bodhisattva realizes Buddhahood or builds False Buddha Schism pressure; a realized Buddha unlocks Powers of the Awakened and a split Final Silence that can end as the Empty Seat aftermath or the terminal world-end.</t>
   </si>
   <si>
     <t xml:space="preserve">Mountain Refuge: forms the Holy Realm, loads the Holy Realm focus tree, initializes the Mandala and Buddhahood counters, and opens defensive refuge, high-pass, shelter, and refugee policy content.</t>
@@ -3502,7 +3502,7 @@
       </c>
       <c r="C4" s="9" t="inlineStr">
         <is>
-          <t>Transforms Tibet first, falling back to Bhutan or Nepal only if Tibet is gone and the fallback exists and is not a special chaos country. All origins use the shared Holy Realm/THR identity. The 112-focus tree builds a defensive refuge into Buddhahood play through Bodhi, Dhyana, Teaching Successes, Meditation Charge, Defilements, World Suffering, Sangha Cohesion, the Sangha Compact, anti-chaos Buddha powers, hidden False Buddha Schism outcomes, and the split Final Silence route. Twelve Holy Realm achievements and DDS icon triplets are registered.</t>
+          <t>Transforms Tibet first, falling back to Bhutan or Nepal only if Tibet is gone and the fallback exists and is not a special chaos country. All origins use the shared Holy Realm/THR identity. The 111-focus tree builds a defensive refuge into Buddhahood play through Bodhi, Dhyana, Teaching Successes, Meditation Charge, Defilements, World Suffering, Sangha Cohesion, the Sangha Compact, anti-chaos Buddha powers, hidden False Buddha Schism outcomes, and the split Final Silence route. Twelve Holy Realm achievements and DDS icon triplets are registered.</t>
         </is>
       </c>
       <c r="D4" s="10" t="inlineStr">

</xml_diff>

<commit_message>
Finalize Tensions Rising fix pass
</commit_message>
<xml_diff>
--- a/docs/spreadsheets/chaos_redux_events_catalog.xlsx
+++ b/docs/spreadsheets/chaos_redux_events_catalog.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Main Sheet" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Info" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Legend" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Main Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Info" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1" iterateDelta="0.0001"/>
@@ -2031,33 +2031,34 @@
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>Tensions Rising is a repeatable diplomatic pressure event. In a calm world it adds +10 world tension and is blocked at full world tension. Higher chaos tiers let it fire even at 100% world tension, adding direct chaos, larger world-tension packets, capped temporary timer pressure, timed relation shocks, delayed reports, event-log and evolution-detail wiring, AI posture hooks, achievement tracking, and cataloged asset hooks, with Stage IV ending in a one-time non-terminal super-event.</t>
+          <t>Tensions Rising is a repeatable diplomatic-pressure incident. In calm conditions it adds world tension and stops once world tension is full. At higher chaos levels it can still fire at maximum world tension, adding indirect pressure through timer pacing, timed opinion penalties, AI readiness ideas, delayed reports, and achievement tracking.
+It does not create war goals, countries, cores, focus trees, formables, or a world-end scenario.</t>
         </is>
       </c>
       <c r="D9" s="10" t="inlineStr">
         <is>
-          <t>Gathering Storm: Cable Traffic Flood. Adds +10 chaos and +10 world tension, can fire at full world tension, opens light timed relation shocks, a capped timer pulse, delayed diplomatic reports, and the first wired evolution and event-log detail updates.</t>
+          <t>Cable Traffic Increase. The first evolved stage moves the incident beyond a simple world-tension increase. Relation shocks begin, and later incidents can briefly gather pace.</t>
         </is>
       </c>
       <c r="E9" s="11" t="inlineStr">
         <is>
-          <t>Rising Chaos: The Accusation Market. Adds +15 chaos and +20 world tension, selects more relation pairs and AI posture targets, and expands the delayed-report and evolution-detail pressure.</t>
+          <t>Competing Accusations. The second stage reaches more capitals. Timed relation damage can affect additional pairs, delayed reports become more likely, and some governments take short-lived readiness postures.</t>
         </is>
       </c>
       <c r="F9" s="12" t="inlineStr">
         <is>
-          <t>Chaos Tier: General Staffs Stop Sleeping. Adds +25 chaos and +50 world tension, applies heavier relation shocks, stronger timer pressure, broader AI posture hooks, and opens the Thin Wire full-tension peace watch.</t>
+          <t>Staff Readiness. The third stage treats the pattern as a planning concern. Relation shocks last longer, diplomatic aftershocks remain temporary, and peaceful players can begin the Thin Wire watch while world tension remains full.</t>
         </is>
       </c>
       <c r="G9" s="13" t="inlineStr">
         <is>
-          <t>Totalen Chaos: The Permanent Alert. Adds +50 chaos and +100 world tension, applies the strongest timed diplomatic shock, and fires the one-time non-terminal super-event The Red Line Disappears.</t>
+          <t>Extended Alert. The fourth stage is the strongest non-terminal form of the incident. It keeps pressure indirect and does not create a direct conflict branch.</t>
         </is>
       </c>
       <c r="H9" s="14" t="n"/>
       <c r="I9" s="15" t="inlineStr">
         <is>
-          <t>No world-end scenario. Stage IV is a one-time non-terminal super-event only; Event 8 never creates direct war goals, countries, focus trees, cores, or formables.</t>
+          <t>No world-end scenario. Event 8 never creates direct war goals, countries, focus trees, cores, or formables; Stage IV remains a normal event-log and evolution stage.</t>
         </is>
       </c>
       <c r="J9" s="28" t="inlineStr">
@@ -2468,7 +2469,7 @@
       </c>
       <c r="Q15" s="20" t="inlineStr">
         <is>
-          <t>Repeatable diplomatic-panic cluster. Current implemented member is Event 8, which pushes world tension and chaos through capped timer pressure, timed relation shocks, delayed reports, event-log and evolution-detail wiring, AI posture hooks, achievement tracking, and cataloged asset hooks without direct war goals, new countries, focus trees, cores, formables, or a world-end scenario.</t>
+          <t>Diplomatic panic pushes world tension, relation damage, ministries, newspapers, and staff offices into a shared crisis pattern without creating direct war goals or new countries.</t>
         </is>
       </c>
       <c r="R15" s="20" t="inlineStr">
@@ -2483,7 +2484,7 @@
       </c>
       <c r="T15" s="27" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>Calm World</t>
         </is>
       </c>
       <c r="U15" s="31" t="inlineStr">

</xml_diff>